<commit_message>
Remove AI fluff, keep concise factual points, update budget table for 2 persons, bump SW v39
</commit_message>
<xml_diff>
--- a/yunnan_travel_plan_2026.xlsx
+++ b/yunnan_travel_plan_2026.xlsx
@@ -402,20 +402,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L64"/>
-  <cols>
-    <col min="1" max="1" width="24.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="60.83203125" customWidth="1"/>
-    <col min="5" max="5" width="38.83203125" customWidth="1"/>
-    <col min="6" max="6" width="18.83203125" customWidth="1"/>
-    <col min="7" max="7" width="35.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="16.83203125" customWidth="1"/>
-    <col min="11" max="11" width="16.83203125" customWidth="1"/>
-    <col min="12" max="12" width="38.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -656,7 +642,7 @@
         <v>02:00 – 10:00</v>
       </c>
       <c r="D7" t="str">
-        <v>เช็กอินเข้าห้องพัก อาบน้ำอุ่น พักผ่อนเอาแรงให้เต็มอิ่ม</v>
+        <v>เช็กอินเข้าห้องพัก พักผ่อน 1 คืน</v>
       </c>
       <c r="E7" t="str">
         <v>腾航大酒店</v>
@@ -1516,7 +1502,7 @@
         <v>-</v>
       </c>
       <c r="L29" t="str">
-        <v>ไฮไลท์ทางชันปราบเซียน</v>
+        <v>ทางชัน 28 โค้ง</v>
       </c>
     </row>
     <row r="30">
@@ -2859,14 +2845,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F6"/>
-  <cols>
-    <col min="1" max="1" width="38.83203125" customWidth="1"/>
-    <col min="2" max="2" width="22.83203125" customWidth="1"/>
-    <col min="3" max="3" width="22.83203125" customWidth="1"/>
-    <col min="4" max="4" width="24.83203125" customWidth="1"/>
-    <col min="5" max="5" width="22.83203125" customWidth="1"/>
-    <col min="6" max="6" width="24.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2998,19 +2976,6 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K71"/>
-  <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="45.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="35.83203125" customWidth="1"/>
-    <col min="5" max="5" width="45.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="20.83203125" customWidth="1"/>
-    <col min="8" max="8" width="26.83203125" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="40.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5507,19 +5472,6 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K30"/>
-  <cols>
-    <col min="1" max="1" width="8.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="45.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="60.83203125" customWidth="1"/>
-    <col min="6" max="6" width="35.83203125" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" customWidth="1"/>
-    <col min="8" max="8" width="20.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="22.83203125" customWidth="1"/>
-    <col min="11" max="11" width="35.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6581,15 +6533,6 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G10"/>
-  <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="22.83203125" customWidth="1"/>
-    <col min="5" max="5" width="18.83203125" customWidth="1"/>
-    <col min="6" max="6" width="20.83203125" customWidth="1"/>
-    <col min="7" max="7" width="35.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>

<commit_message>
Add complete master trip budget covering all 6 categories (flights, hotels, transport, attractions, prep, food) for 2 persons, bump SW v40
</commit_message>
<xml_diff>
--- a/yunnan_travel_plan_2026.xlsx
+++ b/yunnan_travel_plan_2026.xlsx
@@ -2844,131 +2844,595 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:G28"/>
+  <cols>
+    <col min="1" max="1" width="32.83203125" customWidth="1"/>
+    <col min="2" max="2" width="45.83203125" customWidth="1"/>
+    <col min="3" max="3" width="25.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" customWidth="1"/>
+    <col min="6" max="6" width="20.83203125" customWidth="1"/>
+    <col min="7" max="7" width="20.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>ประเภท (Category)</v>
+        <v>หมวดหมู่งบประมาณ (Category)</v>
       </c>
       <c r="B1" t="str">
-        <v>จำนวนครั้ง (Count)</v>
+        <v>รายละเอียด (Description)</v>
       </c>
       <c r="C1" t="str">
-        <v>ราคาต่อคน (หยวน / ¥)</v>
+        <v>การชำระเงิน (Status)</v>
       </c>
       <c r="D1" t="str">
-        <v>ราคาต่อคน (บาท @ 5.0)</v>
+        <v>รวม 2 คน (หยวน / ¥)</v>
       </c>
       <c r="E1" t="str">
-        <v>รวม 2 คน (หยวน / ¥)</v>
+        <v>รวม 2 คน (บาท / ฿)</v>
       </c>
       <c r="F1" t="str">
-        <v>รวม 2 คน (บาท @ 5.0)</v>
+        <v>เฉลี่ยต่อคน (หยวน / ¥)</v>
+      </c>
+      <c r="G1" t="str">
+        <v>เฉลี่ยต่อคน (บาท / ฿)</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>รถแท็กซี่ / DiDi</v>
+        <v>✈️ ตั๋วเครื่องบินไป-กลับ</v>
       </c>
       <c r="B2" t="str">
-        <v>6 ครั้ง</v>
-      </c>
-      <c r="C2">
-        <v>93.5</v>
+        <v>China Eastern 4 เที่ยวบิน (BKK⇄KMG⇄LJG)</v>
+      </c>
+      <c r="C2" t="str">
+        <v>ชำระแล้ว (ออกตั๋วแล้ว)</v>
       </c>
       <c r="D2">
-        <v>467.5</v>
+        <v>3250.45</v>
       </c>
       <c r="E2">
-        <v>187</v>
+        <v>16252.23</v>
       </c>
       <c r="F2">
-        <v>935</v>
+        <v>1625.22</v>
+      </c>
+      <c r="G2">
+        <v>8126.12</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>รถไฟใต้ดิน (Metro)</v>
+        <v>🏨 โรงแรมและที่พัก (7 คืน)</v>
       </c>
       <c r="B3" t="str">
-        <v>5 ครั้ง</v>
-      </c>
-      <c r="C3">
-        <v>30</v>
+        <v>คุนหมิง 1 คืน + ลี่เจียง 3 คืน + เสือกระโจน 1 คืน + แชงกรี-ลา 2 คืน</v>
+      </c>
+      <c r="C3" t="str">
+        <v>ยืนยันการจองแล้ว (Trip.com)</v>
       </c>
       <c r="D3">
-        <v>150</v>
+        <v>733.33</v>
       </c>
       <c r="E3">
-        <v>60</v>
+        <v>3666.67</v>
       </c>
       <c r="F3">
-        <v>300</v>
+        <v>366.67</v>
+      </c>
+      <c r="G3">
+        <v>1833.34</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>รถบัส / รถเมล์ / ตู้ทุ่นแรง</v>
+        <v>🚌 การเดินทางในประเทศจีน</v>
       </c>
       <c r="B4" t="str">
-        <v>7 ครั้ง</v>
-      </c>
-      <c r="C4">
-        <v>236</v>
+        <v>DiDi 6 ครั้ง, Metro 5 ครั้ง, รถบัส, รถไฟความเร็วสูง, รถตู้, ฝากกระเป๋า</v>
+      </c>
+      <c r="C4" t="str">
+        <v>จ่ายหน้างาน (Alipay/เงินสด)</v>
       </c>
       <c r="D4">
-        <v>1180</v>
+        <v>598</v>
       </c>
       <c r="E4">
-        <v>472</v>
+        <v>2990</v>
       </c>
       <c r="F4">
-        <v>2360</v>
+        <v>299</v>
+      </c>
+      <c r="G4">
+        <v>1495</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>ค่าธรรมเนียมบำรุงเมืองเก่า / คฤหาสน์มู่</v>
+        <v>🎟️ ค่าเข้าชมและกิจกรรม</v>
       </c>
       <c r="B5" t="str">
-        <v>1 ครั้ง (ลี่เจียง 7 จุด)</v>
-      </c>
-      <c r="C5">
-        <v>50</v>
+        <v>เสือกระโจน, คฤหาสน์มู่, อุทยานผู่ต๋าชั่ว, วัดซงจ้านหลิน</v>
+      </c>
+      <c r="C5" t="str">
+        <v>จ่ายหน้างาน (Alipay/เคาน์เตอร์)</v>
       </c>
       <c r="D5">
-        <v>250</v>
+        <v>726</v>
       </c>
       <c r="E5">
-        <v>100</v>
+        <v>3630</v>
       </c>
       <c r="F5">
-        <v>500</v>
+        <v>363</v>
+      </c>
+      <c r="G5">
+        <v>1815</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>ยอดรวมทั้งสิ้น (28 รายการเดินทาง)</v>
+        <v>🛡️ เตรียมตัวก่อนเดินทาง</v>
       </c>
       <c r="B6" t="str">
-        <v>28 รายการ</v>
-      </c>
-      <c r="C6">
-        <v>391.5</v>
+        <v>ประกันภัย Insurverse + SIM โรมมิ่งอินเทอร์เน็ต (2 ท่าน)</v>
+      </c>
+      <c r="C6" t="str">
+        <v>ชำระก่อนเดินทาง</v>
       </c>
       <c r="D6">
-        <v>1957.5</v>
+        <v>362.8</v>
       </c>
       <c r="E6">
-        <v>783</v>
+        <v>1814</v>
       </c>
       <c r="F6">
-        <v>3915</v>
+        <v>181.4</v>
+      </c>
+      <c r="G6">
+        <v>907</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>🍜 ค่าอาหารและเครื่องดื่ม</v>
+      </c>
+      <c r="B7" t="str">
+        <v>อาหารมื้อหลักตลอด 8 วัน + สตรีทฟู้ด + คาเฟ่ (ประมาณการ)</v>
+      </c>
+      <c r="C7" t="str">
+        <v>จ่ายหน้างาน (Alipay/WeChat)</v>
+      </c>
+      <c r="D7">
+        <v>1070</v>
+      </c>
+      <c r="E7">
+        <v>5350</v>
+      </c>
+      <c r="F7">
+        <v>535</v>
+      </c>
+      <c r="G7">
+        <v>2675</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>⭐ ยอดรวมงบประมาณทั้งทริป (Grand Total)</v>
+      </c>
+      <c r="B8" t="str">
+        <v>รวมค่าใช้จ่ายทั้งสิ้นตลอดทริป 8 วัน 7 คืน (2 ท่าน)</v>
+      </c>
+      <c r="C8" t="str">
+        <v>ครบทุกหมวดหมู่</v>
+      </c>
+      <c r="D8">
+        <v>6740.58</v>
+      </c>
+      <c r="E8">
+        <v>33702.9</v>
+      </c>
+      <c r="F8">
+        <v>3370.29</v>
+      </c>
+      <c r="G8">
+        <v>16851.45</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>📌 สรุปยอดการชำระเงิน</v>
+      </c>
+      <c r="B10" t="str">
+        <v/>
+      </c>
+      <c r="C10" t="str">
+        <v/>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>1. ชำระล่วงหน้าเรียบร้อยแล้ว (Pre-paid)</v>
+      </c>
+      <c r="B11" t="str">
+        <v>ตั๋วเครื่องบิน + โรงแรม 7 คืน + ประกัน/ซิม</v>
+      </c>
+      <c r="C11" t="str">
+        <v>ชำระแล้ว</v>
+      </c>
+      <c r="D11">
+        <v>4346.58</v>
+      </c>
+      <c r="E11">
+        <v>21732.9</v>
+      </c>
+      <c r="F11">
+        <v>2173.29</v>
+      </c>
+      <c r="G11">
+        <v>10866.45</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>2. เตรียมจ่ายระหว่างเดินทาง (On-trip Alipay)</v>
+      </c>
+      <c r="B12" t="str">
+        <v>การเดินทาง + บัตรเข้าชม + อาหารตลอดทริป</v>
+      </c>
+      <c r="C12" t="str">
+        <v>สแกน Alipay/WeChat</v>
+      </c>
+      <c r="D12">
+        <v>2394</v>
+      </c>
+      <c r="E12">
+        <v>11970</v>
+      </c>
+      <c r="F12">
+        <v>1197</v>
+      </c>
+      <c r="G12">
+        <v>5985</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>🏨 รายละเอียดค่าที่พัก 7 คืน (อ้างอิง Trip.com ยืนยันแล้ว)</v>
+      </c>
+      <c r="B14" t="str">
+        <v/>
+      </c>
+      <c r="C14" t="str">
+        <v/>
+      </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
+      <c r="E14" t="str">
+        <v/>
+      </c>
+      <c r="F14" t="str">
+        <v/>
+      </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>คืนที่ 1 (24 ต.ค.)</v>
+      </c>
+      <c r="B15" t="str">
+        <v>โรงแรมเติงหาง คุนหมิงฉางซุย (腾航大酒店)</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Trip Ref: 1359047990059246</v>
+      </c>
+      <c r="D15">
+        <v>99.71</v>
+      </c>
+      <c r="E15">
+        <v>498.53</v>
+      </c>
+      <c r="F15">
+        <v>49.85</v>
+      </c>
+      <c r="G15">
+        <v>249.27</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>คืนที่ 2 (25 ต.ค.)</v>
+      </c>
+      <c r="B16" t="str">
+        <v>โฮมสเตย์หลงลั่วเหอ สนามบินลี่เจียง (丽江龙落河民宿)</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Trip Ref: 1359048036644931</v>
+      </c>
+      <c r="D16">
+        <v>77.26</v>
+      </c>
+      <c r="E16">
+        <v>386.32</v>
+      </c>
+      <c r="F16">
+        <v>38.63</v>
+      </c>
+      <c r="G16">
+        <v>193.16</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>คืนที่ 3 (26 ต.ค.)</v>
+      </c>
+      <c r="B17" t="str">
+        <v>ชีเยวี่ยหลินอิ๋น เมืองเก่าลี่เจียง (栖悦林隐别院)</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Trip Ref: 1359047990153900</v>
+      </c>
+      <c r="D17">
+        <v>76.26</v>
+      </c>
+      <c r="E17">
+        <v>381.29</v>
+      </c>
+      <c r="F17">
+        <v>38.13</v>
+      </c>
+      <c r="G17">
+        <v>190.65</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>คืนที่ 4 (27 ต.ค.)</v>
+      </c>
+      <c r="B18" t="str">
+        <v>ซานเหม่ยเกสต์เฮาส์ เสือกระโจน (Summit Inn)</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Trip Ref: 1359047990248699</v>
+      </c>
+      <c r="D18">
+        <v>210.56</v>
+      </c>
+      <c r="E18">
+        <v>1052.78</v>
+      </c>
+      <c r="F18">
+        <v>105.28</v>
+      </c>
+      <c r="G18">
+        <v>526.39</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>คืนที่ 5-6 (28-29 ต.ค.)</v>
+      </c>
+      <c r="B19" t="str">
+        <v>หวังซานเสี่ยวย่วน เมืองโบราณตู๋เค่อจง (2 คืน)</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Trip Ref: 1359048589640445</v>
+      </c>
+      <c r="D19">
+        <v>192.76</v>
+      </c>
+      <c r="E19">
+        <v>963.8</v>
+      </c>
+      <c r="F19">
+        <v>96.38</v>
+      </c>
+      <c r="G19">
+        <v>481.9</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>คืนที่ 7 (30 ต.ค.)</v>
+      </c>
+      <c r="B20" t="str">
+        <v>ชีเยวี่ยหลินอิ๋น เมืองเก่าลี่เจียง (栖悦林隐别院)</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Trip Ref: 1359048443168258</v>
+      </c>
+      <c r="D20">
+        <v>76.79</v>
+      </c>
+      <c r="E20">
+        <v>383.95</v>
+      </c>
+      <c r="F20">
+        <v>38.39</v>
+      </c>
+      <c r="G20">
+        <v>191.98</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>รวมค่าที่พัก 7 คืน</v>
+      </c>
+      <c r="B21" t="str">
+        <v>รวม 7 คืน (2 ท่าน)</v>
+      </c>
+      <c r="C21" t="str">
+        <v>ยืนยันแล้วทุกคืน</v>
+      </c>
+      <c r="D21">
+        <v>733.33</v>
+      </c>
+      <c r="E21">
+        <v>3666.67</v>
+      </c>
+      <c r="F21">
+        <v>366.67</v>
+      </c>
+      <c r="G21">
+        <v>1833.34</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>🎟️ รายละเอียดค่าเข้าชมสถานที่ (2 ท่าน)</v>
+      </c>
+      <c r="B23" t="str">
+        <v/>
+      </c>
+      <c r="C23" t="str">
+        <v/>
+      </c>
+      <c r="D23" t="str">
+        <v/>
+      </c>
+      <c r="E23" t="str">
+        <v/>
+      </c>
+      <c r="F23" t="str">
+        <v/>
+      </c>
+      <c r="G23" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>อุทยานเสือกระโจน (Tiger Leaping Gorge)</v>
+      </c>
+      <c r="B24" t="str">
+        <v>บัตรเข้าชมอุทยาน (คนละ ¥45)</v>
+      </c>
+      <c r="C24" t="str">
+        <v>ซื้อหน้าด่าน</v>
+      </c>
+      <c r="D24">
+        <v>90</v>
+      </c>
+      <c r="E24">
+        <v>450</v>
+      </c>
+      <c r="F24">
+        <v>45</v>
+      </c>
+      <c r="G24">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>คฤหาสน์มู่และเมืองเก่าลี่เจียง (Mu Mansion)</v>
+      </c>
+      <c r="B25" t="str">
+        <v>ค่าธรรมเนียมเข้าชม (คนละ ¥50)</v>
+      </c>
+      <c r="C25" t="str">
+        <v>ซื้อหน้าทางเข้า</v>
+      </c>
+      <c r="D25">
+        <v>100</v>
+      </c>
+      <c r="E25">
+        <v>500</v>
+      </c>
+      <c r="F25">
+        <v>50</v>
+      </c>
+      <c r="G25">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>อุทยานแห่งชาติผู่ต๋าชั่ว (Potatso National Park)</v>
+      </c>
+      <c r="B26" t="str">
+        <v>แพ็กเกจบัตรรวม + ชัตเติลบัส + รถรับส่ง (คนละ ¥178)</v>
+      </c>
+      <c r="C26" t="str">
+        <v>จองล่วงหน้า/หน้างาน</v>
+      </c>
+      <c r="D26">
+        <v>356</v>
+      </c>
+      <c r="E26">
+        <v>1780</v>
+      </c>
+      <c r="F26">
+        <v>178</v>
+      </c>
+      <c r="G26">
+        <v>890</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>วัดกาด่านซงจ้านหลิน (Songzanlin Monastery)</v>
+      </c>
+      <c r="B27" t="str">
+        <v>ค่าเข้าชมวัด + บัสในวัด (คนละ ¥90)</v>
+      </c>
+      <c r="C27" t="str">
+        <v>ซื้อศูนย์บริการ</v>
+      </c>
+      <c r="D27">
+        <v>180</v>
+      </c>
+      <c r="E27">
+        <v>900</v>
+      </c>
+      <c r="F27">
+        <v>90</v>
+      </c>
+      <c r="G27">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>รวมค่าเข้าชมสถานที่</v>
+      </c>
+      <c r="B28" t="str">
+        <v>รวม 4 แหล่งท่องเที่ยว (2 ท่าน)</v>
+      </c>
+      <c r="C28" t="str">
+        <v>จ่ายหน้างาน</v>
+      </c>
+      <c r="D28">
+        <v>726</v>
+      </c>
+      <c r="E28">
+        <v>3630</v>
+      </c>
+      <c r="F28">
+        <v>363</v>
+      </c>
+      <c r="G28">
+        <v>1815</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G28"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Remove Mu Mansion ticket fee (saved ฿500 / ¥100 for 2 persons), update budget to ฿33,202.90, bump v43
</commit_message>
<xml_diff>
--- a/yunnan_travel_plan_2026.xlsx
+++ b/yunnan_travel_plan_2026.xlsx
@@ -528,7 +528,7 @@
         <v>20:50 – 00:30</v>
       </c>
       <c r="D4" t="str">
-        <v>✈️ เที่ยวบิน MU-9614: สุวรรณภูมิ (BKK) ➔ ท่าอากาศยานนานาชาติคุนหมิงฉางสุ่ย (KMG) (บินตรง 3 ชม. 40 นาที)</v>
+        <v>เที่ยวบิน MU-9614: สุวรรณภูมิ (BKK)  ท่าอากาศยานนานาชาติคุนหมิงฉางสุ่ย (KMG) (บินตรง 3 ชม. 40 นาที)</v>
       </c>
       <c r="E4" t="str">
         <v>昆明长水国际机场</v>
@@ -721,7 +721,7 @@
         <v>นั่งรถไฟใต้ดิน Metro สาย 6 เข้าเมือง ไปกิน "ก๋วยเตี๋ยวข้ามสะพาน" ร้านระดับตำนาน เจี้ยนซินหยวน</v>
       </c>
       <c r="E9" t="str">
-        <v>腾航大酒店 [250001] ➔ 建新园·宝善街店 [250002]</v>
+        <v>腾航大酒店 [250001]  建新园·宝善街店 [250002]</v>
       </c>
       <c r="F9" t="str">
         <v>รถไฟ</v>
@@ -759,7 +759,7 @@
         <v>เดินเที่ยวถ่ายรูปซุ้มประตูกิมหม่าปี้จีฟาง (ม้าทองไก่หยก) ถนนโบราณคุนหมิงเหล่าเจีย และถนนคนเดินหนานผิง</v>
       </c>
       <c r="E10" t="str">
-        <v>建新园 [250101] ➔ 金马碧鸡坊 [250102] ➔ 南屏步行街 [250103]</v>
+        <v>建新园 [250101]  金马碧鸡坊 [250102]  南屏步行街 [250103]</v>
       </c>
       <c r="F10" t="str">
         <v>เดิน</v>
@@ -797,7 +797,7 @@
         <v>นั่ง DiDi จากย่านเมืองเก่า มุ่งหน้าสู่ตลาดสดและสตรีทฟู้ดต้ากวนจ้วนซิน</v>
       </c>
       <c r="E11" t="str">
-        <v>昆明老街 [250201] ➔ 大观篆新农贸市场 [250202]</v>
+        <v>昆明老街 [250201]  大观篆新农贸市场 [250202]</v>
       </c>
       <c r="F11" t="str">
         <v>Didi</v>
@@ -873,7 +873,7 @@
         <v>นั่งรถไฟใต้ดิน Metro สาย 6 กลับโรงแรมเถิงหัง เพื่อรับกระเป๋าเดินทางใหญ่ที่ฝากไว้</v>
       </c>
       <c r="E13" t="str">
-        <v>大观篆新 [250301] ➔ 腾航大酒店 [250302]</v>
+        <v>大观篆新 [250301]  腾航大酒店 [250302]</v>
       </c>
       <c r="F13" t="str">
         <v>รถไฟ</v>
@@ -911,7 +911,7 @@
         <v>นั่ง Shuttle Bus / DiDi จากโรงแรมไปอาคารผู้โดยสารสนามบินคุนหมิงฉางสุ่ย</v>
       </c>
       <c r="E14" t="str">
-        <v>腾航大酒店 ➔ 昆明长水</v>
+        <v>腾航大酒店  昆明长水</v>
       </c>
       <c r="F14" t="str">
         <v>Didi / รถตู้</v>
@@ -984,7 +984,7 @@
         <v>22:45 – 23:45</v>
       </c>
       <c r="D16" t="str">
-        <v>✈️ เที่ยวบิน MU-5923: คุนหมิง (KMG) ➔ ลี่เจียงซานอี้ (LJG) (บินตรง 1 ชม. ถึง 23:45 น.)</v>
+        <v>เที่ยวบิน MU-5923: คุนหมิง (KMG)  ลี่เจียงซานอี้ (LJG) (บินตรง 1 ชม. ถึง 23:45 น.)</v>
       </c>
       <c r="E16" t="str">
         <v>丽江三义国际机场</v>
@@ -1063,7 +1063,7 @@
         <v>เช็กเอาต์ เรียก DiDi ยิงตรงจากที่พักสนามบิน สู่ที่พักเมืองเก่าลี่เจียง (~28 กม.) ไม่ต้องต่อบัส ไม่ต้องลากกระเป๋า</v>
       </c>
       <c r="E18" t="str">
-        <v>丽江龙落河民宿 [260001] ➔ 栖悦林隐别院</v>
+        <v>丽江龙落河民宿 [260001]  栖悦林隐别院</v>
       </c>
       <c r="F18" t="str">
         <v>Didi</v>
@@ -1139,7 +1139,7 @@
         <v>เส้นทางเดิน 3 จุด: เดิน 2-3 นาทีไปกินหม้อไฟซี่โครงหมูอาผอฉิง แล้วเดินย่อยอาหารลงใต้ไปสถานีขนส่งลี่เจียง ซื้อตั๋วบัสไปสะพานเฉียวโถวรอบเช้า</v>
       </c>
       <c r="E20" t="str">
-        <v>栖悦林隐别院 [260101] ➔ 阿婆情腊排骨(忠义店) [260102] ➔ 丽江客运站 [260103]</v>
+        <v>栖悦林隐别院 [260101]  阿婆情腊排骨(忠义店) [260102]  丽江客运站 [260103]</v>
       </c>
       <c r="F20" t="str">
         <v>เดิน</v>
@@ -1174,10 +1174,10 @@
         <v>13:45 – 14:15</v>
       </c>
       <c r="D21" t="str">
-        <v>เรียก DiDi จากหน้าสถานีขนส่งลี่เจียง ตรงขึ้นไปสระมังกรดำ (黑龙潭公园) เพียง 15 นาที ประหยัดแรงขา</v>
+        <v>เดินเที่ยวไฮไลท์ 7 จุด: สระมังกรดำ (เต๋อเยวี่ยโหลว, สะพานสั่วชุ่ยเฉียว), กังหันน้ำใหญ่, จัตุรัสซื่อฟางเจีย, สะพานหินต้าสือเฉียว, ถ่ายรูปหน้าคฤหาสน์ตระกูลมู่ (ไม่เข้าด้านใน), เดินเข้าที่พัก</v>
       </c>
       <c r="E21" t="str">
-        <v>丽江客运站 [260201] ➔ 黑龙潭公园-得月楼 [260202]</v>
+        <v>丽江客运站 [260201]  黑龙潭公园-得月楼 [260202]</v>
       </c>
       <c r="F21" t="str">
         <v>Didi</v>
@@ -1186,19 +1186,19 @@
         <v>-</v>
       </c>
       <c r="H21">
-        <v>6.5</v>
+        <v>0</v>
       </c>
       <c r="I21">
-        <v>32.5</v>
+        <v>0</v>
       </c>
       <c r="J21">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="K21">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="L21" t="str">
-        <v>DiDi ตรง ไม่ต้องเดินย้อน</v>
+        <v>ชมสถาปัตยกรรมด้านนอก / ฟรี</v>
       </c>
     </row>
     <row r="22">
@@ -1212,10 +1212,10 @@
         <v>14:15 – 18:30</v>
       </c>
       <c r="D22" t="str">
-        <v>เดินเที่ยวไฮไลท์ 7 จุด: สระมังกรดำ (เต๋อเยวี่ยโหลว, สะพานสั่วชุ่ยเฉียว), กังหันน้ำใหญ่, จัตุรัสซื่อฟางเจีย, สะพานหินต้าสือเฉียว, คฤหาสน์ตระกูลมู่, เดินเข้าที่พัก</v>
+        <v>เดินเที่ยวไฮไลท์ 7 จุด: สระมังกรดำ (เต๋อเยวี่ยโหลว, สะพานสั่วชุ่ยเฉียว), กังหันน้ำใหญ่, จัตุรัสซื่อฟางเจีย, สะพานหินต้าสือเฉียว, ถ่ายรูปหน้าคฤหาสน์ตระกูลมู่ (ไม่เข้าด้านใน), เดินเข้าที่พัก</v>
       </c>
       <c r="E22" t="str">
-        <v>得月楼 [260301] ➔ 锁翠桥 [260302] ➔ 大水车 [260303] ➔ 四方街 [260304] ➔ 大石桥 [260305] ➔ 木府 [260306] ➔ 栖悦林隐别院 [260307]</v>
+        <v>得月楼 [260301]  锁翠桥 [260302]  大水车 [260303]  四方街 [260304]  大石桥 [260305]  木府 [260306]  栖悦林隐别院 [260307]</v>
       </c>
       <c r="F22" t="str">
         <v>เดิน</v>
@@ -1224,19 +1224,19 @@
         <v>https://surl.amap.com/2CRjOXV82fSQ</v>
       </c>
       <c r="H22">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="I22">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="J22">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="K22">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="L22" t="str">
-        <v>ค่าบำรุงเมืองเก่า / เข้าคฤหาสน์มู่</v>
+        <v>ชมสถาปัตยกรรมด้านนอก / ฟรี</v>
       </c>
     </row>
     <row r="23">
@@ -1253,7 +1253,7 @@
         <v>เดิน 2-3 นาทีไปชิมสตรีทฟู้ดและปิ้งย่างหม่าล่าที่ถนนคนเดินตลาดโต้รุ่งจงอี้</v>
       </c>
       <c r="E23" t="str">
-        <v>栖悦林隐别院 [260401] ➔ 忠义市场夜市街 [260402]</v>
+        <v>栖悦林隐别院 [260401]  忠义市场夜市街 [260402]</v>
       </c>
       <c r="F23" t="str">
         <v>เดิน</v>
@@ -1329,7 +1329,7 @@
         <v>เช็กเอาต์ เดิน 900 ม. ไปสถานีขนส่งลี่เจียง แจ้งคนขับฝากส่งกระเป๋าใหญ่ 20 กก. ขึ้นรถไปรอที่ Tina's</v>
       </c>
       <c r="E25" t="str">
-        <v>丽江客运站 ➔ Tina's</v>
+        <v>丽江客运站  Tina's</v>
       </c>
       <c r="F25" t="str">
         <v>เดิน</v>
@@ -1367,7 +1367,7 @@
         <v>นั่งรถบัสชมวิวแม่น้ำจินชา สู่สะพานเฉียวโถว (Qiaotou) ซื้อตั๋วเข้าอุทยานเสือกระโจน</v>
       </c>
       <c r="E26" t="str">
-        <v>丽江客运站 ➔ 桥头镇</v>
+        <v>丽江客运站  桥头镇</v>
       </c>
       <c r="F26" t="str">
         <v>รถบัส</v>
@@ -1405,7 +1405,7 @@
         <v>ทริคเด็ดประหยัดแรง: ต่อรถตู้ท้องถิ่นที่ปากทาง ขับตัดทางลูกรัง 2 ชม. ขึ้นตรงสู่หน้า Naxi Family</v>
       </c>
       <c r="E27" t="str">
-        <v>桥头 ➔ 纳西雅阁客栈</v>
+        <v>桥头  纳西雅阁客栈</v>
       </c>
       <c r="F27" t="str">
         <v>รถตู้</v>
@@ -1671,7 +1671,7 @@
         <v>เดิน High Trail เลียบผา ผ่าน Halfway Guesthouse และละอองน้ำตกกวนอิม ลัดเลาะลงสู่ Tina's (~3.5 ชม.)</v>
       </c>
       <c r="E34" t="str">
-        <v>中途客栈 ➔ 观音瀑布 ➔ 中峡蒂娜青年旅舍</v>
+        <v>中途客栈  观音瀑布  中峡蒂娜青年旅舍</v>
       </c>
       <c r="F34" t="str">
         <v>เดิน</v>
@@ -1747,7 +1747,7 @@
         <v>รถบัสสายตรงข้ามที่ราบสูงทิเบต สู่เมืองโบราณตู๋เค่อจง แชงกรี-ลา (~2 ชม.)</v>
       </c>
       <c r="E36" t="str">
-        <v>Tina's ➔ 独克宗古城</v>
+        <v>Tina's  独克宗古城</v>
       </c>
       <c r="F36" t="str">
         <v>รถบัส</v>
@@ -1785,7 +1785,7 @@
         <v>ถึงประตูเหนือตู๋เค่อจง ลากกระเป๋าเข้าเช็กอินโรงแรม Wangshan Xiaoyuan Inn เปลี่ยนใส่เสื้อหนาวหนา</v>
       </c>
       <c r="E37" t="str">
-        <v>独克宗古城(北门) [280101] ➔ 望山小院客栈 [280102]</v>
+        <v>独克宗古城(北门) [280101]  望山小院客栈 [280102]</v>
       </c>
       <c r="F37" t="str">
         <v>เดิน</v>
@@ -1934,10 +1934,10 @@
         <v>08:20 – 09:05</v>
       </c>
       <c r="D41" t="str">
-        <v>🚌 รถบัสตรงสู่ผู่ต๋าชั่ว: ชมวิวธรรมชาติที่ราบสูงยูนนาน</v>
+        <v>รถบัสตรงสู่ผู่ต๋าชั่ว: ชมวิวธรรมชาติที่ราบสูงยูนนาน</v>
       </c>
       <c r="E41" t="str">
-        <v>独克宗东门 ➔ 普达措国家公园</v>
+        <v>独克宗东门  普达措国家公园</v>
       </c>
       <c r="F41" t="str">
         <v>รถบัส</v>
@@ -2010,10 +2010,10 @@
         <v>15:00 – 15:45</v>
       </c>
       <c r="D43" t="str">
-        <v>🚌 รถบัสขากลับ: จากผู่ต๋าชั่วกลับมาส่งที่ประตูตะวันออกตู๋เค่อจง</v>
+        <v>รถบัสขากลับ: จากผู่ต๋าชั่วกลับมาส่งที่ประตูตะวันออกตู๋เค่อจง</v>
       </c>
       <c r="E43" t="str">
-        <v>普达措 ➔ 独克宗东门</v>
+        <v>普达措  独克宗东门</v>
       </c>
       <c r="F43" t="str">
         <v>รถบัส</v>
@@ -2165,7 +2165,7 @@
         <v>เดินจากที่พักไปสัมผัสวิถีชีวิตชาวบ้านที่ตลาดเช้าเซี่ยงหยาง ชิมอาหารเช้าพื้นเมือง</v>
       </c>
       <c r="E47" t="str">
-        <v>望山小院客栈 ➔ 金桥向阳菜市场</v>
+        <v>望山小院客栈  金桥向阳菜市场</v>
       </c>
       <c r="F47" t="str">
         <v>เดิน</v>
@@ -2203,7 +2203,7 @@
         <v>นั่งรถเมล์สาย 3 ไปชมความวิจิตรของ "พระราชวังโปตาลัย้อยุค" วัดซงจ้านหลิน</v>
       </c>
       <c r="E48" t="str">
-        <v>金桥向阳菜市场 ➔ 噶丹松赞林寺</v>
+        <v>金桥向阳菜市场  噶丹松赞林寺</v>
       </c>
       <c r="F48" t="str">
         <v>รถบัส</v>
@@ -2279,7 +2279,7 @@
         <v>นั่งรถเมล์ขากลับจากวัดซงจ้านหลิน สู่ที่พัก Wangshan Xiaoyuan Inn</v>
       </c>
       <c r="E50" t="str">
-        <v>噶丹松赞林寺 ➔ 望山小院客栈</v>
+        <v>噶丹松赞林寺  望山小院客栈</v>
       </c>
       <c r="F50" t="str">
         <v>รถบัส</v>
@@ -2317,7 +2317,7 @@
         <v>เช็กเอาต์ ลากกระเป๋า นั่งรถบัส/รถเมล์ไปสถานีรถไฟความเร็วสูงแชงกรี-ลา</v>
       </c>
       <c r="E51" t="str">
-        <v>望山小院客栈 ➔ 香格里拉站(进站口)</v>
+        <v>望山小院客栈  香格里拉站(进站口)</v>
       </c>
       <c r="F51" t="str">
         <v>รถบัส</v>
@@ -2352,10 +2352,10 @@
         <v>14:45 – 16:15</v>
       </c>
       <c r="D52" t="str">
-        <v>🚄 นั่งรถไฟความเร็วสูง C-Train ชมวิวช่องเขาหิมะกลับสู่สถานีรถไฟลี่เจียง (~1.5 ชม.)</v>
+        <v>นั่งรถไฟความเร็วสูง C-Train ชมวิวช่องเขาหิมะกลับสู่สถานีรถไฟลี่เจียง (~1.5 ชม.)</v>
       </c>
       <c r="E52" t="str">
-        <v>香格里拉站 ➔ 丽江站</v>
+        <v>香格里拉站  丽江站</v>
       </c>
       <c r="F52" t="str">
         <v>รถไฟเร็วสูง</v>
@@ -2393,7 +2393,7 @@
         <v>ถึงสถานีรถไฟลี่เจียง นั่งรถบัสสายตรงเข้าเมืองเก่าลี่เจียง</v>
       </c>
       <c r="E53" t="str">
-        <v>丽江站 ➔ 栖悦林隐别院</v>
+        <v>丽江站  栖悦林隐别院</v>
       </c>
       <c r="F53" t="str">
         <v>รถบัส</v>
@@ -2414,7 +2414,7 @@
         <v>50</v>
       </c>
       <c r="L53" t="str">
-        <v>รถบัสสถานีรถไฟ ➔ เมืองเก่า</v>
+        <v>รถบัสสถานีรถไฟ  เมืองเก่า</v>
       </c>
     </row>
     <row r="54">
@@ -2469,7 +2469,7 @@
         <v>เดินเล่น ซื้อของฝาก และกินมื้อค่ำเก็บตกที่ถนนคนเดินตลาดโต้รุ่งจงอี้</v>
       </c>
       <c r="E55" t="str">
-        <v>栖悦林隐别院 ➔ 忠义市场夜市街</v>
+        <v>栖悦林隐别院  忠义市场夜市街</v>
       </c>
       <c r="F55" t="str">
         <v>เดิน</v>
@@ -2507,7 +2507,7 @@
         <v>เช็กเอาต์แต่เช้า เรียก DiDi จากที่พักตรงไปสนามบินลี่เจียง ซานอี้ (~28 กม.)</v>
       </c>
       <c r="E56" t="str">
-        <v>栖悦林隐别院 [260001] ➔ 丽江龙落河民宿(三义机场店)</v>
+        <v>栖悦林隐别院 [260001]  丽江龙落河民宿(三义机场店)</v>
       </c>
       <c r="F56" t="str">
         <v>Didi</v>
@@ -2580,10 +2580,10 @@
         <v>10:00 – 11:00</v>
       </c>
       <c r="D58" t="str">
-        <v>✈️ เที่ยวบิน MU-5922: ลี่เจียง (LJG) ➔ คุนหมิงฉางสุ่ย (KMG) (บิน 1 ชม. ถึงคุนหมิง 11:00 น.)</v>
+        <v>เที่ยวบิน MU-5922: ลี่เจียง (LJG)  คุนหมิงฉางสุ่ย (KMG) (บิน 1 ชม. ถึงคุนหมิง 11:00 น.)</v>
       </c>
       <c r="E58" t="str">
-        <v>丽江三义 ➔ 昆明长水</v>
+        <v>丽江三义  昆明长水</v>
       </c>
       <c r="F58" t="str">
         <v>เครื่องบิน</v>
@@ -2621,7 +2621,7 @@
         <v>นั่งรถไฟใต้ดิน Metro สาย 6 ต่อสาย 3/4 จากสนามบินคุนหมิง เข้าเมืองไปร้านอาหารกว่างอี้</v>
       </c>
       <c r="E59" t="str">
-        <v>昆明长水国际机场 ➔ 广益饭店(北门街)</v>
+        <v>昆明长水国际机场  广益饭店(北门街)</v>
       </c>
       <c r="F59" t="str">
         <v>รถไฟ</v>
@@ -2697,7 +2697,7 @@
         <v>เดินเที่ยวคุนหมิงตัวเบา 4 จุดต่อเนื่อง: 1. กว่างอี้ 2. สวนชุ่ยหู บึงบัวนกนางนวล 3. โรงเรียนการทหารเจี่ยงอู่ถัง 4. ถนนคนเดินหนานผิง</v>
       </c>
       <c r="E61" t="str">
-        <v>广益饭店 ➔ 翠湖公园 ➔ 云南陆军讲武堂历史博物馆 ➔ 南屏步行街</v>
+        <v>广益饭店  翠湖公园  云南陆军讲武堂历史博物馆  南屏步行街</v>
       </c>
       <c r="F61" t="str">
         <v>เดิน</v>
@@ -2735,7 +2735,7 @@
         <v>นั่งรถไฟใต้ดิน Metro จากถนนคนเดินหนานผิง ตรงกลับสู่สนามบินคุนหมิงฉางสุ่ย</v>
       </c>
       <c r="E62" t="str">
-        <v>南屏步行街 ➔ 昆明长水国际机场</v>
+        <v>南屏步行街  昆明长水国际机场</v>
       </c>
       <c r="F62" t="str">
         <v>รถไฟ</v>
@@ -2808,10 +2808,10 @@
         <v>21:30 – 23:05</v>
       </c>
       <c r="D64" t="str">
-        <v>✈️ เที่ยวบิน MU-9621: คุนหมิง (KMG) ➔ สุวรรณภูมิ (BKK) (บินตรง 1 ชม. 35 นาที) ถึงไทย 23:05 น. รับกระเป๋าที่สายพาน จบทริปโดยสวัสดิภาพ!</v>
+        <v>เที่ยวบิน MU-9621: คุนหมิง (KMG)  สุวรรณภูมิ (BKK) (บินตรง 1 ชม. 35 นาที) ถึงไทย 23:05 น. รับกระเป๋าที่สายพาน จบทริปโดยสวัสดิภาพ!</v>
       </c>
       <c r="E64" t="str">
-        <v>昆明 ➔ กรุงเทพฯ (BKK)</v>
+        <v>昆明  กรุงเทพฯ (BKK)</v>
       </c>
       <c r="F64" t="str">
         <v>เครื่องบิน</v>
@@ -2844,16 +2844,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G28"/>
-  <cols>
-    <col min="1" max="1" width="32.83203125" customWidth="1"/>
-    <col min="2" max="2" width="45.83203125" customWidth="1"/>
-    <col min="3" max="3" width="25.83203125" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" customWidth="1"/>
-    <col min="5" max="5" width="18.83203125" customWidth="1"/>
-    <col min="6" max="6" width="20.83203125" customWidth="1"/>
-    <col min="7" max="7" width="20.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:G27"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2880,7 +2871,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>✈️ ตั๋วเครื่องบินไป-กลับ</v>
+        <v>ตั๋วเครื่องบินไป-กลับ</v>
       </c>
       <c r="B2" t="str">
         <v>China Eastern 4 เที่ยวบิน (BKK⇄KMG⇄LJG)</v>
@@ -2903,7 +2894,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>🏨 โรงแรมและที่พัก (7 คืน)</v>
+        <v>โรงแรมและที่พัก (7 คืน)</v>
       </c>
       <c r="B3" t="str">
         <v>คุนหมิง 1 คืน + ลี่เจียง 3 คืน + เสือกระโจน 1 คืน + แชงกรี-ลา 2 คืน</v>
@@ -2926,7 +2917,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>🚌 การเดินทางในประเทศจีน</v>
+        <v>การเดินทางในประเทศจีน</v>
       </c>
       <c r="B4" t="str">
         <v>DiDi 6 ครั้ง, Metro 5 ครั้ง, รถบัส, รถไฟความเร็วสูง, รถตู้, ฝากกระเป๋า</v>
@@ -2949,30 +2940,30 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>🎟️ ค่าเข้าชมและกิจกรรม</v>
+        <v>ค่าเข้าชมและกิจกรรม (3 จุด)</v>
       </c>
       <c r="B5" t="str">
-        <v>เสือกระโจน, คฤหาสน์มู่, อุทยานผู่ต๋าชั่ว, วัดซงจ้านหลิน</v>
+        <v>เสือกระโจน, อุทยานผู่ต๋าชั่ว, วัดซงจ้านหลิน</v>
       </c>
       <c r="C5" t="str">
         <v>จ่ายหน้างาน (Alipay/เคาน์เตอร์)</v>
       </c>
       <c r="D5">
-        <v>726</v>
+        <v>626</v>
       </c>
       <c r="E5">
-        <v>3630</v>
+        <v>3130</v>
       </c>
       <c r="F5">
-        <v>363</v>
+        <v>313</v>
       </c>
       <c r="G5">
-        <v>1815</v>
+        <v>1565</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>🛡️ เตรียมตัวก่อนเดินทาง</v>
+        <v>เตรียมตัวก่อนเดินทาง</v>
       </c>
       <c r="B6" t="str">
         <v>ประกันภัย Insurverse + SIM โรมมิ่งอินเทอร์เน็ต (2 ท่าน)</v>
@@ -2995,7 +2986,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>🍜 ค่าอาหารและเครื่องดื่ม</v>
+        <v>ค่าอาหารและเครื่องดื่ม</v>
       </c>
       <c r="B7" t="str">
         <v>อาหารมื้อหลักตลอด 8 วัน + สตรีทฟู้ด + คาเฟ่ (ประมาณการ)</v>
@@ -3027,21 +3018,21 @@
         <v>ครบทุกหมวดหมู่</v>
       </c>
       <c r="D8">
-        <v>6740.58</v>
+        <v>6640.58</v>
       </c>
       <c r="E8">
-        <v>33702.9</v>
+        <v>33202.9</v>
       </c>
       <c r="F8">
-        <v>3370.29</v>
+        <v>3320.29</v>
       </c>
       <c r="G8">
-        <v>16851.45</v>
+        <v>16601.45</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>📌 สรุปยอดการชำระเงิน</v>
+        <v>สรุปยอดการชำระเงิน</v>
       </c>
       <c r="B10" t="str">
         <v/>
@@ -3096,21 +3087,21 @@
         <v>สแกน Alipay/WeChat</v>
       </c>
       <c r="D12">
-        <v>2394</v>
+        <v>2294</v>
       </c>
       <c r="E12">
-        <v>11970</v>
+        <v>11470</v>
       </c>
       <c r="F12">
-        <v>1197</v>
+        <v>1147</v>
       </c>
       <c r="G12">
-        <v>5985</v>
+        <v>5735</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>🏨 รายละเอียดค่าที่พัก 7 คืน (อ้างอิง Trip.com ยืนยันแล้ว)</v>
+        <v>รายละเอียดค่าที่พัก 7 คืน (อ้างอิง Trip.com ยืนยันแล้ว)</v>
       </c>
       <c r="B14" t="str">
         <v/>
@@ -3294,7 +3285,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>🎟️ รายละเอียดค่าเข้าชมสถานที่ (2 ท่าน)</v>
+        <v>รายละเอียดค่าเข้าชมสถานที่ (2 ท่าน)</v>
       </c>
       <c r="B23" t="str">
         <v/>
@@ -3340,99 +3331,76 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>คฤหาสน์มู่และเมืองเก่าลี่เจียง (Mu Mansion)</v>
+        <v>อุทยานแห่งชาติผู่ต๋าชั่ว (Potatso National Park)</v>
       </c>
       <c r="B25" t="str">
-        <v>ค่าธรรมเนียมเข้าชม (คนละ ¥50)</v>
+        <v>แพ็กเกจบัตรรวม + ชัตเติลบัส + รถรับส่ง (คนละ ¥178)</v>
       </c>
       <c r="C25" t="str">
-        <v>ซื้อหน้าทางเข้า</v>
+        <v>จองล่วงหน้า/หน้างาน</v>
       </c>
       <c r="D25">
-        <v>100</v>
+        <v>356</v>
       </c>
       <c r="E25">
-        <v>500</v>
+        <v>1780</v>
       </c>
       <c r="F25">
-        <v>50</v>
+        <v>178</v>
       </c>
       <c r="G25">
-        <v>250</v>
+        <v>890</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>อุทยานแห่งชาติผู่ต๋าชั่ว (Potatso National Park)</v>
+        <v>วัดกาด่านซงจ้านหลิน (Songzanlin Monastery)</v>
       </c>
       <c r="B26" t="str">
-        <v>แพ็กเกจบัตรรวม + ชัตเติลบัส + รถรับส่ง (คนละ ¥178)</v>
+        <v>ค่าเข้าชมวัด + บัสในวัด (คนละ ¥90)</v>
       </c>
       <c r="C26" t="str">
-        <v>จองล่วงหน้า/หน้างาน</v>
+        <v>ซื้อศูนย์บริการ</v>
       </c>
       <c r="D26">
-        <v>356</v>
+        <v>180</v>
       </c>
       <c r="E26">
-        <v>1780</v>
+        <v>900</v>
       </c>
       <c r="F26">
-        <v>178</v>
+        <v>90</v>
       </c>
       <c r="G26">
-        <v>890</v>
+        <v>450</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>วัดกาด่านซงจ้านหลิน (Songzanlin Monastery)</v>
+        <v>รวมค่าเข้าชมสถานที่</v>
       </c>
       <c r="B27" t="str">
-        <v>ค่าเข้าชมวัด + บัสในวัด (คนละ ¥90)</v>
+        <v>รวม 3 แหล่งท่องเที่ยว (2 ท่าน)</v>
       </c>
       <c r="C27" t="str">
-        <v>ซื้อศูนย์บริการ</v>
+        <v>จ่ายหน้างาน</v>
       </c>
       <c r="D27">
-        <v>180</v>
+        <v>626</v>
       </c>
       <c r="E27">
-        <v>900</v>
+        <v>3130</v>
       </c>
       <c r="F27">
-        <v>90</v>
+        <v>313</v>
       </c>
       <c r="G27">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="str">
-        <v>รวมค่าเข้าชมสถานที่</v>
-      </c>
-      <c r="B28" t="str">
-        <v>รวม 4 แหล่งท่องเที่ยว (2 ท่าน)</v>
-      </c>
-      <c r="C28" t="str">
-        <v>จ่ายหน้างาน</v>
-      </c>
-      <c r="D28">
-        <v>726</v>
-      </c>
-      <c r="E28">
-        <v>3630</v>
-      </c>
-      <c r="F28">
-        <v>363</v>
-      </c>
-      <c r="G28">
-        <v>1815</v>
+        <v>1565</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G28"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G27"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4196,16 +4164,16 @@
         <v>260301</v>
       </c>
       <c r="G22">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="H22">
         <v>5</v>
       </c>
       <c r="I22">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="J22">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="K22" t="str">
         <v/>
@@ -5911,19 +5879,19 @@
         <v/>
       </c>
       <c r="G71">
-        <v>391.5</v>
+        <v>341.5</v>
       </c>
       <c r="H71">
         <v>5</v>
       </c>
       <c r="I71">
-        <v>1957.5</v>
+        <v>1707.5</v>
       </c>
       <c r="J71">
-        <v>3915</v>
+        <v>3415</v>
       </c>
       <c r="K71" t="str">
-        <v>ยอดรวม 2 คน = ¥783.00 (฿3,915.00) | เฉลี่ยคนละ ¥391.50 (฿1,957.50)</v>
+        <v>ยอดรวม 2 คน = ¥683.00 (฿3,415.00) | เฉลี่ยคนละ ¥341.50 (฿1,707.50)</v>
       </c>
     </row>
   </sheetData>
@@ -5986,7 +5954,7 @@
         <v>Didi</v>
       </c>
       <c r="E2" t="str">
-        <v>昆明长水国际机场 ➔ 腾航大酒店(昆明长水国际机场店)</v>
+        <v>昆明长水国际机场  腾航大酒店(昆明长水国际机场店)</v>
       </c>
       <c r="F2" t="str">
         <v>-</v>
@@ -6021,7 +5989,7 @@
         <v>รถไฟ</v>
       </c>
       <c r="E3" t="str">
-        <v>腾航大酒店(昆明长水国际机场店) [250001] ➔ 建新园·云南过桥米线(宝善街店) [250002]</v>
+        <v>腾航大酒店(昆明长水国际机场店) [250001]  建新园·云南过桥米线(宝善街店) [250002]</v>
       </c>
       <c r="F3" t="str">
         <v>https://surl.amap.com/20U4Hpku15Tq</v>
@@ -6056,7 +6024,7 @@
         <v>เดิน</v>
       </c>
       <c r="E4" t="str">
-        <v>建新园·云南过桥米线(宝善街店) [250101] ➔ 金马碧鸡坊 [250102] ➔ 南屏步行街 [250103]</v>
+        <v>建新园·云南过桥米线(宝善街店) [250101]  金马碧鸡坊 [250102]  南屏步行街 [250103]</v>
       </c>
       <c r="F4" t="str">
         <v>https://surl.amap.com/33RYtbCG73zK</v>
@@ -6091,7 +6059,7 @@
         <v>Didi</v>
       </c>
       <c r="E5" t="str">
-        <v>昆明老街 [250201] ➔ 大观篆新农贸市场 [250202]</v>
+        <v>昆明老街 [250201]  大观篆新农贸市场 [250202]</v>
       </c>
       <c r="F5" t="str">
         <v>-</v>
@@ -6126,7 +6094,7 @@
         <v>รถไฟ</v>
       </c>
       <c r="E6" t="str">
-        <v>大观篆新农贸市场 [250301] ➔ 腾航大酒店(昆明长水国际机场店) [250302]</v>
+        <v>大观篆新农贸市场 [250301]  腾航大酒店(昆明长水国际机场店) [250302]</v>
       </c>
       <c r="F6" t="str">
         <v>https://surl.amap.com/356K2vgmT04T</v>
@@ -6161,7 +6129,7 @@
         <v>Didi</v>
       </c>
       <c r="E7" t="str">
-        <v>腾航大酒店(昆明长水国际机场店) ➔ 昆明长水国际机场</v>
+        <v>腾航大酒店(昆明长水国际机场店)  昆明长水国际机场</v>
       </c>
       <c r="F7" t="str">
         <v>-</v>
@@ -6196,7 +6164,7 @@
         <v>Didi</v>
       </c>
       <c r="E8" t="str">
-        <v>丽江龙落河民宿(三义国际机场店) [260001] ➔ 栖悦林隐别院(丽江古城忠义市场店)</v>
+        <v>丽江龙落河民宿(三义国际机场店) [260001]  栖悦林隐别院(丽江古城忠义市场店)</v>
       </c>
       <c r="F8" t="str">
         <v>-</v>
@@ -6231,7 +6199,7 @@
         <v>เดิน</v>
       </c>
       <c r="E9" t="str">
-        <v>栖悦林隐别院(丽江古城忠义市场店) [260101] ➔ 阿婆情腊排骨火锅·野生菌季(忠义店) [260102] ➔ 丽江客运站 [260103]</v>
+        <v>栖悦林隐别院(丽江古城忠义市场店) [260101]  阿婆情腊排骨火锅·野生菌季(忠义店) [260102]  丽江客运站 [260103]</v>
       </c>
       <c r="F9" t="str">
         <v>https://surl.amap.com/2Dsj0YlcXfGw</v>
@@ -6266,7 +6234,7 @@
         <v>Didi</v>
       </c>
       <c r="E10" t="str">
-        <v>丽江客运站 [260201] ➔ 得月楼 [260202]</v>
+        <v>丽江客运站 [260201]  得月楼 [260202]</v>
       </c>
       <c r="F10" t="str">
         <v>-</v>
@@ -6301,25 +6269,25 @@
         <v>เดิน</v>
       </c>
       <c r="E11" t="str">
-        <v>黑龙潭公园-得月楼 [260301] ➔ 锁翠桥 [260302] ➔ 丽江古城-古城大水车 [260303] ➔ 四方街 [260304] ➔ 大石桥 [260305] ➔ 丽江古城博物院-木府 [260306] ➔ 栖悦林隐别院(丽江古城忠义市场店) [260307]</v>
+        <v>黑龙潭公园-得月楼 [260301]  锁翠桥 [260302]  丽江古城-古城大水车 [260303]  四方街 [260304]  大石桥 [260305]  丽江古城博物院-木府 [260306]  栖悦林隐别院(丽江古城忠义市场店) [260307]</v>
       </c>
       <c r="F11" t="str">
         <v>https://surl.amap.com/2CRjOXV82fSQ</v>
       </c>
       <c r="G11">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="H11">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="I11">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="J11">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="K11" t="str">
-        <v>-</v>
+        <v>ชมสถาปัตยกรรมด้านนอก / ฟรี</v>
       </c>
     </row>
     <row r="12">
@@ -6336,7 +6304,7 @@
         <v>เดิน</v>
       </c>
       <c r="E12" t="str">
-        <v>栖悦林隐别院(丽江古城忠义市场店) [260401] ➔ 忠义市场夜市街 [260402]</v>
+        <v>栖悦林隐别院(丽江古城忠义市场店) [260401]  忠义市场夜市街 [260402]</v>
       </c>
       <c r="F12" t="str">
         <v>https://surl.amap.com/2HSTS4Jc155an</v>
@@ -6371,7 +6339,7 @@
         <v>รถบัส</v>
       </c>
       <c r="E13" t="str">
-        <v>丽江客运站 ➔ 纳西雅阁客栈</v>
+        <v>丽江客运站  纳西雅阁客栈</v>
       </c>
       <c r="F13" t="str">
         <v>-</v>
@@ -6406,7 +6374,7 @@
         <v>เดิน</v>
       </c>
       <c r="E14" t="str">
-        <v>纳西雅阁客栈 ➔ 香格里拉山美客栈(东环线分店)</v>
+        <v>纳西雅阁客栈  香格里拉山美客栈(东环线分店)</v>
       </c>
       <c r="F14" t="str">
         <v>-</v>
@@ -6441,7 +6409,7 @@
         <v>เดิน</v>
       </c>
       <c r="E15" t="str">
-        <v>香格里拉山美客栈(东环线分店) ➔ 中峡国际青年旅舍Tina'S Guest House</v>
+        <v>香格里拉山美客栈(东环线分店)  中峡国际青年旅舍Tina'S Guest House</v>
       </c>
       <c r="F15" t="str">
         <v>-</v>
@@ -6476,7 +6444,7 @@
         <v>เดิน</v>
       </c>
       <c r="E16" t="str">
-        <v>香格里拉市独克宗古城(北门) [280101] ➔ 香格里拉望山小院客栈(独克宗古城店) [280102] ➔ 静静的嘛呢石藏餐吧(北门店) [280103] ➔ 龟山公园 [280104]</v>
+        <v>香格里拉市独克宗古城(北门) [280101]  香格里拉望山小院客栈(独克宗古城店) [280102]  静静的嘛呢石藏餐吧(北门店) [280103]  龟山公园 [280104]</v>
       </c>
       <c r="F16" t="str">
         <v>https://surl.amap.com/2Q0zUvse1n2aI</v>
@@ -6511,7 +6479,7 @@
         <v>รถบัส</v>
       </c>
       <c r="E17" t="str">
-        <v>香格里拉独克宗古城东门客运站售票点 ➔ 普达措国家公园入口游客中心</v>
+        <v>香格里拉独克宗古城东门客运站售票点  普达措国家公园入口游客中心</v>
       </c>
       <c r="F17" t="str">
         <v>-</v>
@@ -6546,7 +6514,7 @@
         <v>รถบัส</v>
       </c>
       <c r="E18" t="str">
-        <v>普达措国家公园入口游客中心 ➔ 香格里拉独克宗古城东门客运站售票点</v>
+        <v>普达措国家公园入口游客中心  香格里拉独克宗古城东门客运站售票点</v>
       </c>
       <c r="F18" t="str">
         <v>-</v>
@@ -6581,7 +6549,7 @@
         <v>เดิน</v>
       </c>
       <c r="E19" t="str">
-        <v>香格里拉望山小院客栈(独克宗古城店) ➔ 古城角落甜茶馆 ➔ 宏宏无烟石板烧烤</v>
+        <v>香格里拉望山小院客栈(独克宗古城店)  古城角落甜茶馆  宏宏无烟石板烧烤</v>
       </c>
       <c r="F19" t="str">
         <v>https://surl.amap.com/3aWWUho1o6Qb</v>
@@ -6616,7 +6584,7 @@
         <v>เดิน</v>
       </c>
       <c r="E20" t="str">
-        <v>香格里拉望山小院客栈(独克宗古城店) ➔ 金桥向阳菜市场(向阳路农贸综合市场店)</v>
+        <v>香格里拉望山小院客栈(独克宗古城店)  金桥向阳菜市场(向阳路农贸综合市场店)</v>
       </c>
       <c r="F20" t="str">
         <v>https://surl.amap.com/37LSs3sS8SI</v>
@@ -6651,7 +6619,7 @@
         <v>รถบัส</v>
       </c>
       <c r="E21" t="str">
-        <v>金桥向阳菜市场(向阳路农贸综合市场店) ➔ 噶丹松赞林寺 ➔ 游客服务中心 (กินข้าว)</v>
+        <v>金桥向阳菜市场(向阳路农贸综合市场店)  噶丹松赞林寺  游客服务中心 (กินข้าว)</v>
       </c>
       <c r="F21" t="str">
         <v>https://surl.amap.com/fe10g66KcYw</v>
@@ -6686,7 +6654,7 @@
         <v>รถบัส</v>
       </c>
       <c r="E22" t="str">
-        <v>噶丹松赞林寺 ➔ 香格里拉望山小院客栈(独克宗古城店)</v>
+        <v>噶丹松赞林寺  香格里拉望山小院客栈(独克宗古城店)</v>
       </c>
       <c r="F22" t="str">
         <v>https://surl.amap.com/2RRM1kq6aIj</v>
@@ -6721,7 +6689,7 @@
         <v>รถบัส</v>
       </c>
       <c r="E23" t="str">
-        <v>香格里拉望山小院客栈(独克宗古城店) ➔ 香格里拉站(进站口)</v>
+        <v>香格里拉望山小院客栈(独克宗古城店)  香格里拉站(进站口)</v>
       </c>
       <c r="F23" t="str">
         <v>https://surl.amap.com/yN182yJoaRv</v>
@@ -6756,7 +6724,7 @@
         <v>รถบัส</v>
       </c>
       <c r="E24" t="str">
-        <v>丽江站 ➔ 栖悦林隐别院(丽江古城忠义市场店)</v>
+        <v>丽江站  栖悦林隐别院(丽江古城忠义市场店)</v>
       </c>
       <c r="F24" t="str">
         <v>https://surl.amap.com/3n4lXMyfeuQ</v>
@@ -6791,7 +6759,7 @@
         <v>เดิน</v>
       </c>
       <c r="E25" t="str">
-        <v>栖悦林隐别院(丽江古城忠义市场店) ➔ 忠义市场夜市街</v>
+        <v>栖悦林隐别院(丽江古城忠义市场店)  忠义市场夜市街</v>
       </c>
       <c r="F25" t="str">
         <v>https://surl.amap.com/2HSTS4Jc155an</v>
@@ -6826,7 +6794,7 @@
         <v>Didi</v>
       </c>
       <c r="E26" t="str">
-        <v>栖悦林隐别院(丽江古城忠义市场店) [260001] ➔ 丽江龙落河民宿(三义国际机场店)</v>
+        <v>栖悦林隐别院(丽江古城忠义市场店) [260001]  丽江龙落河民宿(三义国际机场店)</v>
       </c>
       <c r="F26" t="str">
         <v>-</v>
@@ -6861,7 +6829,7 @@
         <v>รถไฟ</v>
       </c>
       <c r="E27" t="str">
-        <v>昆明长水国际机场 ➔ 广益饭店(北门街)</v>
+        <v>昆明长水国际机场  广益饭店(北门街)</v>
       </c>
       <c r="F27" t="str">
         <v>https://surl.amap.com/4psCbGureAF</v>
@@ -6896,7 +6864,7 @@
         <v>เดิน</v>
       </c>
       <c r="E28" t="str">
-        <v>广益饭店(北门街) ➔ 翠湖公园 ➔ 云南陆军讲武堂历史博物馆 ➔ 南屏步行街</v>
+        <v>广益饭店(北门街)  翠湖公园  云南陆军讲武堂历史博物馆  南屏步行街</v>
       </c>
       <c r="F28" t="str">
         <v>https://surl.amap.com/4r8LFT819c1S</v>
@@ -6931,7 +6899,7 @@
         <v>รถไฟ</v>
       </c>
       <c r="E29" t="str">
-        <v>南屏步行街 ➔ 昆明长水国际机场</v>
+        <v>南屏步行街  昆明长水国际机场</v>
       </c>
       <c r="F29" t="str">
         <v>https://surl.amap.com/tP208A1cceK</v>
@@ -7075,16 +7043,16 @@
         <v>5</v>
       </c>
       <c r="C4">
-        <v>92.5</v>
+        <v>42.5</v>
       </c>
       <c r="D4">
-        <v>463</v>
+        <v>212.5</v>
       </c>
       <c r="E4">
-        <v>185</v>
+        <v>85</v>
       </c>
       <c r="F4">
-        <v>925</v>
+        <v>425</v>
       </c>
       <c r="G4" t="str">
         <v>-</v>
@@ -7213,16 +7181,16 @@
         <v>28</v>
       </c>
       <c r="C10">
-        <v>391.5</v>
+        <v>341.5</v>
       </c>
       <c r="D10">
-        <v>1958</v>
+        <v>1707.5</v>
       </c>
       <c r="E10">
-        <v>783</v>
+        <v>683</v>
       </c>
       <c r="F10">
-        <v>3915</v>
+        <v>3415</v>
       </c>
       <c r="G10" t="str">
         <v>รวม 8 วัน (คณะ 2 คน)</v>

</xml_diff>

<commit_message>
v51: Move midnight activities (immigration, shuttle, hotel sleep) from Day 1 to Day 2 timeline per user request
</commit_message>
<xml_diff>
--- a/yunnan_travel_plan_2026.xlsx
+++ b/yunnan_travel_plan_2026.xlsx
@@ -557,10 +557,10 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>วันที่ 1 : 24 ต.ค. 2569 (ส.)</v>
+        <v>วันที่ 2 : 25 ต.ค. 2569 (อา.)</v>
       </c>
       <c r="B5" t="str">
-        <v>10/24/2026</v>
+        <v>10/25/2026</v>
       </c>
       <c r="C5" t="str">
         <v>00:30 – 01:30</v>
@@ -595,10 +595,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>วันที่ 1 : 24 ต.ค. 2569 (ส.)</v>
+        <v>วันที่ 2 : 25 ต.ค. 2569 (อา.)</v>
       </c>
       <c r="B6" t="str">
-        <v>10/24/2026</v>
+        <v>10/25/2026</v>
       </c>
       <c r="C6" t="str">
         <v>01:30 – 02:00</v>
@@ -633,10 +633,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>วันที่ 1 : 24 ต.ค. 2569 (ส.)</v>
+        <v>วันที่ 2 : 25 ต.ค. 2569 (อา.)</v>
       </c>
       <c r="B7" t="str">
-        <v>10/24/2026</v>
+        <v>10/25/2026</v>
       </c>
       <c r="C7" t="str">
         <v>02:00 – 10:00</v>
@@ -3446,7 +3446,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>10/24/2026</v>
+        <v>10/25/2026</v>
       </c>
       <c r="B2" t="str">
         <v>สนามบินคุนหมิง-ที่พักคุนหมิง</v>
@@ -5945,7 +5945,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>10/24/2026</v>
+        <v>10/25/2026</v>
       </c>
       <c r="C2" t="str">
         <v>สนามบินคุนหมิง-ที่พักคุนหมิง</v>
@@ -6994,16 +6994,16 @@
         <v>10/24/2026</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C2">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D2">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="E2">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F2">
         <v>50</v>
@@ -7017,16 +7017,16 @@
         <v>10/25/2026</v>
       </c>
       <c r="B3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C3">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="D3">
-        <v>110</v>
+        <v>135</v>
       </c>
       <c r="E3">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="F3">
         <v>220</v>

</xml_diff>

<commit_message>
v52: Remove Chinese text in parentheses from Thai text across all sections per user request
</commit_message>
<xml_diff>
--- a/yunnan_travel_plan_2026.xlsx
+++ b/yunnan_travel_plan_2026.xlsx
@@ -1478,7 +1478,7 @@
         <v>11:45 – 13:45</v>
       </c>
       <c r="D29" t="str">
-        <v>เริ่มเดินเที่ยงตรง: พิชิต 28 โค้งหักศอก (二十八道拐) สู่จุดสูงสุด 2,670 ม. วิว 360° แม่น้ำจินชา</v>
+        <v>เริ่มเดินเที่ยงตรง: พิชิต 28 โค้งหักศอก สู่จุดสูงสุด 2,670 ม. วิว 360° แม่น้ำจินชา</v>
       </c>
       <c r="E29" t="str">
         <v>二十八道拐 (28 Bends)</v>
@@ -2656,7 +2656,7 @@
         <v>12:15 – 13:30</v>
       </c>
       <c r="D60" t="str">
-        <v>กินมื้อเที่ยงอาหารยูนนานดั้งเดิมที่ร้านดัง กว่างอี้ฟั่นเตี้ยน (广益饭店·北门街)</v>
+        <v>กินมื้อเที่ยงอาหารยูนนานดั้งเดิมที่ร้านดัง กว่างอี้ฟั่นเตี้ยน</v>
       </c>
       <c r="E60" t="str">
         <v>广益饭店(北门街)</v>

</xml_diff>

<commit_message>
v53: Update โรงแรมเถิงหัง to transliterated Tenghang Hotel (腾航大酒店) per user request
</commit_message>
<xml_diff>
--- a/yunnan_travel_plan_2026.xlsx
+++ b/yunnan_travel_plan_2026.xlsx
@@ -604,7 +604,7 @@
         <v>01:30 – 02:00</v>
       </c>
       <c r="D6" t="str">
-        <v>ขึ้น Shuttle Bus ฟรี / DiDi หน้าอาคารผู้โดยสาร ตรงสู่โรงแรมเถิงหัง (~10 นาที)</v>
+        <v>ขึ้น Shuttle Bus ฟรี / DiDi หน้าอาคารผู้โดยสาร ตรงสู่Tenghang Hotel (~10 นาที)</v>
       </c>
       <c r="E6" t="str">
         <v>腾航大酒店(昆明长水国际机场店)</v>
@@ -680,7 +680,7 @@
         <v>10:00 – 11:00</v>
       </c>
       <c r="D8" t="str">
-        <v>เช็กเอาต์โรงแรมเถิงหัง ฝากกระเป๋าเดินทางใหญ่ 20 กก. ไว้ที่ฟรอนต์ฟรี สะพายเฉพาะเป้เล็กเข้าเมือง</v>
+        <v>เช็กเอาต์Tenghang Hotel ฝากกระเป๋าเดินทางใหญ่ 20 กก. ไว้ที่ฟรอนต์ฟรี สะพายเฉพาะเป้เล็กเข้าเมือง</v>
       </c>
       <c r="E8" t="str">
         <v>腾航大酒店</v>
@@ -870,7 +870,7 @@
         <v>18:30 – 19:30</v>
       </c>
       <c r="D13" t="str">
-        <v>นั่งรถไฟใต้ดิน Metro สาย 6 กลับโรงแรมเถิงหัง เพื่อรับกระเป๋าเดินทางใหญ่ที่ฝากไว้</v>
+        <v>นั่งรถไฟใต้ดิน Metro สาย 6 กลับTenghang Hotel เพื่อรับกระเป๋าเดินทางใหญ่ที่ฝากไว้</v>
       </c>
       <c r="E13" t="str">
         <v>大观篆新 [250301]  腾航大酒店 [250302]</v>

</xml_diff>

<commit_message>
Update master 9-sheet travel plan excel
</commit_message>
<xml_diff>
--- a/yunnan_travel_plan_2026.xlsx
+++ b/yunnan_travel_plan_2026.xlsx
@@ -3,11 +3,15 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="กำหนดการเดินทาง 8 วัน" sheetId="1" r:id="rId1"/>
-    <sheet name="สรุปงบประมาณ 2 คน" sheetId="2" r:id="rId2"/>
-    <sheet name="ตารางหลัก (Master Table)" sheetId="3" r:id="rId3"/>
-    <sheet name="สรุปช่วงการเดินทาง" sheetId="4" r:id="rId4"/>
-    <sheet name="สรุปรายวัน" sheetId="5" r:id="rId5"/>
+    <sheet name="01_กำหนดการ 8 วัน" sheetId="1" r:id="rId1"/>
+    <sheet name="02_สรุปงบประมาณ" sheetId="2" r:id="rId2"/>
+    <sheet name="03_โรงแรมและเที่ยวบิน" sheetId="3" r:id="rId3"/>
+    <sheet name="04_พิกัด Amap &amp; ภาษาจีน" sheetId="4" r:id="rId4"/>
+    <sheet name="05_ประโยคจีนสื่อสาร" sheetId="5" r:id="rId5"/>
+    <sheet name="06_สรุปส่ง LINE รายวัน" sheetId="6" r:id="rId6"/>
+    <sheet name="07_การเดินทาง 28 เที่ยว" sheetId="7" r:id="rId7"/>
+    <sheet name="08_ตารางหลัก (Master)" sheetId="8" r:id="rId8"/>
+    <sheet name="09_สถิติรายวัน" sheetId="9" r:id="rId9"/>
   </sheets>
 </workbook>
 </file>
@@ -402,6 +406,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L64"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="45.83203125" customWidth="1"/>
+    <col min="5" max="5" width="25.83203125" customWidth="1"/>
+    <col min="6" max="6" width="15.83203125" customWidth="1"/>
+    <col min="7" max="7" width="30.83203125" customWidth="1"/>
+    <col min="8" max="8" width="15.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="15.83203125" customWidth="1"/>
+    <col min="11" max="11" width="15.83203125" customWidth="1"/>
+    <col min="12" max="12" width="25.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2845,6 +2863,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G27"/>
+  <cols>
+    <col min="1" max="1" width="25.83203125" customWidth="1"/>
+    <col min="2" max="2" width="40.83203125" customWidth="1"/>
+    <col min="3" max="3" width="22.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3407,6 +3434,2361 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H12"/>
+  <cols>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="32.83203125" customWidth="1"/>
+    <col min="3" max="3" width="35.83203125" customWidth="1"/>
+    <col min="4" max="4" width="28.83203125" customWidth="1"/>
+    <col min="5" max="5" width="22.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="16.83203125" customWidth="1"/>
+    <col min="8" max="8" width="45.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>ประเภท (Type)</v>
+      </c>
+      <c r="B1" t="str">
+        <v>ชื่อรายการ (Title)</v>
+      </c>
+      <c r="C1" t="str">
+        <v>ชื่อภาษาจีน (中文名称)</v>
+      </c>
+      <c r="D1" t="str">
+        <v>หมายเลขอ้างอิง / Booking Ref</v>
+      </c>
+      <c r="E1" t="str">
+        <v>วัน-เวลา (Date/Time)</v>
+      </c>
+      <c r="F1" t="str">
+        <v>ราคา/คน (บาท)</v>
+      </c>
+      <c r="G1" t="str">
+        <v>รวม 2 คน (บาท)</v>
+      </c>
+      <c r="H1" t="str">
+        <v>รายละเอียด &amp; จุดเด่น (Details &amp; Highlights)</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>โรงแรม (คืนที่ 1)</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Tenghang Hotel (腾航大酒店)</v>
+      </c>
+      <c r="C2" t="str">
+        <v>腾航大酒店（昆明长水国际机场店）</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Trip.com: 1359047990059246</v>
+      </c>
+      <c r="E2" t="str">
+        <v>24–25 ต.ค. 2569 (1 คืน)</v>
+      </c>
+      <c r="F2">
+        <v>249.27</v>
+      </c>
+      <c r="G2">
+        <v>498.53</v>
+      </c>
+      <c r="H2" t="str">
+        <v>ใกล้สนามบินคุนหมิงฉางสุ่ย มีรถตู้รับ-ส่งฟรี 24 ชม. (~10 นาที), ฝากกระเป๋าเดินทางใหญ่ 20 กก. ฟรีระหว่างออกไปเที่ยวในเมือง</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>โรงแรม (คืนที่ 2)</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Longluohe Homestay (龙络河客栈)</v>
+      </c>
+      <c r="C3" t="str">
+        <v>丽江龙落河客栈（三义机场店）</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Trip.com: 1359048036644931</v>
+      </c>
+      <c r="E3" t="str">
+        <v>25–26 ต.ค. 2569 (1 คืน)</v>
+      </c>
+      <c r="F3">
+        <v>193.16</v>
+      </c>
+      <c r="G3">
+        <v>386.32</v>
+      </c>
+      <c r="H3" t="str">
+        <v>ใกล้สนามบินลี่เจียงซานอี้ มีรถรับส่งสนามบินฟรี (รับรอบ 23:45 น. และส่งหน้าอาคารผู้โดยสารเช้า 08:00 น.)</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>โรงแรม (คืนที่ 3)</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Qiyue Linyin Bieyuan (栖悦林隐别院)</v>
+      </c>
+      <c r="C4" t="str">
+        <v>栖悦林隐别院（丽江古城忠义市场店）</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Trip.com: 1359047990153900</v>
+      </c>
+      <c r="E4" t="str">
+        <v>26–27 ต.ค. 2569 (1 คืน)</v>
+      </c>
+      <c r="F4">
+        <v>190.65</v>
+      </c>
+      <c r="G4">
+        <v>381.29</v>
+      </c>
+      <c r="H4" t="str">
+        <v>ตั้งอยู่ในเมืองเก่าลี่เจียง สาขาคฤหาสน์มู่ ใกล้ตลาดจงอี้และประตูใต้ เดินทางสะดวก บรรยากาศเงียบสงบ</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>ที่พัก (คืนที่ 4)</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Summit Inn (虎跳峡山美客栈)</v>
+      </c>
+      <c r="C5" t="str">
+        <v>虎跳峡山美客栈（雅叉村）</v>
+      </c>
+      <c r="D5" t="str">
+        <v>จองตรง / ณ จุดพัก</v>
+      </c>
+      <c r="E5" t="str">
+        <v>27–28 ต.ค. 2569 (1 คืน)</v>
+      </c>
+      <c r="F5">
+        <v>526.39</v>
+      </c>
+      <c r="G5">
+        <v>1052.78</v>
+      </c>
+      <c r="H5" t="str">
+        <v>ที่พักบนเส้นทาง High Trail เสือกระโจน วิวระเบียงหน้าผาอวี้หลง ชมพระอาทิตย์ตกดินสีทองฉาบยอดเขาหิมะและดูดาวเต็มฟ้า</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>โรงแรม (คืนที่ 5-6)</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Shangri-La Wangshan Xiaoyuan Inn (望山小院)</v>
+      </c>
+      <c r="C6" t="str">
+        <v>香格里拉望山小院客栈（独克宗古城店）</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Trip.com: 1359048443168258</v>
+      </c>
+      <c r="E6" t="str">
+        <v>28–30 ต.ค. 2569 (2 คืน)</v>
+      </c>
+      <c r="F6">
+        <v>481.9</v>
+      </c>
+      <c r="G6">
+        <v>963.8</v>
+      </c>
+      <c r="H6" t="str">
+        <v>ตั้งอยู่ในเมืองโบราณตู๋เค่อจง ใกล้วัดกุยซานและกงล้อมนต์ยักษ์ มีเครื่องทำความร้อนพร้อมรับอากาศหนาวเลขตัวเดียว</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>โรงแรม (คืนที่ 7)</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Qiyue Linyin Bieyuan (栖悦林隐别院)</v>
+      </c>
+      <c r="C7" t="str">
+        <v>栖悦林隐别院（丽江古城忠义市场店）</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Trip.com: 1359047990153900</v>
+      </c>
+      <c r="E7" t="str">
+        <v>30–31 ต.ค. 2569 (1 คืน)</v>
+      </c>
+      <c r="F7">
+        <v>190.65</v>
+      </c>
+      <c r="G7">
+        <v>381.29</v>
+      </c>
+      <c r="H7" t="str">
+        <v>พักคืนสุดท้ายในเมืองเก่าลี่เจียง ช้อปปิ้งของฝากและเดินเล่นตลาดโต้รุ่งจงอี้ก่อนบินกลับ</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>เที่ยวบิน ขาไป 1</v>
+      </c>
+      <c r="B8" t="str">
+        <v>China Eastern เที่ยวบิน MU-9614</v>
+      </c>
+      <c r="C8" t="str">
+        <v>中国东方航空 MU-9614</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Trip.com E-Ticket ขาไป</v>
+      </c>
+      <c r="E8" t="str">
+        <v>24 ต.ค. 2569 (20:50 – 00:30+1)</v>
+      </c>
+      <c r="F8" t="str">
+        <v>รวมในแพ็กเกจ</v>
+      </c>
+      <c r="G8" t="str">
+        <v>รวมในแพ็กเกจ</v>
+      </c>
+      <c r="H8" t="str">
+        <v>สุวรรณภูมิ (BKK) → คุนหมิงฉางสุ่ย (KMG) บินตรง 3 ชม. 40 นาที โหลดกระเป๋า 20 กก. (เช็กอินเคาน์เตอร์เท่านั้น)</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>เที่ยวบิน ขาไป 2</v>
+      </c>
+      <c r="B9" t="str">
+        <v>China Eastern เที่ยวบิน MU-5923</v>
+      </c>
+      <c r="C9" t="str">
+        <v>中国东方航空 MU-5923</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Trip.com E-Ticket ขาไป</v>
+      </c>
+      <c r="E9" t="str">
+        <v>25 ต.ค. 2569 (22:45 – 23:45)</v>
+      </c>
+      <c r="F9" t="str">
+        <v>รวมในแพ็กเกจ</v>
+      </c>
+      <c r="G9" t="str">
+        <v>รวมในแพ็กเกจ</v>
+      </c>
+      <c r="H9" t="str">
+        <v>คุนหมิงฉางสุ่ย (KMG) → ลี่เจียงซานอี้ (LJG) บินตรง 1 ชม. ไฟลต์ในประเทศ โหลดกระเป๋า 20 กก.</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>เที่ยวบิน ขากลับ 1</v>
+      </c>
+      <c r="B10" t="str">
+        <v>China Eastern เที่ยวบิน MU-5922</v>
+      </c>
+      <c r="C10" t="str">
+        <v>中国东方航空 MU-5922</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Trip.com E-Ticket ขากลับ</v>
+      </c>
+      <c r="E10" t="str">
+        <v>31 ต.ค. 2569 (10:00 – 11:00)</v>
+      </c>
+      <c r="F10" t="str">
+        <v>รวมในแพ็กเกจ</v>
+      </c>
+      <c r="G10" t="str">
+        <v>รวมในแพ็กเกจ</v>
+      </c>
+      <c r="H10" t="str">
+        <v>ลี่เจียงซานอี้ (LJG) → คุนหมิงฉางสุ่ย (KMG) บินตรง 1 ชม. (แจ้งเจ้าหน้าที่เคาน์เตอร์ทำ Through Check-in ยิงกระเป๋าตรงถึง BKK)</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>เที่ยวบิน ขากลับ 2</v>
+      </c>
+      <c r="B11" t="str">
+        <v>China Eastern เที่ยวบิน MU-9621</v>
+      </c>
+      <c r="C11" t="str">
+        <v>中国东方航空 MU-9621</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Trip.com E-Ticket ขากลับ</v>
+      </c>
+      <c r="E11" t="str">
+        <v>31 ต.ค. 2569 (21:30 – 23:05)</v>
+      </c>
+      <c r="F11" t="str">
+        <v>รวมในแพ็กเกจ</v>
+      </c>
+      <c r="G11" t="str">
+        <v>รวมในแพ็กเกจ</v>
+      </c>
+      <c r="H11" t="str">
+        <v>คุนหมิงฉางสุ่ย (KMG) → สุวรรณภูมิ (BKK) บินตรง 1 ชม. 35 นาที รับกระเป๋าใหญ่ 20 กก. ที่สายพานสุวรรณภูมิ จบทริป</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>รถไฟความเร็วสูง</v>
+      </c>
+      <c r="B12" t="str">
+        <v>รถไฟความเร็วสูง ขบวน C116</v>
+      </c>
+      <c r="C12" t="str">
+        <v>中国高铁 C116 次列车</v>
+      </c>
+      <c r="D12" t="str">
+        <v>12306 / Trip.com</v>
+      </c>
+      <c r="E12" t="str">
+        <v>30 ต.ค. 2569 (14:45 – 16:04)</v>
+      </c>
+      <c r="F12">
+        <v>315</v>
+      </c>
+      <c r="G12">
+        <v>630</v>
+      </c>
+      <c r="H12" t="str">
+        <v>สถานีแชงกรี-ลา (香格里拉站) → สถานีลี่เจียง (丽江站) เดินทาง 1 ชม. 19 นาที (~63 หยวน/คน)</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H12"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F27"/>
+  <cols>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="30.83203125" customWidth="1"/>
+    <col min="3" max="3" width="32.83203125" customWidth="1"/>
+    <col min="4" max="4" width="35.83203125" customWidth="1"/>
+    <col min="5" max="5" width="32.83203125" customWidth="1"/>
+    <col min="6" max="6" width="40.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>หมวดหมู่ (Category)</v>
+      </c>
+      <c r="B1" t="str">
+        <v>ชื่อสถานที่ (ภาษาไทย)</v>
+      </c>
+      <c r="C1" t="str">
+        <v>ชื่อภาษาจีน (中文名称)</v>
+      </c>
+      <c r="D1" t="str">
+        <v>พินอิน (Pinyin)</v>
+      </c>
+      <c r="E1" t="str">
+        <v>ลิงก์ Amap (Navigation Link)</v>
+      </c>
+      <c r="F1" t="str">
+        <v>คำแนะนำ / ข้อควรรู้ (Tips)</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>สนามบิน</v>
+      </c>
+      <c r="B2" t="str">
+        <v>ท่าอากาศยานนานาชาติคุนหมิงฉางสุ่ย</v>
+      </c>
+      <c r="C2" t="str">
+        <v>昆明长水国际机场</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Kūnmíng Chángshuǐ Guójì Jīchǎng</v>
+      </c>
+      <c r="E2" t="str">
+        <v>https://surl.amap.com/20U4Hpku15Tq</v>
+      </c>
+      <c r="F2" t="str">
+        <v>สนามบินหลักของคุนหมิง มี Metro สาย 6 เชื่อมต่อเข้าเมือง</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>สนามบิน</v>
+      </c>
+      <c r="B3" t="str">
+        <v>ท่าอากาศยานลี่เจียงซานอี้</v>
+      </c>
+      <c r="C3" t="str">
+        <v>丽江三义国际机场</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Lìjiāng Sānyì Guójì Jīchǎng</v>
+      </c>
+      <c r="E3" t="str">
+        <v>https://surl.amap.com/2YcW76l49qY</v>
+      </c>
+      <c r="F3" t="str">
+        <v>สนามบินลี่เจียง มีบัสสนามบิน 20 หยวนตรงสู่ประตูใต้เมืองเก่า</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>สถานีรถไฟ</v>
+      </c>
+      <c r="B4" t="str">
+        <v>สถานีรถไฟแชงกรี-ลา</v>
+      </c>
+      <c r="C4" t="str">
+        <v>香格里拉站</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Xiānggélǐlā Zhàn</v>
+      </c>
+      <c r="E4" t="str">
+        <v>https://surl.amap.com/yN182yJoaRv</v>
+      </c>
+      <c r="F4" t="str">
+        <v>สถานีรถไฟความเร็วสูงสายแชงกรี-ลา–ลี่เจียง</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>สถานีรถไฟ</v>
+      </c>
+      <c r="B5" t="str">
+        <v>สถานีรถไฟลี่เจียง</v>
+      </c>
+      <c r="C5" t="str">
+        <v>丽江站</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Lìjiāng Zhàn</v>
+      </c>
+      <c r="E5" t="str">
+        <v>https://surl.amap.com/2Dsj0YlcXfGw</v>
+      </c>
+      <c r="F5" t="str">
+        <v>สถานีรถไฟลี่เจียง มีรถบัสและแท็กซี่เข้าเมืองเก่า</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>สถานีขนส่ง</v>
+      </c>
+      <c r="B6" t="str">
+        <v>สถานีขนส่งผู้โดยสารลี่เจียง</v>
+      </c>
+      <c r="C6" t="str">
+        <v>丽江客运站</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Lìjiāng Kèyùnzhàn</v>
+      </c>
+      <c r="E6" t="str">
+        <v>https://surl.amap.com/2Dsj0YlcXfGw</v>
+      </c>
+      <c r="F6" t="str">
+        <v>จุดขึ้นรถบัสไปสะพานเฉียวโถว (เสือกระโจน) รอบ 08:00 และ 08:30 น.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>โรงแรม</v>
+      </c>
+      <c r="B7" t="str">
+        <v>โรงแรมเถิงหัง (สนามบินคุนหมิง)</v>
+      </c>
+      <c r="C7" t="str">
+        <v>腾航大酒店（昆明长水国际机场店）</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Téngháng Dàjiǔdiàn (Kūnmíng Chángshuǐ Jīchǎng Diàn)</v>
+      </c>
+      <c r="E7" t="str">
+        <v>https://surl.amap.com/20U4Hpku15Tq</v>
+      </c>
+      <c r="F7" t="str">
+        <v>มีรถรับส่งฟรี 24 ชม. โทรแจ้งฟรอนต์เมื่อถึงอาคารผู้โดยสาร</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>โรงแรม</v>
+      </c>
+      <c r="B8" t="str">
+        <v>โฮมสเตย์หลงลั่วเหอ (สนามบินลี่เจียง)</v>
+      </c>
+      <c r="C8" t="str">
+        <v>丽江龙落河客栈（三义机场店）</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Lìjiāng Lóngluòhé Kèzhàn (Sānyì Jīchǎng Diàn)</v>
+      </c>
+      <c r="E8" t="str">
+        <v>https://www.amap.com/search?query=%E4%B8%BD%E6%B1%9F%E9%BE%99%E8%90%BD%E6%B2%B3%E6%B0%91%E5%AE%BF</v>
+      </c>
+      <c r="F8" t="str">
+        <v>ห่างสนามบิน ~5 นาที มีรถรับส่งฟรี</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>โรงแรม</v>
+      </c>
+      <c r="B9" t="str">
+        <v>โรงแรมชีเย่ว์ หลินอิ่น เปี๋ยย่วน (ลี่เจียง)</v>
+      </c>
+      <c r="C9" t="str">
+        <v>栖悦林隐别院（丽江古城忠义市场店）</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Qīyuè Línyǐn Biéyuàn (Lìjiāng Gǔchéng Zhōngyì Shìchǎng Diàn)</v>
+      </c>
+      <c r="E9" t="str">
+        <v>https://surl.amap.com/2Dsj0YlcXfGw</v>
+      </c>
+      <c r="F9" t="str">
+        <v>ใกล้ตลาดจงอี้ ประตูใต้เมืองเก่าลี่เจียง</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>โรงแรม</v>
+      </c>
+      <c r="B10" t="str">
+        <v>ที่พักซัมมิท อินน์ (เสือกระโจน)</v>
+      </c>
+      <c r="C10" t="str">
+        <v>虎跳峡山美客栈（雅叉村）</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Hǔtiàoxiá Shānměi Kèzhàn (Yǎchā Cūn)</v>
+      </c>
+      <c r="E10" t="str">
+        <v>https://surl.amap.com/2H0D91k13mP</v>
+      </c>
+      <c r="F10" t="str">
+        <v>จุดพักค้างคืนบน High Trail ระหว่างทางเทรคกิ้ง</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>โรงแรม</v>
+      </c>
+      <c r="B11" t="str">
+        <v>โรงแรมว่างซาน เสี่ยวหย่วน (แชงกรี-ลา)</v>
+      </c>
+      <c r="C11" t="str">
+        <v>香格里拉望山小院客栈（独克宗古城店）</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Xiānggélǐlā Wàngshān Xiǎoyuàn Kèzhàn</v>
+      </c>
+      <c r="E11" t="str">
+        <v>https://surl.amap.com/2Q0zUvse1n2aI</v>
+      </c>
+      <c r="F11" t="str">
+        <v>ตั้งอยู่ในเมืองโบราณตู๋เค่อจง ใกล้วัดกุยซาน</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>จุดท่องเที่ยว</v>
+      </c>
+      <c r="B12" t="str">
+        <v>สวนสาธารณะชุ่ยหู คุนหมิง</v>
+      </c>
+      <c r="C12" t="str">
+        <v>翠湖公园</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Cuìhú Gōngyuán</v>
+      </c>
+      <c r="E12" t="str">
+        <v>https://surl.amap.com/4r8LFT819c1S</v>
+      </c>
+      <c r="F12" t="str">
+        <v>สวนมรกตใจกลางเมืองคุนหมิง บรรยากาศร่มรื่น เข้าชมฟรี</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>จุดท่องเที่ยว</v>
+      </c>
+      <c r="B13" t="str">
+        <v>ซุ้มประตูม้าทองไก่หยก</v>
+      </c>
+      <c r="C13" t="str">
+        <v>金马碧鸡坊</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Jīnmǎ Bìjī Fāng</v>
+      </c>
+      <c r="E13" t="str">
+        <v>https://surl.amap.com/33RYtbCG73zK</v>
+      </c>
+      <c r="F13" t="str">
+        <v>สัญลักษณ์โบราณใจกลางเมืองคุนหมิง ย่านถนนคนเดินหนานผิง</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>จุดท่องเที่ยว</v>
+      </c>
+      <c r="B14" t="str">
+        <v>ตลาดสดต้ากวนจ้วนซิน</v>
+      </c>
+      <c r="C14" t="str">
+        <v>大观篆新农贸市场</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Dàguān Zhuànxīn Nóngmào Shìchǎng</v>
+      </c>
+      <c r="E14" t="str">
+        <v>https://surl.amap.com/356K2vgmT04T</v>
+      </c>
+      <c r="F14" t="str">
+        <v>ตลาดสดอาหารและสตรีทฟู้ดยูนนานที่ใหญ่และคึกคักที่สุดในคุนหมิง</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>จุดท่องเที่ยว</v>
+      </c>
+      <c r="B15" t="str">
+        <v>สระมังกรดำ (เฮยหลงถาน)</v>
+      </c>
+      <c r="C15" t="str">
+        <v>黑龙潭公园</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Hēilóngtán Gōngyuán</v>
+      </c>
+      <c r="E15" t="str">
+        <v>https://surl.amap.com/2CRjOXV82fSQ</v>
+      </c>
+      <c r="F15" t="str">
+        <v>จุดถ่ายรูปสะพานหินสะท้อนเงายอดเขาหิมะมังกรหยก</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>จุดท่องเที่ยว</v>
+      </c>
+      <c r="B16" t="str">
+        <v>ตลาดโต้รุ่งจงอี้ ลี่เจียง</v>
+      </c>
+      <c r="C16" t="str">
+        <v>忠义市场夜市街</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Zhōngyì Shìchǎng Yèshì Jiē</v>
+      </c>
+      <c r="E16" t="str">
+        <v>https://surl.amap.com/2HSTS4Jc155an</v>
+      </c>
+      <c r="F16" t="str">
+        <v>ตลาดเช้าชาวนาซี และตลาดโต้รุ่งสตรีทฟู้ดปิ้งย่างหม่าล่า</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>จุดท่องเที่ยว</v>
+      </c>
+      <c r="B17" t="str">
+        <v>หุบเขาเสือกระโจน (ด่านจำหน่ายตั๋ว)</v>
+      </c>
+      <c r="C17" t="str">
+        <v>虎跳峡景区售票处</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Hǔtiàoxiá Jǐngqū Shòupiàochù</v>
+      </c>
+      <c r="E17" t="str">
+        <v>https://surl.amap.com/2FfC04n6U3R</v>
+      </c>
+      <c r="F17" t="str">
+        <v>ค่าบัตรผ่านประตู 45 หยวน/คน</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>จุดท่องเที่ยว</v>
+      </c>
+      <c r="B18" t="str">
+        <v>เกสต์เฮาส์น่าซี แฟมิลี่ (เสือกระโจน)</v>
+      </c>
+      <c r="C18" t="str">
+        <v>纳西雅阁客栈</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Nàxī Yǎgé Kèzhàn</v>
+      </c>
+      <c r="E18" t="str">
+        <v>https://surl.amap.com/2P3B73kdfXk</v>
+      </c>
+      <c r="F18" t="str">
+        <v>จุดแวะพักทานมื้อเที่ยงก่อนเริ่มปีน 28 โค้งชัน</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>จุดท่องเที่ยว</v>
+      </c>
+      <c r="B19" t="str">
+        <v>ชาหม่า เกสต์เฮาส์ (Tea Horse)</v>
+      </c>
+      <c r="C19" t="str">
+        <v>虎跳峡茶马客栈</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Hǔtiàoxiá Chámǎ Kèzhàn</v>
+      </c>
+      <c r="E19" t="str">
+        <v>https://surl.amap.com/2GvK08nd26R</v>
+      </c>
+      <c r="F19" t="str">
+        <v>จุดพักดื่มน้ำชมวิวหน้าผาหลังพ้นยอด 28 โค้ง</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>จุดท่องเที่ยว</v>
+      </c>
+      <c r="B20" t="str">
+        <v>ฮาล์ฟเวย์ เกสต์เฮาส์ (Halfway)</v>
+      </c>
+      <c r="C20" t="str">
+        <v>中途客栈</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Zhōngtú Kèzhàn</v>
+      </c>
+      <c r="E20" t="str">
+        <v>https://surl.amap.com/2J7M48k81yN</v>
+      </c>
+      <c r="F20" t="str">
+        <v>ระเบียงชมวิว爽死你阳台 วิวหน้าผาอวี้หลงระดับตำนาน</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>จุดท่องเที่ยว</v>
+      </c>
+      <c r="B21" t="str">
+        <v>ทิน่า เกสต์เฮาส์ (Tina's)</v>
+      </c>
+      <c r="C21" t="str">
+        <v>中峡蒂娜青年旅舍</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Zhōngxiá Dìnà Qīngnián Lǚshè</v>
+      </c>
+      <c r="E21" t="str">
+        <v>https://surl.amap.com/2YcW76l49qY</v>
+      </c>
+      <c r="F21" t="str">
+        <v>จุดรับกระเป๋าใหญ่คืน ทานมื้อเที่ยง และขึ้นรถบัสไปแชงกรี-ลา</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>จุดท่องเที่ยว</v>
+      </c>
+      <c r="B22" t="str">
+        <v>กงล้อมนต์ยักษ์ วัดกุยซาน</v>
+      </c>
+      <c r="C22" t="str">
+        <v>龟山公园·大转经筒</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Guīshān Gōngyuán Dà Zhuànjīngtǒng</v>
+      </c>
+      <c r="E22" t="str">
+        <v>https://surl.amap.com/2Q0zUvse1n2aI</v>
+      </c>
+      <c r="F22" t="str">
+        <v>กงล้อมนต์ทองคำที่ใหญ่ที่สุดในโลก หมุนตามเข็มนาฬิกา 3 รอบเพื่อความเป็นสิริมงคล</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>จุดท่องเที่ยว</v>
+      </c>
+      <c r="B23" t="str">
+        <v>อุทยานแห่งชาติผู่ต๋าชั่ว</v>
+      </c>
+      <c r="C23" t="str">
+        <v>普达措国家公园</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Pǔdácuò Guójiā Gōngyuán</v>
+      </c>
+      <c r="E23" t="str">
+        <v>https://www.amap.com/search?query=%E6%99%AE%E8%BE%BE%E6%8E%AA%E5%9B%BD%E5%AE%B6%E5%85%AC%E5%9B%AD</v>
+      </c>
+      <c r="F23" t="str">
+        <v>ทะเลสาบซู่ตู๋หู ป่าสนอัลไพน์ ค่าเข้า+รถบัส 138 หยวน</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>จุดท่องเที่ยว</v>
+      </c>
+      <c r="B24" t="str">
+        <v>วัดกาด่านซงจ้านหลิน</v>
+      </c>
+      <c r="C24" t="str">
+        <v>噶丹松赞林寺</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Gádān Sōngzànlín Sì</v>
+      </c>
+      <c r="E24" t="str">
+        <v>https://surl.amap.com/fe10g66KcYw</v>
+      </c>
+      <c r="F24" t="str">
+        <v>วัดทิเบตที่ใหญ่ที่สุดในยูนนาน พระราชวังโปตาลาน้อย ค่าเข้า+รถ 90 หยวน</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>ร้านอาหาร</v>
+      </c>
+      <c r="B25" t="str">
+        <v>ร้านเจี้ยนซินหยวน (ก๋วยเตี๋ยวข้ามสะพาน)</v>
+      </c>
+      <c r="C25" t="str">
+        <v>建新园·云南过桥米线(宝善街店)</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Jiànxīnyuán Yúnnán Guòqiáo Mǐxiàn</v>
+      </c>
+      <c r="E25" t="str">
+        <v>https://surl.amap.com/20U4Hpku15Tq</v>
+      </c>
+      <c r="F25" t="str">
+        <v>ร้านก๋วยเตี๋ยวข้ามสะพานระดับตำนานอายุกว่า 100 ปี</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>ร้านอาหาร</v>
+      </c>
+      <c r="B26" t="str">
+        <v>ร้านอาผอฉิง (หม้อไฟซี่โครงหมู ลี่เจียง)</v>
+      </c>
+      <c r="C26" t="str">
+        <v>阿婆情腊排骨(南门总店)</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Āpóqíng Làpáigǔ (Nánmén Zǒngdiàn)</v>
+      </c>
+      <c r="E26" t="str">
+        <v>https://surl.amap.com/2Dsj0YlcXfGw</v>
+      </c>
+      <c r="F26" t="str">
+        <v>หม้อไฟซี่โครงหมูหมักเกลือดั้งเดิม ใกล้สะพานหนานเหมิน</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>ร้านอาหาร</v>
+      </c>
+      <c r="B27" t="str">
+        <v>ร้านอาหารกว่างอี้ คุนหมิง</v>
+      </c>
+      <c r="C27" t="str">
+        <v>广益饭店(北门街)</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Guǎngyì Fàndiàn (Běimén Jiē)</v>
+      </c>
+      <c r="E27" t="str">
+        <v>https://surl.amap.com/4psCbGureAF</v>
+      </c>
+      <c r="F27" t="str">
+        <v>ร้านอาหารพื้นเมืองยูนนาน ใกล้สวนชุ่ยหู</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F27"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E8"/>
+  <cols>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="38.83203125" customWidth="1"/>
+    <col min="3" max="3" width="45.83203125" customWidth="1"/>
+    <col min="4" max="4" width="45.83203125" customWidth="1"/>
+    <col min="5" max="5" width="40.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>สถานการณ์ (Situation)</v>
+      </c>
+      <c r="B1" t="str">
+        <v>ความหมายภาษาไทย (Thai Meaning)</v>
+      </c>
+      <c r="C1" t="str">
+        <v>ประโยคภาษาจีน (中文句子)</v>
+      </c>
+      <c r="D1" t="str">
+        <v>คำอ่านพินอิน (Pinyin)</v>
+      </c>
+      <c r="E1" t="str">
+        <v>คำแนะนำการใช้งาน (Usage Guide)</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>เช็กอินสนามบิน</v>
+      </c>
+      <c r="B2" t="str">
+        <v>ช่วยทำ Through Check-in ยิงกระเป๋าตรงสู่กรุงเทพฯ (BKK) ได้ไหมครับ จะได้ไม่ต้องรับกระเป๋าที่คุนหมิง</v>
+      </c>
+      <c r="C2" t="str">
+        <v>请问可以帮我们办理行李直挂到曼谷（BKK）吗？我们是在昆明中转，谢谢！</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Qǐngwèn kěyǐ bāng wǒmen bànlǐ xínglǐ zhíguà dào Màngǔ (BKK) ma? Wǒmen shì zài Kūnmíng zhōngzhuǎn, xièxiè!</v>
+      </c>
+      <c r="E2" t="str">
+        <v>ยื่นให้เจ้าหน้าที่เคาน์เตอร์ China Eastern ที่สนามบินลี่เจียง (LJG) ในเช้าวันที่ 8 เพื่อยิงกระเป๋าตรงถึงสุวรรณภูมิ</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>ส่งกระเป๋าเดินทางใหญ่</v>
+      </c>
+      <c r="B3" t="str">
+        <v>รบกวนช่วยฝากส่งกระเป๋าเดินทางใบใหญ่นี้ไปรอที่ Tina's Guesthouse ได้ไหมครับ พวกเราจะเดินเทรคกิ้งไปรับที่โน่น</v>
+      </c>
+      <c r="C3" t="str">
+        <v>师傅您好，请问这件大行李可以帮我们托运送到中峡蒂娜客栈（Tina's Guesthouse）吗？我们徒步过去取，谢谢！</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Shīfu nínhǎo, qǐngwèn zhè jiàn dà xínglǐ kěyǐ bāng wǒmen tuōyùn sòng dào Zhōngxiá Dìnà Kèzhàn (Tina's Guesthouse) ma? Wǒmen túbù guòqù qǔ, xièxiè!</v>
+      </c>
+      <c r="E3" t="str">
+        <v>ยื่นให้คนขับรถบัสที่สถานีขนส่งลี่เจียงเช้าวันที่ 4 ก่อนขึ้นรถ (ค่าฝากประมาณ 20 หยวน/ใบ)</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>รถรับ-ส่งโรงแรม</v>
+      </c>
+      <c r="B4" t="str">
+        <v>สวัสดีครับ พวกเราจองห้องพักคืนนี้ไว้ ไม่ทราบว่าตอนนี้มีบริการรถตู้รับฟรีจากสนามบินไปโรงแรมไหมครับ</v>
+      </c>
+      <c r="C4" t="str">
+        <v>您好，我们预订了今晚的房间，请问现在可以安排免费接机服务吗？我们在机场到达厅门口。</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Nínhǎo, wǒmen yùdìng le jīnwǎn de fángjiān, qǐngwèn xiànzài kěyǐ ānpái miǎnfèi jiējī fúwù ma? Wǒmen zài jīchǎng dàodátīng ménkǒu.</v>
+      </c>
+      <c r="E4" t="str">
+        <v>ใช้ติดต่อโรงแรม Tenghang หรือ Longluohe ผ่านแอป Trip.com หรือโทรเมื่อเดินทางถึงสนามบิน</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>ฝากกระเป๋าที่โรงแรม</v>
+      </c>
+      <c r="B5" t="str">
+        <v>สวัสดีครับ พวกเราเช็กเอาต์แล้ว ขออนุญาตฝากกระเป๋าเดินทางใบใหญ่ไว้ที่ฟรอนต์ฟรีได้ไหมครับ เดี๋ยวช่วงค่ำกลับมารับ</v>
+      </c>
+      <c r="C5" t="str">
+        <v>您好，我们已经办理退房，请问可以把大行李免费寄存一下前台吗？我们下午/晚上回来取，谢谢！</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Nínhǎo, wǒmen yǐjīng bànlǐ tuìfáng, qǐngwèn kěyǐ bǎ dà xínglǐ miǎnfèi jìcún yíxià qiántái ma? Wǒmen xiàwǔ/wǎnshang huílái qǔ, xièxiè!</v>
+      </c>
+      <c r="E5" t="str">
+        <v>ยื่นให้พนักงานฟรอนต์โรงแรม Tenghang (วันอาทิตย์ที่ 25 ต.ค.) หรือ Qiyue (วันจันทร์ที่ 26 ต.ค.)</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>ขึ้นรถบัสไปสะพานเฉียวโถว</v>
+      </c>
+      <c r="B6" t="str">
+        <v>ขอสอบถามหน่อยครับ รถบัสที่จะไปสะพานเฉียวโถว (จุดเริ่มเดินเทรคกิ้งหุบเขาเสือกระโจน) ขึ้นที่ชานชาลาไหนครับ</v>
+      </c>
+      <c r="C6" t="str">
+        <v>请问去桥头（虎跳峡徒步起点）的大巴是在哪个检票口上车？</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Qǐngwèn qù Qiáotóu (Hǔtiàoxiá túbù qǐdiǎn) de dàbā shì zài nǎge jiǎnpiàokǒu shàngchē?</v>
+      </c>
+      <c r="E6" t="str">
+        <v>ยื่นให้เจ้าหน้าที่ตรวจตั๋วที่สถานีขนส่งลี่เจียง</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>รับกระเป๋าคืนที่ Tina's</v>
+      </c>
+      <c r="B7" t="str">
+        <v>สวัสดีครับ พวกเรามาติดต่อรับกระเป๋าเดินทางใหญ่ที่ฝากส่งมาจากรถบัสตอนเช้าครับ</v>
+      </c>
+      <c r="C7" t="str">
+        <v>您好，我们来取今天早上从丽江大巴托运过来的大件行李，谢谢！</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Nínhǎo, wǒmen lái qǔ jīntiān zǎoshang cóng Lìjiāng dàbā tuōyùn guòlái de dàjiàn xínglǐ, xièxiè!</v>
+      </c>
+      <c r="E7" t="str">
+        <v>ยื่นให้พนักงานที่เคาน์เตอร์ Tina's Guesthouse / คาเฟ่ Moye บ่ายวันที่ 5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>เรียกรถ DiDi / แท็กซี่</v>
+      </c>
+      <c r="B8" t="str">
+        <v>พี่คนขับครับ รบกวนไปส่งตามพิกัดแผนที่นี้ ขับตามระบบนำทางได้เลยครับ ขอบคุณครับ</v>
+      </c>
+      <c r="C8" t="str">
+        <v>师傅您好，请送我们到这个地方，跟着导航走就可以，谢谢！</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Shīfu nínhǎo, qǐng sòng wǒmen dào zhège dìfang, gēnzhe dǎoháng zǒu jiù kěyǐ, xièxiè!</v>
+      </c>
+      <c r="E8" t="str">
+        <v>ยื่นให้คนขับแท็กซี่หรือ DiDi พร้อมเปิดพิกัด Amap ในโทรศัพท์</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D9"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="70.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>วัน (Day)</v>
+      </c>
+      <c r="B1" t="str">
+        <v>วันที่ (Date)</v>
+      </c>
+      <c r="C1" t="str">
+        <v>หัวข้อแพลนประจำวัน (Title)</v>
+      </c>
+      <c r="D1" t="str">
+        <v>ข้อความสรุปสำหรับส่ง LINE (Formatted Message Text)</v>
+      </c>
+    </row>
+    <row r="2" xml:space="preserve">
+      <c r="A2" t="str">
+        <v>DAY 01</v>
+      </c>
+      <c r="B2" t="str">
+        <v>24 ต.ค. 2569 (ส.)</v>
+      </c>
+      <c r="C2" t="str">
+        <v>กรุงเทพฯ สู่ คุนหมิง</v>
+      </c>
+      <c r="D2" t="str" xml:space="preserve">
+        <v xml:space="preserve">แผนเที่ยววันที่ 1 (24 ต.ค. 2569)
+กรุงเทพฯ สู่ คุนหมิง
+------------------------------
+• 17:50 เช็กอินเคาน์เตอร์ China Eastern สุวรรณภูมิ (BKK)
+• 20:50 บินตรงสู่คุนหมิง (เที่ยวบิน MU-9614)
+• 00:30 ถึงสนามบินคุนหมิงฉางสุ่ย (เวลาจีน)
+------------------------------
+ดูแผนเต็ม: https://yunnan-trip-2026-9g2.pages.dev/</v>
+      </c>
+    </row>
+    <row r="3" xml:space="preserve">
+      <c r="A3" t="str">
+        <v>DAY 02</v>
+      </c>
+      <c r="B3" t="str">
+        <v>25 ต.ค. 2569 (อา.)</v>
+      </c>
+      <c r="C3" t="str">
+        <v>คุนหมิง &amp; บินสู่ลี่เจียง</v>
+      </c>
+      <c r="D3" t="str" xml:space="preserve">
+        <v xml:space="preserve">แผนเที่ยววันที่ 2 (25 ต.ค. 2569)
+คุนหมิง &amp; บินสู่ลี่เจียง
+------------------------------
+• 00:30 ผ่าน ตม. คุนหมิง และรับกระเป๋าใหญ่ 20 กก.
+• 01:30 รถรับส่งสู่ที่พัก Tenghang Hotel พักผ่อนเอาแรง
+• 10:00 เช็กเอาต์ Tenghang Hotel ฝากกระเป๋าเดินทางใหญ่
+• 11:00 นั่ง Metro สาย 6 ชิมก๋วยเตี๋ยวข้ามสะพานร้านเจี้ยนซินหยวน
+• 12:30 ซุ้มประตูกิมหม่าปี้จีฟาง, ถนนคนเดินหนานผิง, เมืองเก่าคุนหมิงเหล่าเจีย
+• 15:00 เดินตลาดสดต้ากวนจ้วนซิน ชิมสตรีทฟู้ดพื้นเมือง
+• 18:30 นั่ง Metro สาย 6 กลับ Tenghang Hotel รับกระเป๋า
+• 20:30 เช็กอินเคาน์เตอร์ China Eastern สนามบินคุนหมิงฉางสุ่ย
+• 22:45 บินตรงสู่ลี่เจียง (เที่ยวบิน MU-5923) ถึง 23:45 น.
+• 23:45 รถรับส่งเข้าพัก Longluohe Homestay
+------------------------------
+ดูแผนเต็ม: https://yunnan-trip-2026-9g2.pages.dev/</v>
+      </c>
+    </row>
+    <row r="4" xml:space="preserve">
+      <c r="A4" t="str">
+        <v>DAY 03</v>
+      </c>
+      <c r="B4" t="str">
+        <v>26 ต.ค. 2569 (จ.)</v>
+      </c>
+      <c r="C4" t="str">
+        <v>เมืองเก่าลี่เจียง &amp; สระมังกรดำ</v>
+      </c>
+      <c r="D4" t="str" xml:space="preserve">
+        <v xml:space="preserve">แผนเที่ยววันที่ 3 (26 ต.ค. 2569)
+เมืองเก่าลี่เจียง &amp; สระมังกรดำ
+------------------------------
+• 08:30 เช็กเอาต์ นั่ง DiDi ยิงตรงสู่ที่พักเมืองเก่าลี่เจียง
+• 11:30 กินหม้อไฟซี่โครงหมูอาผอฉิง &amp; ซื้อตั๋วบัสไปเสือกระโจน
+• 13:45 สระมังกรดำ (ศาลาเต๋อเยวี่ยโหลว, สะพานสั่วชุ่ยเฉียว ชมวิวมังกรหยก)
+• 14:15 เดินไฮไลท์เมืองเก่า: กังหันน้ำใหญ่, จัตุรัสซื่อฟางเจีย, สะพานหินต้าสือเฉียว, หน้าคฤหาสน์ตระกูลมู่
+• 18:30 สตรีทฟู้ดและปิ้งย่างหม่าล่าตลาดโต้รุ่งจงอี้
+• พัก: Qiyue Linyin Bieyuan
+------------------------------
+ดูแผนเต็ม: https://yunnan-trip-2026-9g2.pages.dev/</v>
+      </c>
+    </row>
+    <row r="5" xml:space="preserve">
+      <c r="A5" t="str">
+        <v>DAY 04</v>
+      </c>
+      <c r="B5" t="str">
+        <v>27 ต.ค. 2569 (อ.)</v>
+      </c>
+      <c r="C5" t="str">
+        <v>เทรคกิ้งหุบเขาเสือกระโจน (วันแรก)</v>
+      </c>
+      <c r="D5" t="str" xml:space="preserve">
+        <v xml:space="preserve">แผนเที่ยววันที่ 4 (27 ต.ค. 2569)
+เทรคกิ้งหุบเขาเสือกระโจน (วันแรก)
+------------------------------
+• 07:15 เดินไปสถานีขนส่งลี่เจียง ฝากส่งกระเป๋าใหญ่ 20 กก. ไป Tina's
+• 08:00 รถบัสไปสะพานเฉียวโถว / ด่านจำหน่ายตั๋วเสือกระโจน
+• 10:15 รถตู้ท้องถิ่นไป Naxi Family Guesthouse
+• 11:45 มื้อเที่ยงที่ Naxi Family Guesthouse เติมพลัง
+• 14:00 พิชิต 28 โค้งหักศอก สู่จุดชมวิวสูงสุด 2,670 ม.
+• 16:30 พักดื่มน้ำ Tea Horse Guesthouse
+• 18:00 ถึงที่พัก Summit Inn พักผ่อนชมวิวหน้าผาหุบเขาเสือกระโจน
+• พัก: Summit Inn
+------------------------------
+ดูแผนเต็ม: https://yunnan-trip-2026-9g2.pages.dev/</v>
+      </c>
+    </row>
+    <row r="6" xml:space="preserve">
+      <c r="A6" t="str">
+        <v>DAY 05</v>
+      </c>
+      <c r="B6" t="str">
+        <v>28 ต.ค. 2569 (พ.)</v>
+      </c>
+      <c r="C6" t="str">
+        <v>เสือกระโจน (วันที่สอง) สู่ แชงกรี-ลา</v>
+      </c>
+      <c r="D6" t="str" xml:space="preserve">
+        <v xml:space="preserve">แผนเที่ยววันที่ 5 (28 ต.ค. 2569)
+เสือกระโจน (วันที่สอง) สู่ แชงกรี-ลา
+------------------------------
+• 07:30 กินมื้อเช้าที่ Summit Inn ท่ามกลางอากาศบริสุทธิ์
+• 09:00 เดินเทรคเลียบหน้าผา Halfway Guesthouse → น้ำตกกวนอิม → Tina's Guesthouse
+• 12:30 กินมื้อเที่ยง &amp; รับกระเป๋าใหญ่ที่ Tina's Guesthouse
+• 15:30 รถบัสจาก Tina's มุ่งหน้าเมืองโบราณตู๋เค่อจง แชงกรี-ลา
+• 17:30 เช็กอินที่พัก Shangri-La Wangshan Xiaoyuan Inn
+• 18:15 หมุนกงล้อมนต์ทองคำยักษ์ &amp; ชมวิวไฟกลางคืนวัดกุยซาน
+• 19:45 ดินเนอร์หม้อไฟเนื้อจามรี &amp; ชิมสตรีทฟู้ดเมืองโบราณ
+• พัก: Shangri-La Wangshan Xiaoyuan Inn
+------------------------------
+ดูแผนเต็ม: https://yunnan-trip-2026-9g2.pages.dev/</v>
+      </c>
+    </row>
+    <row r="7" xml:space="preserve">
+      <c r="A7" t="str">
+        <v>DAY 06</v>
+      </c>
+      <c r="B7" t="str">
+        <v>29 ต.ค. 2569 (พฤ.)</v>
+      </c>
+      <c r="C7" t="str">
+        <v>อุทยานแห่งชาติผู่ต๋าชั่ว แชงกรี-ลา</v>
+      </c>
+      <c r="D7" t="str" xml:space="preserve">
+        <v xml:space="preserve">แผนเที่ยววันที่ 6 (29 ต.ค. 2569)
+อุทยานแห่งชาติผู่ต๋าชั่ว แชงกรี-ลา
+------------------------------
+• 07:30 มื้อเช้า เดินไปขึ้นรถบัสประตูตะวันออกตู๋เค่อจง
+• 08:20 นั่งรถบัสสู่อุทยานแห่งชาติผู่ต๋าชั่ว
+• 09:05 ชมทะเลสาบสู่ตูหู เดินเลียบสะพานไม้ธรรมชาติ 3.3 กม.
+• 15:00 นั่งรถบัสกลับเมืองโบราณตู๋เค่อจง
+• 16:00 จิบชาเนยทิเบต คาเฟ่กู่เฉิงเจี่ยวลั่ว
+• 17:30 ปิ้งย่างหินทิเบตร้านหงหง
+• 19:30 เดินเล่นชมไฟเมืองโบราณตู๋เค่อจงยามค่ำคืน
+• พัก: Shangri-La Wangshan Xiaoyuan Inn
+------------------------------
+ดูแผนเต็ม: https://yunnan-trip-2026-9g2.pages.dev/</v>
+      </c>
+    </row>
+    <row r="8" xml:space="preserve">
+      <c r="A8" t="str">
+        <v>DAY 07</v>
+      </c>
+      <c r="B8" t="str">
+        <v>30 ต.ค. 2569 (ศ.)</v>
+      </c>
+      <c r="C8" t="str">
+        <v>วัดซงจ้านหลิน &amp; รถไฟความเร็วสูงสู่ลี่เจียง</v>
+      </c>
+      <c r="D8" t="str" xml:space="preserve">
+        <v xml:space="preserve">แผนเที่ยววันที่ 7 (30 ต.ค. 2569)
+วัดซงจ้านหลิน &amp; รถไฟความเร็วสูงสู่ลี่เจียง
+------------------------------
+• 07:30 เดินเที่ยวตลาดเช้าเซี่ยงหยาง ชิมอาหารพื้นเมือง
+• 09:00 รถเมล์สาย 3 ไปวัดซงจ้านหลิน (พระราชวังโปตาลาน้อย)
+• 13:30 เช็กเอาต์ เดินทางไปสถานีรถไฟความเร็วสูงแชงกรี-ลา
+• 14:45 รถไฟความเร็วสูง C116: แชงกรี-ลา → ลี่เจียง (1 ชม. 19 นาที)
+• 16:15 รถบัสตรงเข้าเมืองเก่าลี่เจียง เช็กอิน Qiyue Linyin Bieyuan
+• 17:00 เดินถ่ายรูปเมืองเก่าลี่เจียง &amp; ถนนสายร่มหลากสี
+• 18:30 ชิมสตรีทฟู้ดตลาดโต้รุ่งจงอี้
+• พัก: Qiyue Linyin Bieyuan
+------------------------------
+ดูแผนเต็ม: https://yunnan-trip-2026-9g2.pages.dev/</v>
+      </c>
+    </row>
+    <row r="9" xml:space="preserve">
+      <c r="A9" t="str">
+        <v>DAY 08</v>
+      </c>
+      <c r="B9" t="str">
+        <v>31 ต.ค. 2569 (ส.)</v>
+      </c>
+      <c r="C9" t="str">
+        <v>ลี่เจียง → คุนหมิง (เที่ยวเมืองเก่า) → กรุงเทพฯ</v>
+      </c>
+      <c r="D9" t="str" xml:space="preserve">
+        <v xml:space="preserve">แผนเที่ยววันที่ 8 (31 ต.ค. 2569)
+ลี่เจียง → คุนหมิง (เที่ยวเมืองเก่า) → กรุงเทพฯ
+------------------------------
+• 06:30 นั่ง DiDi ไปสนามบินลี่เจียงซานอี้ (LJG)
+• 07:30 เช็กอินเคาน์เตอร์ China Eastern (แจ้ง Through Check-in)
+• 10:00 บินตรงสู่คุนหมิง (เที่ยวบิน MU-5922) ถึง 11:00 น.
+• 12:15 นั่ง Metro สาย 6 + 3 เข้าเมืองคุนหมิง
+• 13:30 มื้อเที่ยงร้านกว่างอี้, เดินเล่นสวนสาธารณะชุ่ยหู, พิพิธภัณฑ์ทหารยูนนาน, ถนนคนเดินหนานผิง
+• 17:15 นั่ง Metro สาย 3 + 6 กลับสนามบินคุนหมิงฉางสุ่ย (KMG)
+• 19:00 ผ่าน ตม. ขาออก ตรวจความปลอดภัย รอขึ้นเครื่องที่เกต
+• 21:30 เที่ยวบิน China Eastern MU-9621 บินตรงสู่กรุงเทพฯ
+• 23:05 เดินทางถึงสนามบินสุวรรณภูมิ (BKK) โดยสวัสดิภาพ
+------------------------------
+ดูแผนเต็ม: https://yunnan-trip-2026-9g2.pages.dev/</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D9"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:K30"/>
+  <cols>
+    <col min="1" max="1" width="8.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="28.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" customWidth="1"/>
+    <col min="5" max="5" width="45.83203125" customWidth="1"/>
+    <col min="6" max="6" width="28.83203125" customWidth="1"/>
+    <col min="7" max="7" width="15.83203125" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" customWidth="1"/>
+    <col min="9" max="9" width="15.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="20.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>ลำดับ</v>
+      </c>
+      <c r="B1" t="str">
+        <v>วันที่ (Date)</v>
+      </c>
+      <c r="C1" t="str">
+        <v>ชื่อช่วงการเดินทาง (Name)</v>
+      </c>
+      <c r="D1" t="str">
+        <v>การเดินทาง (Transportation)</v>
+      </c>
+      <c r="E1" t="str">
+        <v>เส้นทาง (Route)</v>
+      </c>
+      <c r="F1" t="str">
+        <v>AMap Link</v>
+      </c>
+      <c r="G1" t="str">
+        <v>ราคา/คน (หยวน)</v>
+      </c>
+      <c r="H1" t="str">
+        <v>ราคา/คน (บาท @ 5.0)</v>
+      </c>
+      <c r="I1" t="str">
+        <v>รวม 2 คน (หยวน)</v>
+      </c>
+      <c r="J1" t="str">
+        <v>รวม 2 คน (บาท @ 5.0)</v>
+      </c>
+      <c r="K1" t="str">
+        <v>หมายเหตุ (Notes)</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>10/25/2026</v>
+      </c>
+      <c r="C2" t="str">
+        <v>สนามบินคุนหมิง-ที่พักคุนหมิง</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Didi</v>
+      </c>
+      <c r="E2" t="str">
+        <v>昆明长水国际机场  腾航大酒店(昆明长水国际机场店)</v>
+      </c>
+      <c r="F2" t="str">
+        <v>-</v>
+      </c>
+      <c r="G2">
+        <v>5</v>
+      </c>
+      <c r="H2">
+        <v>25</v>
+      </c>
+      <c r="I2">
+        <v>10</v>
+      </c>
+      <c r="J2">
+        <v>50</v>
+      </c>
+      <c r="K2" t="str">
+        <v>-</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>10/25/2026</v>
+      </c>
+      <c r="C3" t="str">
+        <v>ที่พักคุนหมิง-ร้านก๋วยเตี๋ยวข้ามสะพาน</v>
+      </c>
+      <c r="D3" t="str">
+        <v>รถไฟ</v>
+      </c>
+      <c r="E3" t="str">
+        <v>腾航大酒店(昆明长水国际机场店) [250001]  建新园·云南过桥米线(宝善街店) [250002]</v>
+      </c>
+      <c r="F3" t="str">
+        <v>https://surl.amap.com/20U4Hpku15Tq</v>
+      </c>
+      <c r="G3">
+        <v>6</v>
+      </c>
+      <c r="H3">
+        <v>30</v>
+      </c>
+      <c r="I3">
+        <v>12</v>
+      </c>
+      <c r="J3">
+        <v>60</v>
+      </c>
+      <c r="K3" t="str">
+        <v>-</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>10/25/2026</v>
+      </c>
+      <c r="C4" t="str">
+        <v>ร้านก๋วยเตี๋ยวข้ามสะพาน-ถนนคนเดินคุนหมิง</v>
+      </c>
+      <c r="D4" t="str">
+        <v>เดิน</v>
+      </c>
+      <c r="E4" t="str">
+        <v>建新园·云南过桥米线(宝善街店) [250101]  金马碧鸡坊 [250102]  南屏步行街 [250103]</v>
+      </c>
+      <c r="F4" t="str">
+        <v>https://surl.amap.com/33RYtbCG73zK</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4" t="str">
+        <v>-</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>10/25/2026</v>
+      </c>
+      <c r="C5" t="str">
+        <v>ถนนคนเดินคุนหมิง-ตลาดคุนหมิง</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Didi</v>
+      </c>
+      <c r="E5" t="str">
+        <v>昆明老街 [250201]  大观篆新农贸市场 [250202]</v>
+      </c>
+      <c r="F5" t="str">
+        <v>-</v>
+      </c>
+      <c r="G5">
+        <v>5</v>
+      </c>
+      <c r="H5">
+        <v>25</v>
+      </c>
+      <c r="I5">
+        <v>10</v>
+      </c>
+      <c r="J5">
+        <v>50</v>
+      </c>
+      <c r="K5" t="str">
+        <v>-</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>10/25/2026</v>
+      </c>
+      <c r="C6" t="str">
+        <v>ตลาดคุนหมิง-ที่พักคุนหมิง</v>
+      </c>
+      <c r="D6" t="str">
+        <v>รถไฟ</v>
+      </c>
+      <c r="E6" t="str">
+        <v>大观篆新农贸市场 [250301]  腾航大酒店(昆明长水国际机场店) [250302]</v>
+      </c>
+      <c r="F6" t="str">
+        <v>https://surl.amap.com/356K2vgmT04T</v>
+      </c>
+      <c r="G6">
+        <v>6</v>
+      </c>
+      <c r="H6">
+        <v>30</v>
+      </c>
+      <c r="I6">
+        <v>12</v>
+      </c>
+      <c r="J6">
+        <v>60</v>
+      </c>
+      <c r="K6" t="str">
+        <v>-</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="str">
+        <v>10/25/2026</v>
+      </c>
+      <c r="C7" t="str">
+        <v>ที่พักคุนหมิง-สนามบินคุนหมิง</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Didi</v>
+      </c>
+      <c r="E7" t="str">
+        <v>腾航大酒店(昆明长水国际机场店)  昆明长水国际机场</v>
+      </c>
+      <c r="F7" t="str">
+        <v>-</v>
+      </c>
+      <c r="G7">
+        <v>5</v>
+      </c>
+      <c r="H7">
+        <v>25</v>
+      </c>
+      <c r="I7">
+        <v>10</v>
+      </c>
+      <c r="J7">
+        <v>50</v>
+      </c>
+      <c r="K7" t="str">
+        <v>-</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="str">
+        <v>10/26/2026</v>
+      </c>
+      <c r="C8" t="str">
+        <v>ที่พักสนามบินลี่เจียง-ที่พักเมืองเก่าลี่เจียง</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Didi</v>
+      </c>
+      <c r="E8" t="str">
+        <v>丽江龙落河民宿(三义国际机场店) [260001]  栖悦林隐别院(丽江古城忠义市场店)</v>
+      </c>
+      <c r="F8" t="str">
+        <v>-</v>
+      </c>
+      <c r="G8">
+        <v>36</v>
+      </c>
+      <c r="H8">
+        <v>180</v>
+      </c>
+      <c r="I8">
+        <v>72</v>
+      </c>
+      <c r="J8">
+        <v>360</v>
+      </c>
+      <c r="K8" t="str">
+        <v>-</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="str">
+        <v>10/26/2026</v>
+      </c>
+      <c r="C9" t="str">
+        <v>ที่พักเมืองเก่าลี่เจียง-สถานีขนส่งลี่เจียง</v>
+      </c>
+      <c r="D9" t="str">
+        <v>เดิน</v>
+      </c>
+      <c r="E9" t="str">
+        <v>栖悦林隐别院(丽江古城忠义市场店) [260101]  阿婆情腊排骨火锅·野生菌季(忠义店) [260102]  丽江客运站 [260103]</v>
+      </c>
+      <c r="F9" t="str">
+        <v>https://surl.amap.com/2Dsj0YlcXfGw</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
+      <c r="K9" t="str">
+        <v>-</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="str">
+        <v>10/26/2026</v>
+      </c>
+      <c r="C10" t="str">
+        <v>สถานีขนส่งลี่เจียง-สระมังกรดำ</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Didi</v>
+      </c>
+      <c r="E10" t="str">
+        <v>丽江客运站 [260201]  得月楼 [260202]</v>
+      </c>
+      <c r="F10" t="str">
+        <v>-</v>
+      </c>
+      <c r="G10">
+        <v>6.5</v>
+      </c>
+      <c r="H10">
+        <v>32.5</v>
+      </c>
+      <c r="I10">
+        <v>13</v>
+      </c>
+      <c r="J10">
+        <v>65</v>
+      </c>
+      <c r="K10" t="str">
+        <v>-</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>10/26/2026</v>
+      </c>
+      <c r="C11" t="str">
+        <v>เดินสระมังกรดำ-เมืองเก่าลี้เจียง-ที่พักเมืองเก่าลี่เจียง</v>
+      </c>
+      <c r="D11" t="str">
+        <v>เดิน</v>
+      </c>
+      <c r="E11" t="str">
+        <v>黑龙潭公园-得月楼 [260301]  锁翠桥 [260302]  丽江古城-古城大水车 [260303]  四方街 [260304]  大石桥 [260305]  丽江古城博物院-木府 [260306]  栖悦林隐别院(丽江古城忠义市场店) [260307]</v>
+      </c>
+      <c r="F11" t="str">
+        <v>https://surl.amap.com/2CRjOXV82fSQ</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="K11" t="str">
+        <v>ชมสถาปัตยกรรมด้านนอก / ฟรี</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>10/26/2026</v>
+      </c>
+      <c r="C12" t="str">
+        <v>ที่พักเมืองเก่าลี่เจียง-ตลาดจงอี้</v>
+      </c>
+      <c r="D12" t="str">
+        <v>เดิน</v>
+      </c>
+      <c r="E12" t="str">
+        <v>栖悦林隐别院(丽江古城忠义市场店) [260401]  忠义市场夜市街 [260402]</v>
+      </c>
+      <c r="F12" t="str">
+        <v>https://surl.amap.com/2HSTS4Jc155an</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
+      <c r="K12" t="str">
+        <v>-</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>10/27/2026</v>
+      </c>
+      <c r="C13" t="str">
+        <v>เมืองเก่าลี่เจียง-หุบเขาเสือกระโจน</v>
+      </c>
+      <c r="D13" t="str">
+        <v>รถบัส</v>
+      </c>
+      <c r="E13" t="str">
+        <v>丽江客运站  纳西雅阁客栈</v>
+      </c>
+      <c r="F13" t="str">
+        <v>-</v>
+      </c>
+      <c r="G13">
+        <v>35</v>
+      </c>
+      <c r="H13">
+        <v>175</v>
+      </c>
+      <c r="I13">
+        <v>70</v>
+      </c>
+      <c r="J13">
+        <v>350</v>
+      </c>
+      <c r="K13" t="str">
+        <v>-</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>10/27/2026</v>
+      </c>
+      <c r="C14" t="str">
+        <v>เทรคกิ้ง 28 โค้ง</v>
+      </c>
+      <c r="D14" t="str">
+        <v>เดิน</v>
+      </c>
+      <c r="E14" t="str">
+        <v>纳西雅阁客栈  香格里拉山美客栈(东环线分店)</v>
+      </c>
+      <c r="F14" t="str">
+        <v>-</v>
+      </c>
+      <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14">
+        <v>0</v>
+      </c>
+      <c r="I14">
+        <v>0</v>
+      </c>
+      <c r="J14">
+        <v>0</v>
+      </c>
+      <c r="K14" t="str">
+        <v>-</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="str">
+        <v>10/28/2026</v>
+      </c>
+      <c r="C15" t="str">
+        <v>เทรคกิ้งเสือกระโจน วันสอง</v>
+      </c>
+      <c r="D15" t="str">
+        <v>เดิน</v>
+      </c>
+      <c r="E15" t="str">
+        <v>香格里拉山美客栈(东环线分店)  中峡国际青年旅舍Tina'S Guest House</v>
+      </c>
+      <c r="F15" t="str">
+        <v>-</v>
+      </c>
+      <c r="G15">
+        <v>0</v>
+      </c>
+      <c r="H15">
+        <v>0</v>
+      </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+      <c r="J15">
+        <v>0</v>
+      </c>
+      <c r="K15" t="str">
+        <v>-</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="str">
+        <v>10/28/2026</v>
+      </c>
+      <c r="C16" t="str">
+        <v>เมืองโบราณตู๋เค่อจง-ที่พักแชงกีลา</v>
+      </c>
+      <c r="D16" t="str">
+        <v>เดิน</v>
+      </c>
+      <c r="E16" t="str">
+        <v>香格里拉市独克宗古城(北门) [280101]  香格里拉望山小院客栈(独克宗古城店) [280102]  静静的嘛呢石藏餐吧(北门店) [280103]  龟山公园 [280104]</v>
+      </c>
+      <c r="F16" t="str">
+        <v>https://surl.amap.com/2Q0zUvse1n2aI</v>
+      </c>
+      <c r="G16">
+        <v>0</v>
+      </c>
+      <c r="H16">
+        <v>0</v>
+      </c>
+      <c r="I16">
+        <v>0</v>
+      </c>
+      <c r="J16">
+        <v>0</v>
+      </c>
+      <c r="K16" t="str">
+        <v>-</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="str">
+        <v>10/29/2026</v>
+      </c>
+      <c r="C17" t="str">
+        <v>ที่พักแชงกีลา-อุทยานผู่ต๋าชั่ว</v>
+      </c>
+      <c r="D17" t="str">
+        <v>รถบัส</v>
+      </c>
+      <c r="E17" t="str">
+        <v>香格里拉独克宗古城东门客运站售票点  普达措国家公园入口游客中心</v>
+      </c>
+      <c r="F17" t="str">
+        <v>-</v>
+      </c>
+      <c r="G17">
+        <v>178</v>
+      </c>
+      <c r="H17">
+        <v>890</v>
+      </c>
+      <c r="I17">
+        <v>356</v>
+      </c>
+      <c r="J17">
+        <v>1780</v>
+      </c>
+      <c r="K17" t="str">
+        <v>ไป 8.20-9.05</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="str">
+        <v>10/29/2026</v>
+      </c>
+      <c r="C18" t="str">
+        <v>อุทยานผู่ต๋าชั่ว-ที่พักแชงกีลา</v>
+      </c>
+      <c r="D18" t="str">
+        <v>รถบัส</v>
+      </c>
+      <c r="E18" t="str">
+        <v>普达措国家公园入口游客中心  香格里拉独克宗古城东门客运站售票点</v>
+      </c>
+      <c r="F18" t="str">
+        <v>-</v>
+      </c>
+      <c r="G18">
+        <v>0</v>
+      </c>
+      <c r="H18">
+        <v>0</v>
+      </c>
+      <c r="I18">
+        <v>0</v>
+      </c>
+      <c r="J18">
+        <v>0</v>
+      </c>
+      <c r="K18" t="str">
+        <v>กลับ 15.00-15.45</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="str">
+        <v>10/29/2026</v>
+      </c>
+      <c r="C19" t="str">
+        <v>ที่พักแชงกีลา-คาเฟ่-ร้านอาหาร</v>
+      </c>
+      <c r="D19" t="str">
+        <v>เดิน</v>
+      </c>
+      <c r="E19" t="str">
+        <v>香格里拉望山小院客栈(独克宗古城店)  古城角落甜茶馆  宏宏无烟石板烧烤</v>
+      </c>
+      <c r="F19" t="str">
+        <v>https://surl.amap.com/3aWWUho1o6Qb</v>
+      </c>
+      <c r="G19">
+        <v>0</v>
+      </c>
+      <c r="H19">
+        <v>0</v>
+      </c>
+      <c r="I19">
+        <v>0</v>
+      </c>
+      <c r="J19">
+        <v>0</v>
+      </c>
+      <c r="K19" t="str">
+        <v>-</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="str">
+        <v>10/30/2026</v>
+      </c>
+      <c r="C20" t="str">
+        <v>ที่พักแชงกีลา-ตลาด</v>
+      </c>
+      <c r="D20" t="str">
+        <v>เดิน</v>
+      </c>
+      <c r="E20" t="str">
+        <v>香格里拉望山小院客栈(独克宗古城店)  金桥向阳菜市场(向阳路农贸综合市场店)</v>
+      </c>
+      <c r="F20" t="str">
+        <v>https://surl.amap.com/37LSs3sS8SI</v>
+      </c>
+      <c r="G20">
+        <v>0</v>
+      </c>
+      <c r="H20">
+        <v>0</v>
+      </c>
+      <c r="I20">
+        <v>0</v>
+      </c>
+      <c r="J20">
+        <v>0</v>
+      </c>
+      <c r="K20" t="str">
+        <v>-</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="str">
+        <v>10/30/2026</v>
+      </c>
+      <c r="C21" t="str">
+        <v>ตลาด-วัดซงจ้านหลิน</v>
+      </c>
+      <c r="D21" t="str">
+        <v>รถบัส</v>
+      </c>
+      <c r="E21" t="str">
+        <v>金桥向阳菜市场(向阳路农贸综合市场店)  噶丹松赞林寺  游客服务中心 (กินข้าว)</v>
+      </c>
+      <c r="F21" t="str">
+        <v>https://surl.amap.com/fe10g66KcYw</v>
+      </c>
+      <c r="G21">
+        <v>2</v>
+      </c>
+      <c r="H21">
+        <v>10</v>
+      </c>
+      <c r="I21">
+        <v>4</v>
+      </c>
+      <c r="J21">
+        <v>20</v>
+      </c>
+      <c r="K21" t="str">
+        <v>กินข้าวที่游客服务中心</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="str">
+        <v>10/30/2026</v>
+      </c>
+      <c r="C22" t="str">
+        <v>วัดซงจ้านหลิน-ที่พักแชงกีลา</v>
+      </c>
+      <c r="D22" t="str">
+        <v>รถบัส</v>
+      </c>
+      <c r="E22" t="str">
+        <v>噶丹松赞林寺  香格里拉望山小院客栈(独克宗古城店)</v>
+      </c>
+      <c r="F22" t="str">
+        <v>https://surl.amap.com/2RRM1kq6aIj</v>
+      </c>
+      <c r="G22">
+        <v>2</v>
+      </c>
+      <c r="H22">
+        <v>10</v>
+      </c>
+      <c r="I22">
+        <v>4</v>
+      </c>
+      <c r="J22">
+        <v>20</v>
+      </c>
+      <c r="K22" t="str">
+        <v>-</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="str">
+        <v>10/30/2026</v>
+      </c>
+      <c r="C23" t="str">
+        <v>ที่พักแชงกีลา-สถานีแชงกีลา</v>
+      </c>
+      <c r="D23" t="str">
+        <v>รถบัส</v>
+      </c>
+      <c r="E23" t="str">
+        <v>香格里拉望山小院客栈(独克宗古城店)  香格里拉站(进站口)</v>
+      </c>
+      <c r="F23" t="str">
+        <v>https://surl.amap.com/yN182yJoaRv</v>
+      </c>
+      <c r="G23">
+        <v>2</v>
+      </c>
+      <c r="H23">
+        <v>10</v>
+      </c>
+      <c r="I23">
+        <v>4</v>
+      </c>
+      <c r="J23">
+        <v>20</v>
+      </c>
+      <c r="K23" t="str">
+        <v>-</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="str">
+        <v>10/30/2026</v>
+      </c>
+      <c r="C24" t="str">
+        <v>สถานีลี่เจียง-ที่พักเมืองเก่าลี่เจียง</v>
+      </c>
+      <c r="D24" t="str">
+        <v>รถบัส</v>
+      </c>
+      <c r="E24" t="str">
+        <v>丽江站  栖悦林隐别院(丽江古城忠义市场店)</v>
+      </c>
+      <c r="F24" t="str">
+        <v>https://surl.amap.com/3n4lXMyfeuQ</v>
+      </c>
+      <c r="G24">
+        <v>5</v>
+      </c>
+      <c r="H24">
+        <v>25</v>
+      </c>
+      <c r="I24">
+        <v>10</v>
+      </c>
+      <c r="J24">
+        <v>50</v>
+      </c>
+      <c r="K24" t="str">
+        <v>-</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="str">
+        <v>10/30/2026</v>
+      </c>
+      <c r="C25" t="str">
+        <v>ที่พักเมืองเก่าลี่เจียง-ตลาดจงอี้</v>
+      </c>
+      <c r="D25" t="str">
+        <v>เดิน</v>
+      </c>
+      <c r="E25" t="str">
+        <v>栖悦林隐别院(丽江古城忠义市场店)  忠义市场夜市街</v>
+      </c>
+      <c r="F25" t="str">
+        <v>https://surl.amap.com/2HSTS4Jc155an</v>
+      </c>
+      <c r="G25">
+        <v>0</v>
+      </c>
+      <c r="H25">
+        <v>0</v>
+      </c>
+      <c r="I25">
+        <v>0</v>
+      </c>
+      <c r="J25">
+        <v>0</v>
+      </c>
+      <c r="K25" t="str">
+        <v>-</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="str">
+        <v>10/31/2026</v>
+      </c>
+      <c r="C26" t="str">
+        <v>ที่พักเมืองเก่าลี่เจียง-สนามบินลี่เจียง</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Didi</v>
+      </c>
+      <c r="E26" t="str">
+        <v>栖悦林隐别院(丽江古城忠义市场店) [260001]  丽江龙落河民宿(三义国际机场店)</v>
+      </c>
+      <c r="F26" t="str">
+        <v>-</v>
+      </c>
+      <c r="G26">
+        <v>36</v>
+      </c>
+      <c r="H26">
+        <v>180</v>
+      </c>
+      <c r="I26">
+        <v>72</v>
+      </c>
+      <c r="J26">
+        <v>360</v>
+      </c>
+      <c r="K26" t="str">
+        <v>-</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="str">
+        <v>10/31/2026</v>
+      </c>
+      <c r="C27" t="str">
+        <v>สนามบินคุณหมิง-ร้านอาหาร</v>
+      </c>
+      <c r="D27" t="str">
+        <v>รถไฟ</v>
+      </c>
+      <c r="E27" t="str">
+        <v>昆明长水国际机场  广益饭店(北门街)</v>
+      </c>
+      <c r="F27" t="str">
+        <v>https://surl.amap.com/4psCbGureAF</v>
+      </c>
+      <c r="G27">
+        <v>6</v>
+      </c>
+      <c r="H27">
+        <v>30</v>
+      </c>
+      <c r="I27">
+        <v>12</v>
+      </c>
+      <c r="J27">
+        <v>60</v>
+      </c>
+      <c r="K27" t="str">
+        <v>-</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="str">
+        <v>10/31/2026</v>
+      </c>
+      <c r="C28" t="str">
+        <v>ร้านอาหาร-สวนสาธารณะ</v>
+      </c>
+      <c r="D28" t="str">
+        <v>เดิน</v>
+      </c>
+      <c r="E28" t="str">
+        <v>广益饭店(北门街)  翠湖公园  云南陆军讲武堂历史博物馆  南屏步行街</v>
+      </c>
+      <c r="F28" t="str">
+        <v>https://surl.amap.com/4r8LFT819c1S</v>
+      </c>
+      <c r="G28">
+        <v>0</v>
+      </c>
+      <c r="H28">
+        <v>0</v>
+      </c>
+      <c r="I28">
+        <v>0</v>
+      </c>
+      <c r="J28">
+        <v>0</v>
+      </c>
+      <c r="K28" t="str">
+        <v>-</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="str">
+        <v>10/31/2026</v>
+      </c>
+      <c r="C29" t="str">
+        <v>ถนนคนเดิน-สนามบินคุณหมิง</v>
+      </c>
+      <c r="D29" t="str">
+        <v>รถไฟ</v>
+      </c>
+      <c r="E29" t="str">
+        <v>南屏步行街  昆明长水国际机场</v>
+      </c>
+      <c r="F29" t="str">
+        <v>https://surl.amap.com/tP208A1cceK</v>
+      </c>
+      <c r="G29">
+        <v>6</v>
+      </c>
+      <c r="H29">
+        <v>30</v>
+      </c>
+      <c r="I29">
+        <v>12</v>
+      </c>
+      <c r="J29">
+        <v>60</v>
+      </c>
+      <c r="K29" t="str">
+        <v>-</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v/>
+      </c>
+      <c r="B30" t="str">
+        <v>รวมทั้งหมด (คณะ 2 คน)</v>
+      </c>
+      <c r="C30" t="str">
+        <v/>
+      </c>
+      <c r="D30" t="str">
+        <v/>
+      </c>
+      <c r="E30" t="str">
+        <v/>
+      </c>
+      <c r="F30" t="str">
+        <v/>
+      </c>
+      <c r="G30">
+        <v>391.5</v>
+      </c>
+      <c r="H30">
+        <v>1957.5</v>
+      </c>
+      <c r="I30">
+        <v>783</v>
+      </c>
+      <c r="J30">
+        <v>3915</v>
+      </c>
+      <c r="K30" t="str">
+        <v>ยอดรวม 2 คน = ¥783.00 (฿3,915.00) | เฉลี่ยคนละ ¥391.50 (฿1,957.50)</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:K30"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K71"/>
   <sheetData>
     <row r="1">
@@ -5901,1068 +8283,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K30"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>ลำดับ</v>
-      </c>
-      <c r="B1" t="str">
-        <v>วันที่ (Date)</v>
-      </c>
-      <c r="C1" t="str">
-        <v>ชื่อช่วงการเดินทาง (Name)</v>
-      </c>
-      <c r="D1" t="str">
-        <v>การเดินทาง (Transportation)</v>
-      </c>
-      <c r="E1" t="str">
-        <v>เส้นทาง (Route)</v>
-      </c>
-      <c r="F1" t="str">
-        <v>AMap Link</v>
-      </c>
-      <c r="G1" t="str">
-        <v>ราคา/คน (หยวน)</v>
-      </c>
-      <c r="H1" t="str">
-        <v>ราคา/คน (บาท @ 5.0)</v>
-      </c>
-      <c r="I1" t="str">
-        <v>รวม 2 คน (หยวน)</v>
-      </c>
-      <c r="J1" t="str">
-        <v>รวม 2 คน (บาท @ 5.0)</v>
-      </c>
-      <c r="K1" t="str">
-        <v>หมายเหตุ (Notes)</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="str">
-        <v>10/25/2026</v>
-      </c>
-      <c r="C2" t="str">
-        <v>สนามบินคุนหมิง-ที่พักคุนหมิง</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Didi</v>
-      </c>
-      <c r="E2" t="str">
-        <v>昆明长水国际机场  腾航大酒店(昆明长水国际机场店)</v>
-      </c>
-      <c r="F2" t="str">
-        <v>-</v>
-      </c>
-      <c r="G2">
-        <v>5</v>
-      </c>
-      <c r="H2">
-        <v>25</v>
-      </c>
-      <c r="I2">
-        <v>10</v>
-      </c>
-      <c r="J2">
-        <v>50</v>
-      </c>
-      <c r="K2" t="str">
-        <v>-</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="str">
-        <v>10/25/2026</v>
-      </c>
-      <c r="C3" t="str">
-        <v>ที่พักคุนหมิง-ร้านก๋วยเตี๋ยวข้ามสะพาน</v>
-      </c>
-      <c r="D3" t="str">
-        <v>รถไฟ</v>
-      </c>
-      <c r="E3" t="str">
-        <v>腾航大酒店(昆明长水国际机场店) [250001]  建新园·云南过桥米线(宝善街店) [250002]</v>
-      </c>
-      <c r="F3" t="str">
-        <v>https://surl.amap.com/20U4Hpku15Tq</v>
-      </c>
-      <c r="G3">
-        <v>6</v>
-      </c>
-      <c r="H3">
-        <v>30</v>
-      </c>
-      <c r="I3">
-        <v>12</v>
-      </c>
-      <c r="J3">
-        <v>60</v>
-      </c>
-      <c r="K3" t="str">
-        <v>-</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="str">
-        <v>10/25/2026</v>
-      </c>
-      <c r="C4" t="str">
-        <v>ร้านก๋วยเตี๋ยวข้ามสะพาน-ถนนคนเดินคุนหมิง</v>
-      </c>
-      <c r="D4" t="str">
-        <v>เดิน</v>
-      </c>
-      <c r="E4" t="str">
-        <v>建新园·云南过桥米线(宝善街店) [250101]  金马碧鸡坊 [250102]  南屏步行街 [250103]</v>
-      </c>
-      <c r="F4" t="str">
-        <v>https://surl.amap.com/33RYtbCG73zK</v>
-      </c>
-      <c r="G4">
-        <v>0</v>
-      </c>
-      <c r="H4">
-        <v>0</v>
-      </c>
-      <c r="I4">
-        <v>0</v>
-      </c>
-      <c r="J4">
-        <v>0</v>
-      </c>
-      <c r="K4" t="str">
-        <v>-</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" t="str">
-        <v>10/25/2026</v>
-      </c>
-      <c r="C5" t="str">
-        <v>ถนนคนเดินคุนหมิง-ตลาดคุนหมิง</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Didi</v>
-      </c>
-      <c r="E5" t="str">
-        <v>昆明老街 [250201]  大观篆新农贸市场 [250202]</v>
-      </c>
-      <c r="F5" t="str">
-        <v>-</v>
-      </c>
-      <c r="G5">
-        <v>5</v>
-      </c>
-      <c r="H5">
-        <v>25</v>
-      </c>
-      <c r="I5">
-        <v>10</v>
-      </c>
-      <c r="J5">
-        <v>50</v>
-      </c>
-      <c r="K5" t="str">
-        <v>-</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" t="str">
-        <v>10/25/2026</v>
-      </c>
-      <c r="C6" t="str">
-        <v>ตลาดคุนหมิง-ที่พักคุนหมิง</v>
-      </c>
-      <c r="D6" t="str">
-        <v>รถไฟ</v>
-      </c>
-      <c r="E6" t="str">
-        <v>大观篆新农贸市场 [250301]  腾航大酒店(昆明长水国际机场店) [250302]</v>
-      </c>
-      <c r="F6" t="str">
-        <v>https://surl.amap.com/356K2vgmT04T</v>
-      </c>
-      <c r="G6">
-        <v>6</v>
-      </c>
-      <c r="H6">
-        <v>30</v>
-      </c>
-      <c r="I6">
-        <v>12</v>
-      </c>
-      <c r="J6">
-        <v>60</v>
-      </c>
-      <c r="K6" t="str">
-        <v>-</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" t="str">
-        <v>10/25/2026</v>
-      </c>
-      <c r="C7" t="str">
-        <v>ที่พักคุนหมิง-สนามบินคุนหมิง</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Didi</v>
-      </c>
-      <c r="E7" t="str">
-        <v>腾航大酒店(昆明长水国际机场店)  昆明长水国际机场</v>
-      </c>
-      <c r="F7" t="str">
-        <v>-</v>
-      </c>
-      <c r="G7">
-        <v>5</v>
-      </c>
-      <c r="H7">
-        <v>25</v>
-      </c>
-      <c r="I7">
-        <v>10</v>
-      </c>
-      <c r="J7">
-        <v>50</v>
-      </c>
-      <c r="K7" t="str">
-        <v>-</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="str">
-        <v>10/26/2026</v>
-      </c>
-      <c r="C8" t="str">
-        <v>ที่พักสนามบินลี่เจียง-ที่พักเมืองเก่าลี่เจียง</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Didi</v>
-      </c>
-      <c r="E8" t="str">
-        <v>丽江龙落河民宿(三义国际机场店) [260001]  栖悦林隐别院(丽江古城忠义市场店)</v>
-      </c>
-      <c r="F8" t="str">
-        <v>-</v>
-      </c>
-      <c r="G8">
-        <v>36</v>
-      </c>
-      <c r="H8">
-        <v>180</v>
-      </c>
-      <c r="I8">
-        <v>72</v>
-      </c>
-      <c r="J8">
-        <v>360</v>
-      </c>
-      <c r="K8" t="str">
-        <v>-</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" t="str">
-        <v>10/26/2026</v>
-      </c>
-      <c r="C9" t="str">
-        <v>ที่พักเมืองเก่าลี่เจียง-สถานีขนส่งลี่เจียง</v>
-      </c>
-      <c r="D9" t="str">
-        <v>เดิน</v>
-      </c>
-      <c r="E9" t="str">
-        <v>栖悦林隐别院(丽江古城忠义市场店) [260101]  阿婆情腊排骨火锅·野生菌季(忠义店) [260102]  丽江客运站 [260103]</v>
-      </c>
-      <c r="F9" t="str">
-        <v>https://surl.amap.com/2Dsj0YlcXfGw</v>
-      </c>
-      <c r="G9">
-        <v>0</v>
-      </c>
-      <c r="H9">
-        <v>0</v>
-      </c>
-      <c r="I9">
-        <v>0</v>
-      </c>
-      <c r="J9">
-        <v>0</v>
-      </c>
-      <c r="K9" t="str">
-        <v>-</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" t="str">
-        <v>10/26/2026</v>
-      </c>
-      <c r="C10" t="str">
-        <v>สถานีขนส่งลี่เจียง-สระมังกรดำ</v>
-      </c>
-      <c r="D10" t="str">
-        <v>Didi</v>
-      </c>
-      <c r="E10" t="str">
-        <v>丽江客运站 [260201]  得月楼 [260202]</v>
-      </c>
-      <c r="F10" t="str">
-        <v>-</v>
-      </c>
-      <c r="G10">
-        <v>6.5</v>
-      </c>
-      <c r="H10">
-        <v>32.5</v>
-      </c>
-      <c r="I10">
-        <v>13</v>
-      </c>
-      <c r="J10">
-        <v>65</v>
-      </c>
-      <c r="K10" t="str">
-        <v>-</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" t="str">
-        <v>10/26/2026</v>
-      </c>
-      <c r="C11" t="str">
-        <v>เดินสระมังกรดำ-เมืองเก่าลี้เจียง-ที่พักเมืองเก่าลี่เจียง</v>
-      </c>
-      <c r="D11" t="str">
-        <v>เดิน</v>
-      </c>
-      <c r="E11" t="str">
-        <v>黑龙潭公园-得月楼 [260301]  锁翠桥 [260302]  丽江古城-古城大水车 [260303]  四方街 [260304]  大石桥 [260305]  丽江古城博物院-木府 [260306]  栖悦林隐别院(丽江古城忠义市场店) [260307]</v>
-      </c>
-      <c r="F11" t="str">
-        <v>https://surl.amap.com/2CRjOXV82fSQ</v>
-      </c>
-      <c r="G11">
-        <v>0</v>
-      </c>
-      <c r="H11">
-        <v>0</v>
-      </c>
-      <c r="I11">
-        <v>0</v>
-      </c>
-      <c r="J11">
-        <v>0</v>
-      </c>
-      <c r="K11" t="str">
-        <v>ชมสถาปัตยกรรมด้านนอก / ฟรี</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12" t="str">
-        <v>10/26/2026</v>
-      </c>
-      <c r="C12" t="str">
-        <v>ที่พักเมืองเก่าลี่เจียง-ตลาดจงอี้</v>
-      </c>
-      <c r="D12" t="str">
-        <v>เดิน</v>
-      </c>
-      <c r="E12" t="str">
-        <v>栖悦林隐别院(丽江古城忠义市场店) [260401]  忠义市场夜市街 [260402]</v>
-      </c>
-      <c r="F12" t="str">
-        <v>https://surl.amap.com/2HSTS4Jc155an</v>
-      </c>
-      <c r="G12">
-        <v>0</v>
-      </c>
-      <c r="H12">
-        <v>0</v>
-      </c>
-      <c r="I12">
-        <v>0</v>
-      </c>
-      <c r="J12">
-        <v>0</v>
-      </c>
-      <c r="K12" t="str">
-        <v>-</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13" t="str">
-        <v>10/27/2026</v>
-      </c>
-      <c r="C13" t="str">
-        <v>เมืองเก่าลี่เจียง-หุบเขาเสือกระโจน</v>
-      </c>
-      <c r="D13" t="str">
-        <v>รถบัส</v>
-      </c>
-      <c r="E13" t="str">
-        <v>丽江客运站  纳西雅阁客栈</v>
-      </c>
-      <c r="F13" t="str">
-        <v>-</v>
-      </c>
-      <c r="G13">
-        <v>35</v>
-      </c>
-      <c r="H13">
-        <v>175</v>
-      </c>
-      <c r="I13">
-        <v>70</v>
-      </c>
-      <c r="J13">
-        <v>350</v>
-      </c>
-      <c r="K13" t="str">
-        <v>-</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14" t="str">
-        <v>10/27/2026</v>
-      </c>
-      <c r="C14" t="str">
-        <v>เทรคกิ้ง 28 โค้ง</v>
-      </c>
-      <c r="D14" t="str">
-        <v>เดิน</v>
-      </c>
-      <c r="E14" t="str">
-        <v>纳西雅阁客栈  香格里拉山美客栈(东环线分店)</v>
-      </c>
-      <c r="F14" t="str">
-        <v>-</v>
-      </c>
-      <c r="G14">
-        <v>0</v>
-      </c>
-      <c r="H14">
-        <v>0</v>
-      </c>
-      <c r="I14">
-        <v>0</v>
-      </c>
-      <c r="J14">
-        <v>0</v>
-      </c>
-      <c r="K14" t="str">
-        <v>-</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15">
-        <v>14</v>
-      </c>
-      <c r="B15" t="str">
-        <v>10/28/2026</v>
-      </c>
-      <c r="C15" t="str">
-        <v>เทรคกิ้งเสือกระโจน วันสอง</v>
-      </c>
-      <c r="D15" t="str">
-        <v>เดิน</v>
-      </c>
-      <c r="E15" t="str">
-        <v>香格里拉山美客栈(东环线分店)  中峡国际青年旅舍Tina'S Guest House</v>
-      </c>
-      <c r="F15" t="str">
-        <v>-</v>
-      </c>
-      <c r="G15">
-        <v>0</v>
-      </c>
-      <c r="H15">
-        <v>0</v>
-      </c>
-      <c r="I15">
-        <v>0</v>
-      </c>
-      <c r="J15">
-        <v>0</v>
-      </c>
-      <c r="K15" t="str">
-        <v>-</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16">
-        <v>15</v>
-      </c>
-      <c r="B16" t="str">
-        <v>10/28/2026</v>
-      </c>
-      <c r="C16" t="str">
-        <v>เมืองโบราณตู๋เค่อจง-ที่พักแชงกีลา</v>
-      </c>
-      <c r="D16" t="str">
-        <v>เดิน</v>
-      </c>
-      <c r="E16" t="str">
-        <v>香格里拉市独克宗古城(北门) [280101]  香格里拉望山小院客栈(独克宗古城店) [280102]  静静的嘛呢石藏餐吧(北门店) [280103]  龟山公园 [280104]</v>
-      </c>
-      <c r="F16" t="str">
-        <v>https://surl.amap.com/2Q0zUvse1n2aI</v>
-      </c>
-      <c r="G16">
-        <v>0</v>
-      </c>
-      <c r="H16">
-        <v>0</v>
-      </c>
-      <c r="I16">
-        <v>0</v>
-      </c>
-      <c r="J16">
-        <v>0</v>
-      </c>
-      <c r="K16" t="str">
-        <v>-</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17">
-        <v>16</v>
-      </c>
-      <c r="B17" t="str">
-        <v>10/29/2026</v>
-      </c>
-      <c r="C17" t="str">
-        <v>ที่พักแชงกีลา-อุทยานผู่ต๋าชั่ว</v>
-      </c>
-      <c r="D17" t="str">
-        <v>รถบัส</v>
-      </c>
-      <c r="E17" t="str">
-        <v>香格里拉独克宗古城东门客运站售票点  普达措国家公园入口游客中心</v>
-      </c>
-      <c r="F17" t="str">
-        <v>-</v>
-      </c>
-      <c r="G17">
-        <v>178</v>
-      </c>
-      <c r="H17">
-        <v>890</v>
-      </c>
-      <c r="I17">
-        <v>356</v>
-      </c>
-      <c r="J17">
-        <v>1780</v>
-      </c>
-      <c r="K17" t="str">
-        <v>ไป 8.20-9.05</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18">
-        <v>17</v>
-      </c>
-      <c r="B18" t="str">
-        <v>10/29/2026</v>
-      </c>
-      <c r="C18" t="str">
-        <v>อุทยานผู่ต๋าชั่ว-ที่พักแชงกีลา</v>
-      </c>
-      <c r="D18" t="str">
-        <v>รถบัส</v>
-      </c>
-      <c r="E18" t="str">
-        <v>普达措国家公园入口游客中心  香格里拉独克宗古城东门客运站售票点</v>
-      </c>
-      <c r="F18" t="str">
-        <v>-</v>
-      </c>
-      <c r="G18">
-        <v>0</v>
-      </c>
-      <c r="H18">
-        <v>0</v>
-      </c>
-      <c r="I18">
-        <v>0</v>
-      </c>
-      <c r="J18">
-        <v>0</v>
-      </c>
-      <c r="K18" t="str">
-        <v>กลับ 15.00-15.45</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19">
-        <v>18</v>
-      </c>
-      <c r="B19" t="str">
-        <v>10/29/2026</v>
-      </c>
-      <c r="C19" t="str">
-        <v>ที่พักแชงกีลา-คาเฟ่-ร้านอาหาร</v>
-      </c>
-      <c r="D19" t="str">
-        <v>เดิน</v>
-      </c>
-      <c r="E19" t="str">
-        <v>香格里拉望山小院客栈(独克宗古城店)  古城角落甜茶馆  宏宏无烟石板烧烤</v>
-      </c>
-      <c r="F19" t="str">
-        <v>https://surl.amap.com/3aWWUho1o6Qb</v>
-      </c>
-      <c r="G19">
-        <v>0</v>
-      </c>
-      <c r="H19">
-        <v>0</v>
-      </c>
-      <c r="I19">
-        <v>0</v>
-      </c>
-      <c r="J19">
-        <v>0</v>
-      </c>
-      <c r="K19" t="str">
-        <v>-</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20">
-        <v>19</v>
-      </c>
-      <c r="B20" t="str">
-        <v>10/30/2026</v>
-      </c>
-      <c r="C20" t="str">
-        <v>ที่พักแชงกีลา-ตลาด</v>
-      </c>
-      <c r="D20" t="str">
-        <v>เดิน</v>
-      </c>
-      <c r="E20" t="str">
-        <v>香格里拉望山小院客栈(独克宗古城店)  金桥向阳菜市场(向阳路农贸综合市场店)</v>
-      </c>
-      <c r="F20" t="str">
-        <v>https://surl.amap.com/37LSs3sS8SI</v>
-      </c>
-      <c r="G20">
-        <v>0</v>
-      </c>
-      <c r="H20">
-        <v>0</v>
-      </c>
-      <c r="I20">
-        <v>0</v>
-      </c>
-      <c r="J20">
-        <v>0</v>
-      </c>
-      <c r="K20" t="str">
-        <v>-</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21">
-        <v>20</v>
-      </c>
-      <c r="B21" t="str">
-        <v>10/30/2026</v>
-      </c>
-      <c r="C21" t="str">
-        <v>ตลาด-วัดซงจ้านหลิน</v>
-      </c>
-      <c r="D21" t="str">
-        <v>รถบัส</v>
-      </c>
-      <c r="E21" t="str">
-        <v>金桥向阳菜市场(向阳路农贸综合市场店)  噶丹松赞林寺  游客服务中心 (กินข้าว)</v>
-      </c>
-      <c r="F21" t="str">
-        <v>https://surl.amap.com/fe10g66KcYw</v>
-      </c>
-      <c r="G21">
-        <v>2</v>
-      </c>
-      <c r="H21">
-        <v>10</v>
-      </c>
-      <c r="I21">
-        <v>4</v>
-      </c>
-      <c r="J21">
-        <v>20</v>
-      </c>
-      <c r="K21" t="str">
-        <v>กินข้าวที่游客服务中心</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22">
-        <v>21</v>
-      </c>
-      <c r="B22" t="str">
-        <v>10/30/2026</v>
-      </c>
-      <c r="C22" t="str">
-        <v>วัดซงจ้านหลิน-ที่พักแชงกีลา</v>
-      </c>
-      <c r="D22" t="str">
-        <v>รถบัส</v>
-      </c>
-      <c r="E22" t="str">
-        <v>噶丹松赞林寺  香格里拉望山小院客栈(独克宗古城店)</v>
-      </c>
-      <c r="F22" t="str">
-        <v>https://surl.amap.com/2RRM1kq6aIj</v>
-      </c>
-      <c r="G22">
-        <v>2</v>
-      </c>
-      <c r="H22">
-        <v>10</v>
-      </c>
-      <c r="I22">
-        <v>4</v>
-      </c>
-      <c r="J22">
-        <v>20</v>
-      </c>
-      <c r="K22" t="str">
-        <v>-</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23">
-        <v>22</v>
-      </c>
-      <c r="B23" t="str">
-        <v>10/30/2026</v>
-      </c>
-      <c r="C23" t="str">
-        <v>ที่พักแชงกีลา-สถานีแชงกีลา</v>
-      </c>
-      <c r="D23" t="str">
-        <v>รถบัส</v>
-      </c>
-      <c r="E23" t="str">
-        <v>香格里拉望山小院客栈(独克宗古城店)  香格里拉站(进站口)</v>
-      </c>
-      <c r="F23" t="str">
-        <v>https://surl.amap.com/yN182yJoaRv</v>
-      </c>
-      <c r="G23">
-        <v>2</v>
-      </c>
-      <c r="H23">
-        <v>10</v>
-      </c>
-      <c r="I23">
-        <v>4</v>
-      </c>
-      <c r="J23">
-        <v>20</v>
-      </c>
-      <c r="K23" t="str">
-        <v>-</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24">
-        <v>23</v>
-      </c>
-      <c r="B24" t="str">
-        <v>10/30/2026</v>
-      </c>
-      <c r="C24" t="str">
-        <v>สถานีลี่เจียง-ที่พักเมืองเก่าลี่เจียง</v>
-      </c>
-      <c r="D24" t="str">
-        <v>รถบัส</v>
-      </c>
-      <c r="E24" t="str">
-        <v>丽江站  栖悦林隐别院(丽江古城忠义市场店)</v>
-      </c>
-      <c r="F24" t="str">
-        <v>https://surl.amap.com/3n4lXMyfeuQ</v>
-      </c>
-      <c r="G24">
-        <v>5</v>
-      </c>
-      <c r="H24">
-        <v>25</v>
-      </c>
-      <c r="I24">
-        <v>10</v>
-      </c>
-      <c r="J24">
-        <v>50</v>
-      </c>
-      <c r="K24" t="str">
-        <v>-</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25">
-        <v>24</v>
-      </c>
-      <c r="B25" t="str">
-        <v>10/30/2026</v>
-      </c>
-      <c r="C25" t="str">
-        <v>ที่พักเมืองเก่าลี่เจียง-ตลาดจงอี้</v>
-      </c>
-      <c r="D25" t="str">
-        <v>เดิน</v>
-      </c>
-      <c r="E25" t="str">
-        <v>栖悦林隐别院(丽江古城忠义市场店)  忠义市场夜市街</v>
-      </c>
-      <c r="F25" t="str">
-        <v>https://surl.amap.com/2HSTS4Jc155an</v>
-      </c>
-      <c r="G25">
-        <v>0</v>
-      </c>
-      <c r="H25">
-        <v>0</v>
-      </c>
-      <c r="I25">
-        <v>0</v>
-      </c>
-      <c r="J25">
-        <v>0</v>
-      </c>
-      <c r="K25" t="str">
-        <v>-</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26">
-        <v>25</v>
-      </c>
-      <c r="B26" t="str">
-        <v>10/31/2026</v>
-      </c>
-      <c r="C26" t="str">
-        <v>ที่พักเมืองเก่าลี่เจียง-สนามบินลี่เจียง</v>
-      </c>
-      <c r="D26" t="str">
-        <v>Didi</v>
-      </c>
-      <c r="E26" t="str">
-        <v>栖悦林隐别院(丽江古城忠义市场店) [260001]  丽江龙落河民宿(三义国际机场店)</v>
-      </c>
-      <c r="F26" t="str">
-        <v>-</v>
-      </c>
-      <c r="G26">
-        <v>36</v>
-      </c>
-      <c r="H26">
-        <v>180</v>
-      </c>
-      <c r="I26">
-        <v>72</v>
-      </c>
-      <c r="J26">
-        <v>360</v>
-      </c>
-      <c r="K26" t="str">
-        <v>-</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27">
-        <v>26</v>
-      </c>
-      <c r="B27" t="str">
-        <v>10/31/2026</v>
-      </c>
-      <c r="C27" t="str">
-        <v>สนามบินคุณหมิง-ร้านอาหาร</v>
-      </c>
-      <c r="D27" t="str">
-        <v>รถไฟ</v>
-      </c>
-      <c r="E27" t="str">
-        <v>昆明长水国际机场  广益饭店(北门街)</v>
-      </c>
-      <c r="F27" t="str">
-        <v>https://surl.amap.com/4psCbGureAF</v>
-      </c>
-      <c r="G27">
-        <v>6</v>
-      </c>
-      <c r="H27">
-        <v>30</v>
-      </c>
-      <c r="I27">
-        <v>12</v>
-      </c>
-      <c r="J27">
-        <v>60</v>
-      </c>
-      <c r="K27" t="str">
-        <v>-</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28">
-        <v>27</v>
-      </c>
-      <c r="B28" t="str">
-        <v>10/31/2026</v>
-      </c>
-      <c r="C28" t="str">
-        <v>ร้านอาหาร-สวนสาธารณะ</v>
-      </c>
-      <c r="D28" t="str">
-        <v>เดิน</v>
-      </c>
-      <c r="E28" t="str">
-        <v>广益饭店(北门街)  翠湖公园  云南陆军讲武堂历史博物馆  南屏步行街</v>
-      </c>
-      <c r="F28" t="str">
-        <v>https://surl.amap.com/4r8LFT819c1S</v>
-      </c>
-      <c r="G28">
-        <v>0</v>
-      </c>
-      <c r="H28">
-        <v>0</v>
-      </c>
-      <c r="I28">
-        <v>0</v>
-      </c>
-      <c r="J28">
-        <v>0</v>
-      </c>
-      <c r="K28" t="str">
-        <v>-</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29">
-        <v>28</v>
-      </c>
-      <c r="B29" t="str">
-        <v>10/31/2026</v>
-      </c>
-      <c r="C29" t="str">
-        <v>ถนนคนเดิน-สนามบินคุณหมิง</v>
-      </c>
-      <c r="D29" t="str">
-        <v>รถไฟ</v>
-      </c>
-      <c r="E29" t="str">
-        <v>南屏步行街  昆明长水国际机场</v>
-      </c>
-      <c r="F29" t="str">
-        <v>https://surl.amap.com/tP208A1cceK</v>
-      </c>
-      <c r="G29">
-        <v>6</v>
-      </c>
-      <c r="H29">
-        <v>30</v>
-      </c>
-      <c r="I29">
-        <v>12</v>
-      </c>
-      <c r="J29">
-        <v>60</v>
-      </c>
-      <c r="K29" t="str">
-        <v>-</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="str">
-        <v/>
-      </c>
-      <c r="B30" t="str">
-        <v>รวมทั้งหมด (คณะ 2 คน)</v>
-      </c>
-      <c r="C30" t="str">
-        <v/>
-      </c>
-      <c r="D30" t="str">
-        <v/>
-      </c>
-      <c r="E30" t="str">
-        <v/>
-      </c>
-      <c r="F30" t="str">
-        <v/>
-      </c>
-      <c r="G30">
-        <v>391.5</v>
-      </c>
-      <c r="H30">
-        <v>1957.5</v>
-      </c>
-      <c r="I30">
-        <v>783</v>
-      </c>
-      <c r="J30">
-        <v>3915</v>
-      </c>
-      <c r="K30" t="str">
-        <v>ยอดรวม 2 คน = ¥783.00 (฿3,915.00) | เฉลี่ยคนละ ¥391.50 (฿1,957.50)</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K30"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G10"/>
   <sheetData>

</xml_diff>

<commit_message>
Add sheet 10_งบอาหารรายร้าน with all 21 meal breakdowns
</commit_message>
<xml_diff>
--- a/yunnan_travel_plan_2026.xlsx
+++ b/yunnan_travel_plan_2026.xlsx
@@ -12,6 +12,7 @@
     <sheet name="07_การเดินทาง 28 เที่ยว" sheetId="7" r:id="rId7"/>
     <sheet name="08_ตารางหลัก (Master)" sheetId="8" r:id="rId8"/>
     <sheet name="09_สถิติรายวัน" sheetId="9" r:id="rId9"/>
+    <sheet name="10_งบอาหารรายร้าน" sheetId="10" r:id="rId10"/>
   </sheets>
 </workbook>
 </file>
@@ -406,20 +407,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L64"/>
-  <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="45.83203125" customWidth="1"/>
-    <col min="5" max="5" width="25.83203125" customWidth="1"/>
-    <col min="6" max="6" width="15.83203125" customWidth="1"/>
-    <col min="7" max="7" width="30.83203125" customWidth="1"/>
-    <col min="8" max="8" width="15.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="15.83203125" customWidth="1"/>
-    <col min="11" max="11" width="15.83203125" customWidth="1"/>
-    <col min="12" max="12" width="25.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2860,18 +2847,698 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I23"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="42.83203125" customWidth="1"/>
+    <col min="4" max="4" width="46.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="16.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="35.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>วัน</v>
+      </c>
+      <c r="B1" t="str">
+        <v>มื้อ</v>
+      </c>
+      <c r="C1" t="str">
+        <v>ร้านอาหาร / สถานที่</v>
+      </c>
+      <c r="D1" t="str">
+        <v>เมนูแนะนำ</v>
+      </c>
+      <c r="E1" t="str">
+        <v>ราคา/คน (¥)</v>
+      </c>
+      <c r="F1" t="str">
+        <v>ราคา/คน (฿)</v>
+      </c>
+      <c r="G1" t="str">
+        <v>รวม 2 คน (¥)</v>
+      </c>
+      <c r="H1" t="str">
+        <v>รวม 2 คน (฿)</v>
+      </c>
+      <c r="I1" t="str">
+        <v>หมายเหตุ</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Day 2</v>
+      </c>
+      <c r="B2" t="str">
+        <v>มื้อเที่ยง</v>
+      </c>
+      <c r="C2" t="str">
+        <v>ร้านก๋วยเตี๋ยวข้ามสะพาน เจี้ยนซินหยวน (建新园 宝善街店)</v>
+      </c>
+      <c r="D2" t="str">
+        <v>ชุดก๋วยเตี๋ยวข้ามสะพานซุปไก่ทองคำเดือดจัด เครื่องเคียงครบเซต</v>
+      </c>
+      <c r="E2">
+        <v>35</v>
+      </c>
+      <c r="F2">
+        <v>175</v>
+      </c>
+      <c r="G2">
+        <v>70</v>
+      </c>
+      <c r="H2">
+        <v>350</v>
+      </c>
+      <c r="I2" t="str">
+        <v>แบรนด์เก่าแก่ร้อยปียูนนาน</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Day 2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>ของว่างบ่าย</v>
+      </c>
+      <c r="C3" t="str">
+        <v>ถนนคนเดินหนานผิง &amp; สวนชุ่ยหู</v>
+      </c>
+      <c r="D3" t="str">
+        <v>ขนมเปี๊ยะดอกไม้สด (鲜花饼), ชานมยูนนาน</v>
+      </c>
+      <c r="E3">
+        <v>15</v>
+      </c>
+      <c r="F3">
+        <v>75</v>
+      </c>
+      <c r="G3">
+        <v>30</v>
+      </c>
+      <c r="H3">
+        <v>150</v>
+      </c>
+      <c r="I3" t="str">
+        <v>ขนมเปี๊ยะอบสดหอมกลิ่นกุหลาบ</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Day 2</v>
+      </c>
+      <c r="B4" t="str">
+        <v>มื้อเย็น</v>
+      </c>
+      <c r="C4" t="str">
+        <v>ตลาดสดต้ากวนจ้วนซิน (大观篆新农贸市场)</v>
+      </c>
+      <c r="D4" t="str">
+        <v>ไก่ฉีก, เต้าหู้ย่าง, ข้าวผัดยูนนาน, ผลไม้สด</v>
+      </c>
+      <c r="E4">
+        <v>40</v>
+      </c>
+      <c r="F4">
+        <v>200</v>
+      </c>
+      <c r="G4">
+        <v>80</v>
+      </c>
+      <c r="H4">
+        <v>400</v>
+      </c>
+      <c r="I4" t="str">
+        <v>ตลาดอาหารพื้นเมืองชื่อดังคุนหมิง</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Day 3</v>
+      </c>
+      <c r="B5" t="str">
+        <v>มื้อเช้า</v>
+      </c>
+      <c r="C5" t="str">
+        <v>ร้านอาหารเช้าใกล้ที่พัก / สนามบินลี่เจียง</v>
+      </c>
+      <c r="D5" t="str">
+        <v>ซาลาเปาร้อน, โจ๊ก, นมถั่วเหลืองสด</v>
+      </c>
+      <c r="E5">
+        <v>15</v>
+      </c>
+      <c r="F5">
+        <v>75</v>
+      </c>
+      <c r="G5">
+        <v>30</v>
+      </c>
+      <c r="H5">
+        <v>150</v>
+      </c>
+      <c r="I5" t="str">
+        <v>อาหารเช้าเติมพลังก่อนเข้าเมือง</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Day 3</v>
+      </c>
+      <c r="B6" t="str">
+        <v>มื้อเที่ยง</v>
+      </c>
+      <c r="C6" t="str">
+        <v>หม้อไฟซี่โครงหมูดั้งเดิม อาผอฉิง (阿婆情腊排骨 忠义店)</v>
+      </c>
+      <c r="D6" t="str">
+        <v>หม้อไฟซี่โครงหมูหมักเกลือสูตรน่าซี ผักสด เห็ดป่า ซุปกระดูกเข้มข้น</v>
+      </c>
+      <c r="E6">
+        <v>60</v>
+      </c>
+      <c r="F6">
+        <v>300</v>
+      </c>
+      <c r="G6">
+        <v>120</v>
+      </c>
+      <c r="H6">
+        <v>600</v>
+      </c>
+      <c r="I6" t="str">
+        <v>ร้านดังใกล้ประตูใต้เมืองเก่า</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Day 3</v>
+      </c>
+      <c r="B7" t="str">
+        <v>มื้อค่ำ</v>
+      </c>
+      <c r="C7" t="str">
+        <v>ตลาดโต้รุ่งจงอี้ &amp; เมืองเก่าลี่เจียง (忠义夜市)</v>
+      </c>
+      <c r="D7" t="str">
+        <v>ปิ้งย่างหม่าล่า, ข้าวปุกงาดำปิ้ง (烤饵块), โรตีทิเบต (粑粑)</v>
+      </c>
+      <c r="E7">
+        <v>40</v>
+      </c>
+      <c r="F7">
+        <v>200</v>
+      </c>
+      <c r="G7">
+        <v>80</v>
+      </c>
+      <c r="H7">
+        <v>400</v>
+      </c>
+      <c r="I7" t="str">
+        <v>สตรีทฟู้ดชาวน่าซีแท้ๆ</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Day 4</v>
+      </c>
+      <c r="B8" t="str">
+        <v>มื้อเช้า</v>
+      </c>
+      <c r="C8" t="str">
+        <v>ร้านอาหารเช้าก่อนขึ้นรถบัส สถานีขนส่งลี่เจียง</v>
+      </c>
+      <c r="D8" t="str">
+        <v>ซาลาเปา, ขนมปัง, กาแฟ, ไข่ต้มพกเดินป่า</v>
+      </c>
+      <c r="E8">
+        <v>15</v>
+      </c>
+      <c r="F8">
+        <v>75</v>
+      </c>
+      <c r="G8">
+        <v>30</v>
+      </c>
+      <c r="H8">
+        <v>150</v>
+      </c>
+      <c r="I8" t="str">
+        <v>พกขนมและน้ำขึ้นรถบัส</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Day 4</v>
+      </c>
+      <c r="B9" t="str">
+        <v>มื้อเที่ยง</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Naxi Family Guesthouse (纳西雅阁)</v>
+      </c>
+      <c r="D9" t="str">
+        <v>ข้าวผัดไข่, ผัดผักกาดตามสั่ง, ซุปมะเขือเทศร้อน</v>
+      </c>
+      <c r="E9">
+        <v>35</v>
+      </c>
+      <c r="F9">
+        <v>175</v>
+      </c>
+      <c r="G9">
+        <v>70</v>
+      </c>
+      <c r="H9">
+        <v>350</v>
+      </c>
+      <c r="I9" t="str">
+        <v>จุดพักเติมพลังก่อนขึ้น 28 Bends</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Day 4</v>
+      </c>
+      <c r="B10" t="str">
+        <v>มื้อเย็น</v>
+      </c>
+      <c r="C10" t="str">
+        <v>ห้องอาหาร Summit Inn (虎跳峡山美客栈)</v>
+      </c>
+      <c r="D10" t="str">
+        <v>ผัดไก่พริกขิง, ผัดมะเขือยาว, ซุปผัก ชมวิวระเบียงช่องเขา</v>
+      </c>
+      <c r="E10">
+        <v>50</v>
+      </c>
+      <c r="F10">
+        <v>250</v>
+      </c>
+      <c r="G10">
+        <v>100</v>
+      </c>
+      <c r="H10">
+        <v>500</v>
+      </c>
+      <c r="I10" t="str">
+        <v>อาหารปรุงสดบนเขาเสือกระโจน</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Day 5</v>
+      </c>
+      <c r="B11" t="str">
+        <v>มื้อเช้า</v>
+      </c>
+      <c r="C11" t="str">
+        <v>ห้องอาหาร Summit Inn / Halfway Guesthouse</v>
+      </c>
+      <c r="D11" t="str">
+        <v>แพนเค้กไข่, บะหมี่น้ำร้อน, กาแฟดริปชมวิวเขา</v>
+      </c>
+      <c r="E11">
+        <v>25</v>
+      </c>
+      <c r="F11">
+        <v>125</v>
+      </c>
+      <c r="G11">
+        <v>50</v>
+      </c>
+      <c r="H11">
+        <v>250</v>
+      </c>
+      <c r="I11" t="str">
+        <v>ชมแสงเช้าหน้าผาหิน</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Day 5</v>
+      </c>
+      <c r="B12" t="str">
+        <v>มื้อเที่ยง</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Tina's Guesthouse / คาเฟ่ Moye (墨野咖啡)</v>
+      </c>
+      <c r="D12" t="str">
+        <v>ข้าวผัดเนื้อจามรี, บะหมี่ผัด, แซนด์วิช, กาแฟสด</v>
+      </c>
+      <c r="E12">
+        <v>35</v>
+      </c>
+      <c r="F12">
+        <v>175</v>
+      </c>
+      <c r="G12">
+        <v>70</v>
+      </c>
+      <c r="H12">
+        <v>350</v>
+      </c>
+      <c r="I12" t="str">
+        <v>พักผ่อนรอรถบัสไปแชงกรี-ลา</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Day 5</v>
+      </c>
+      <c r="B13" t="str">
+        <v>มื้อค่ำ</v>
+      </c>
+      <c r="C13" t="str">
+        <v>ร้านอาหารทิเบต จิ้งจิ้งเตอะมานีฉือ (静静的嘛呢石藏餐吧)</v>
+      </c>
+      <c r="D13" t="str">
+        <v>ซี่โครงแกะย่างทิเบต, ชาเนยจามรีร้อน, ขนมปังบาบานมจามรี, ผัดเนื้อจามรี</v>
+      </c>
+      <c r="E13">
+        <v>65</v>
+      </c>
+      <c r="F13">
+        <v>325</v>
+      </c>
+      <c r="G13">
+        <v>130</v>
+      </c>
+      <c r="H13">
+        <v>650</v>
+      </c>
+      <c r="I13" t="str">
+        <v>ร้านอาหารทิเบตชื่อดังประตูเหนือตู๋เค่อจง</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Day 6</v>
+      </c>
+      <c r="B14" t="str">
+        <v>มื้อเช้า</v>
+      </c>
+      <c r="C14" t="str">
+        <v>ร้านอาหารเช้าใกล้ที่พัก เมืองโบราณตู๋เค่อจง</v>
+      </c>
+      <c r="D14" t="str">
+        <v>ซาลาเปานึ่งสด, ชาร้อน, โจ๊กเนื้อจามรี, ไข่ต้ม</v>
+      </c>
+      <c r="E14">
+        <v>15</v>
+      </c>
+      <c r="F14">
+        <v>75</v>
+      </c>
+      <c r="G14">
+        <v>30</v>
+      </c>
+      <c r="H14">
+        <v>150</v>
+      </c>
+      <c r="I14" t="str">
+        <v>อาหารเช้าก่อนขึ้นที่สูงผู่ต๋าชั่ว</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Day 6</v>
+      </c>
+      <c r="B15" t="str">
+        <v>มื้อเที่ยง</v>
+      </c>
+      <c r="C15" t="str">
+        <v>ศูนย์บริการนักท่องเที่ยวอุทยานแห่งชาติผู่ต๋าชั่ว</v>
+      </c>
+      <c r="D15" t="str">
+        <v>ข้าวกล่องร้อน, บะหมี่ซุปเนื้อ, ชาขิงคลายหนาว</v>
+      </c>
+      <c r="E15">
+        <v>35</v>
+      </c>
+      <c r="F15">
+        <v>175</v>
+      </c>
+      <c r="G15">
+        <v>70</v>
+      </c>
+      <c r="H15">
+        <v>350</v>
+      </c>
+      <c r="I15" t="str">
+        <v>ทานในอาคารศูนย์บริการคลายหนาว</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Day 6</v>
+      </c>
+      <c r="B16" t="str">
+        <v>มื้อเย็น</v>
+      </c>
+      <c r="C16" t="str">
+        <v>ร้านปิ้งย่างบนแผ่นหิน หงหง (宏宏无烟石板烧烤)</v>
+      </c>
+      <c r="D16" t="str">
+        <v>ปิ้งย่างแผ่นหินเนื้อจามรี, เห็ดป่าย่างเนย, มันฝรั่งทิเบต</v>
+      </c>
+      <c r="E16">
+        <v>60</v>
+      </c>
+      <c r="F16">
+        <v>300</v>
+      </c>
+      <c r="G16">
+        <v>120</v>
+      </c>
+      <c r="H16">
+        <v>600</v>
+      </c>
+      <c r="I16" t="str">
+        <v>ปิ้งย่างบนแผ่นหินร้อนไร้ควันยอดนิยม</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Day 7</v>
+      </c>
+      <c r="B17" t="str">
+        <v>มื้อเช้า</v>
+      </c>
+      <c r="C17" t="str">
+        <v>ตลาดเช้าจินเฉียวเซี่ยงหยาง (金桥向阳菜市场)</v>
+      </c>
+      <c r="D17" t="str">
+        <v>นมจามรีต้มสด, ปาท่องโก๋ยักษ์, เสี่ยวหลงเปาทิเบต</v>
+      </c>
+      <c r="E17">
+        <v>15</v>
+      </c>
+      <c r="F17">
+        <v>75</v>
+      </c>
+      <c r="G17">
+        <v>30</v>
+      </c>
+      <c r="H17">
+        <v>150</v>
+      </c>
+      <c r="I17" t="str">
+        <v>สัมผัสวิถีชีวิตชาวบ้านยามเช้า</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Day 7</v>
+      </c>
+      <c r="B18" t="str">
+        <v>มื้อเที่ยง</v>
+      </c>
+      <c r="C18" t="str">
+        <v>ศูนย์บริการนักท่องเที่ยววัดซงจ้านหลิน</v>
+      </c>
+      <c r="D18" t="str">
+        <v>ข้าวราดแกงยูนนาน, บะหมี่ซุปเนื้อน้ำใส</v>
+      </c>
+      <c r="E18">
+        <v>30</v>
+      </c>
+      <c r="F18">
+        <v>150</v>
+      </c>
+      <c r="G18">
+        <v>60</v>
+      </c>
+      <c r="H18">
+        <v>300</v>
+      </c>
+      <c r="I18" t="str">
+        <v>ทานก่อนขึ้นรถไฟความเร็วสูงกลับลี่เจียง</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Day 7</v>
+      </c>
+      <c r="B19" t="str">
+        <v>มื้อค่ำ</v>
+      </c>
+      <c r="C19" t="str">
+        <v>ตลาดโต้รุ่งจงอี้ ลี่เจียง / ซอยอาหารน่าซี</v>
+      </c>
+      <c r="D19" t="str">
+        <v>หม้อไฟปลาหิมะยูนนาน, ปิ้งย่างน่าซี, วุ้นถั่วไก่ (鸡豆凉粉)</v>
+      </c>
+      <c r="E19">
+        <v>50</v>
+      </c>
+      <c r="F19">
+        <v>250</v>
+      </c>
+      <c r="G19">
+        <v>100</v>
+      </c>
+      <c r="H19">
+        <v>500</v>
+      </c>
+      <c r="I19" t="str">
+        <v>ฉลองค่ำคืนสุดท้ายในลี่เจียง</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Day 8</v>
+      </c>
+      <c r="B20" t="str">
+        <v>มื้อเช้า</v>
+      </c>
+      <c r="C20" t="str">
+        <v>ร้านอาหารเช้าหน้าสนามบินลี่เจียง (LJG)</v>
+      </c>
+      <c r="D20" t="str">
+        <v>กาแฟร้อน, ซาลาเปา, แซนด์วิชเบาๆ</v>
+      </c>
+      <c r="E20">
+        <v>15</v>
+      </c>
+      <c r="F20">
+        <v>75</v>
+      </c>
+      <c r="G20">
+        <v>30</v>
+      </c>
+      <c r="H20">
+        <v>150</v>
+      </c>
+      <c r="I20" t="str">
+        <v>ก่อนขึ้นไฟลท์ MU-5922</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Day 8</v>
+      </c>
+      <c r="B21" t="str">
+        <v>มื้อเที่ยง</v>
+      </c>
+      <c r="C21" t="str">
+        <v>ร้านกว่างอี้ฟั่นเตี้ยน (广益饭店 北门街店 คุนหมิง)</v>
+      </c>
+      <c r="D21" t="str">
+        <v>หมูสามชั้นตุ๋นน้ำแดงยูนนาน, ไก่ผัดพริกแห้ง, ซุปเห็ดรวม</v>
+      </c>
+      <c r="E21">
+        <v>50</v>
+      </c>
+      <c r="F21">
+        <v>250</v>
+      </c>
+      <c r="G21">
+        <v>100</v>
+      </c>
+      <c r="H21">
+        <v>500</v>
+      </c>
+      <c r="I21" t="str">
+        <v>ร้านอาหารยูนนานเก่าแก่ใกล้สวนชุ่ยหู</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Day 8</v>
+      </c>
+      <c r="B22" t="str">
+        <v>มื้อค่ำ</v>
+      </c>
+      <c r="C22" t="str">
+        <v>สนามบินคุนหมิงฉางสุ่ย (KMG) ก่อนบินกลับ</v>
+      </c>
+      <c r="D22" t="str">
+        <v>ก๋วยเตี๋ยวร้อน, ชายูนนาน, ขนมเปี๊ยะสด</v>
+      </c>
+      <c r="E22">
+        <v>40</v>
+      </c>
+      <c r="F22">
+        <v>200</v>
+      </c>
+      <c r="G22">
+        <v>80</v>
+      </c>
+      <c r="H22">
+        <v>400</v>
+      </c>
+      <c r="I22" t="str">
+        <v>ทานก่อนผ่านเกตขึ้นเครื่องกลับไทย</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>รวมทั้งหมด</v>
+      </c>
+      <c r="B23" t="str">
+        <v>21 มื้อ ตลอดทริป</v>
+      </c>
+      <c r="C23" t="str">
+        <v>รวมทุกร้านอาหาร/สตรีทฟู้ด/ตลาดสด/คาเฟ่</v>
+      </c>
+      <c r="D23" t="str">
+        <v>ครอบคลุมครบทุกมื้อเช้า เที่ยง ค่ำ ตลอด 8 วัน</v>
+      </c>
+      <c r="E23">
+        <v>770</v>
+      </c>
+      <c r="F23">
+        <v>3850</v>
+      </c>
+      <c r="G23">
+        <v>1540</v>
+      </c>
+      <c r="H23">
+        <v>7700</v>
+      </c>
+      <c r="I23" t="str">
+        <v>ประมาณการเฉลี่ย ¥770 (฿3,850)/คน (รวม 2 คน ฿7,700)</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:I23"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G27"/>
-  <cols>
-    <col min="1" max="1" width="25.83203125" customWidth="1"/>
-    <col min="2" max="2" width="40.83203125" customWidth="1"/>
-    <col min="3" max="3" width="22.83203125" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" customWidth="1"/>
-    <col min="5" max="5" width="18.83203125" customWidth="1"/>
-    <col min="6" max="6" width="18.83203125" customWidth="1"/>
-    <col min="7" max="7" width="18.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3435,16 +4102,6 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H12"/>
-  <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="32.83203125" customWidth="1"/>
-    <col min="3" max="3" width="35.83203125" customWidth="1"/>
-    <col min="4" max="4" width="28.83203125" customWidth="1"/>
-    <col min="5" max="5" width="22.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" customWidth="1"/>
-    <col min="8" max="8" width="45.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3768,14 +4425,6 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F27"/>
-  <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="32.83203125" customWidth="1"/>
-    <col min="4" max="4" width="35.83203125" customWidth="1"/>
-    <col min="5" max="5" width="32.83203125" customWidth="1"/>
-    <col min="6" max="6" width="40.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4327,13 +4976,6 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E8"/>
-  <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="38.83203125" customWidth="1"/>
-    <col min="3" max="3" width="45.83203125" customWidth="1"/>
-    <col min="4" max="4" width="45.83203125" customWidth="1"/>
-    <col min="5" max="5" width="40.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4481,12 +5123,6 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D9"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="70.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4716,19 +5352,6 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K30"/>
-  <cols>
-    <col min="1" max="1" width="8.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="28.83203125" customWidth="1"/>
-    <col min="4" max="4" width="15.83203125" customWidth="1"/>
-    <col min="5" max="5" width="45.83203125" customWidth="1"/>
-    <col min="6" max="6" width="28.83203125" customWidth="1"/>
-    <col min="7" max="7" width="15.83203125" customWidth="1"/>
-    <col min="8" max="8" width="18.83203125" customWidth="1"/>
-    <col min="9" max="9" width="15.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="20.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>

<commit_message>
Clean Excel master sheets removing 21-meal breakdown sheet
</commit_message>
<xml_diff>
--- a/yunnan_travel_plan_2026.xlsx
+++ b/yunnan_travel_plan_2026.xlsx
@@ -12,7 +12,6 @@
     <sheet name="07_การเดินทาง 28 เที่ยว" sheetId="7" r:id="rId7"/>
     <sheet name="08_ตารางหลัก (Master)" sheetId="8" r:id="rId8"/>
     <sheet name="09_สถิติรายวัน" sheetId="9" r:id="rId9"/>
-    <sheet name="10_งบอาหารรายร้าน" sheetId="10" r:id="rId10"/>
   </sheets>
 </workbook>
 </file>
@@ -2847,695 +2846,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I23"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="42.83203125" customWidth="1"/>
-    <col min="4" max="4" width="46.83203125" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="35.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>วัน</v>
-      </c>
-      <c r="B1" t="str">
-        <v>มื้อ</v>
-      </c>
-      <c r="C1" t="str">
-        <v>ร้านอาหาร / สถานที่</v>
-      </c>
-      <c r="D1" t="str">
-        <v>เมนูแนะนำ</v>
-      </c>
-      <c r="E1" t="str">
-        <v>ราคา/คน (¥)</v>
-      </c>
-      <c r="F1" t="str">
-        <v>ราคา/คน (฿)</v>
-      </c>
-      <c r="G1" t="str">
-        <v>รวม 2 คน (¥)</v>
-      </c>
-      <c r="H1" t="str">
-        <v>รวม 2 คน (฿)</v>
-      </c>
-      <c r="I1" t="str">
-        <v>หมายเหตุ</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Day 2</v>
-      </c>
-      <c r="B2" t="str">
-        <v>มื้อเที่ยง</v>
-      </c>
-      <c r="C2" t="str">
-        <v>ร้านก๋วยเตี๋ยวข้ามสะพาน เจี้ยนซินหยวน (建新园 宝善街店)</v>
-      </c>
-      <c r="D2" t="str">
-        <v>ชุดก๋วยเตี๋ยวข้ามสะพานซุปไก่ทองคำเดือดจัด เครื่องเคียงครบเซต</v>
-      </c>
-      <c r="E2">
-        <v>35</v>
-      </c>
-      <c r="F2">
-        <v>175</v>
-      </c>
-      <c r="G2">
-        <v>70</v>
-      </c>
-      <c r="H2">
-        <v>350</v>
-      </c>
-      <c r="I2" t="str">
-        <v>แบรนด์เก่าแก่ร้อยปียูนนาน</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Day 2</v>
-      </c>
-      <c r="B3" t="str">
-        <v>ของว่างบ่าย</v>
-      </c>
-      <c r="C3" t="str">
-        <v>ถนนคนเดินหนานผิง &amp; สวนชุ่ยหู</v>
-      </c>
-      <c r="D3" t="str">
-        <v>ขนมเปี๊ยะดอกไม้สด (鲜花饼), ชานมยูนนาน</v>
-      </c>
-      <c r="E3">
-        <v>15</v>
-      </c>
-      <c r="F3">
-        <v>75</v>
-      </c>
-      <c r="G3">
-        <v>30</v>
-      </c>
-      <c r="H3">
-        <v>150</v>
-      </c>
-      <c r="I3" t="str">
-        <v>ขนมเปี๊ยะอบสดหอมกลิ่นกุหลาบ</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Day 2</v>
-      </c>
-      <c r="B4" t="str">
-        <v>มื้อเย็น</v>
-      </c>
-      <c r="C4" t="str">
-        <v>ตลาดสดต้ากวนจ้วนซิน (大观篆新农贸市场)</v>
-      </c>
-      <c r="D4" t="str">
-        <v>ไก่ฉีก, เต้าหู้ย่าง, ข้าวผัดยูนนาน, ผลไม้สด</v>
-      </c>
-      <c r="E4">
-        <v>40</v>
-      </c>
-      <c r="F4">
-        <v>200</v>
-      </c>
-      <c r="G4">
-        <v>80</v>
-      </c>
-      <c r="H4">
-        <v>400</v>
-      </c>
-      <c r="I4" t="str">
-        <v>ตลาดอาหารพื้นเมืองชื่อดังคุนหมิง</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Day 3</v>
-      </c>
-      <c r="B5" t="str">
-        <v>มื้อเช้า</v>
-      </c>
-      <c r="C5" t="str">
-        <v>ร้านอาหารเช้าใกล้ที่พัก / สนามบินลี่เจียง</v>
-      </c>
-      <c r="D5" t="str">
-        <v>ซาลาเปาร้อน, โจ๊ก, นมถั่วเหลืองสด</v>
-      </c>
-      <c r="E5">
-        <v>15</v>
-      </c>
-      <c r="F5">
-        <v>75</v>
-      </c>
-      <c r="G5">
-        <v>30</v>
-      </c>
-      <c r="H5">
-        <v>150</v>
-      </c>
-      <c r="I5" t="str">
-        <v>อาหารเช้าเติมพลังก่อนเข้าเมือง</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Day 3</v>
-      </c>
-      <c r="B6" t="str">
-        <v>มื้อเที่ยง</v>
-      </c>
-      <c r="C6" t="str">
-        <v>หม้อไฟซี่โครงหมูดั้งเดิม อาผอฉิง (阿婆情腊排骨 忠义店)</v>
-      </c>
-      <c r="D6" t="str">
-        <v>หม้อไฟซี่โครงหมูหมักเกลือสูตรน่าซี ผักสด เห็ดป่า ซุปกระดูกเข้มข้น</v>
-      </c>
-      <c r="E6">
-        <v>60</v>
-      </c>
-      <c r="F6">
-        <v>300</v>
-      </c>
-      <c r="G6">
-        <v>120</v>
-      </c>
-      <c r="H6">
-        <v>600</v>
-      </c>
-      <c r="I6" t="str">
-        <v>ร้านดังใกล้ประตูใต้เมืองเก่า</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Day 3</v>
-      </c>
-      <c r="B7" t="str">
-        <v>มื้อค่ำ</v>
-      </c>
-      <c r="C7" t="str">
-        <v>ตลาดโต้รุ่งจงอี้ &amp; เมืองเก่าลี่เจียง (忠义夜市)</v>
-      </c>
-      <c r="D7" t="str">
-        <v>ปิ้งย่างหม่าล่า, ข้าวปุกงาดำปิ้ง (烤饵块), โรตีทิเบต (粑粑)</v>
-      </c>
-      <c r="E7">
-        <v>40</v>
-      </c>
-      <c r="F7">
-        <v>200</v>
-      </c>
-      <c r="G7">
-        <v>80</v>
-      </c>
-      <c r="H7">
-        <v>400</v>
-      </c>
-      <c r="I7" t="str">
-        <v>สตรีทฟู้ดชาวน่าซีแท้ๆ</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Day 4</v>
-      </c>
-      <c r="B8" t="str">
-        <v>มื้อเช้า</v>
-      </c>
-      <c r="C8" t="str">
-        <v>ร้านอาหารเช้าก่อนขึ้นรถบัส สถานีขนส่งลี่เจียง</v>
-      </c>
-      <c r="D8" t="str">
-        <v>ซาลาเปา, ขนมปัง, กาแฟ, ไข่ต้มพกเดินป่า</v>
-      </c>
-      <c r="E8">
-        <v>15</v>
-      </c>
-      <c r="F8">
-        <v>75</v>
-      </c>
-      <c r="G8">
-        <v>30</v>
-      </c>
-      <c r="H8">
-        <v>150</v>
-      </c>
-      <c r="I8" t="str">
-        <v>พกขนมและน้ำขึ้นรถบัส</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Day 4</v>
-      </c>
-      <c r="B9" t="str">
-        <v>มื้อเที่ยง</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Naxi Family Guesthouse (纳西雅阁)</v>
-      </c>
-      <c r="D9" t="str">
-        <v>ข้าวผัดไข่, ผัดผักกาดตามสั่ง, ซุปมะเขือเทศร้อน</v>
-      </c>
-      <c r="E9">
-        <v>35</v>
-      </c>
-      <c r="F9">
-        <v>175</v>
-      </c>
-      <c r="G9">
-        <v>70</v>
-      </c>
-      <c r="H9">
-        <v>350</v>
-      </c>
-      <c r="I9" t="str">
-        <v>จุดพักเติมพลังก่อนขึ้น 28 Bends</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>Day 4</v>
-      </c>
-      <c r="B10" t="str">
-        <v>มื้อเย็น</v>
-      </c>
-      <c r="C10" t="str">
-        <v>ห้องอาหาร Summit Inn (虎跳峡山美客栈)</v>
-      </c>
-      <c r="D10" t="str">
-        <v>ผัดไก่พริกขิง, ผัดมะเขือยาว, ซุปผัก ชมวิวระเบียงช่องเขา</v>
-      </c>
-      <c r="E10">
-        <v>50</v>
-      </c>
-      <c r="F10">
-        <v>250</v>
-      </c>
-      <c r="G10">
-        <v>100</v>
-      </c>
-      <c r="H10">
-        <v>500</v>
-      </c>
-      <c r="I10" t="str">
-        <v>อาหารปรุงสดบนเขาเสือกระโจน</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>Day 5</v>
-      </c>
-      <c r="B11" t="str">
-        <v>มื้อเช้า</v>
-      </c>
-      <c r="C11" t="str">
-        <v>ห้องอาหาร Summit Inn / Halfway Guesthouse</v>
-      </c>
-      <c r="D11" t="str">
-        <v>แพนเค้กไข่, บะหมี่น้ำร้อน, กาแฟดริปชมวิวเขา</v>
-      </c>
-      <c r="E11">
-        <v>25</v>
-      </c>
-      <c r="F11">
-        <v>125</v>
-      </c>
-      <c r="G11">
-        <v>50</v>
-      </c>
-      <c r="H11">
-        <v>250</v>
-      </c>
-      <c r="I11" t="str">
-        <v>ชมแสงเช้าหน้าผาหิน</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>Day 5</v>
-      </c>
-      <c r="B12" t="str">
-        <v>มื้อเที่ยง</v>
-      </c>
-      <c r="C12" t="str">
-        <v>Tina's Guesthouse / คาเฟ่ Moye (墨野咖啡)</v>
-      </c>
-      <c r="D12" t="str">
-        <v>ข้าวผัดเนื้อจามรี, บะหมี่ผัด, แซนด์วิช, กาแฟสด</v>
-      </c>
-      <c r="E12">
-        <v>35</v>
-      </c>
-      <c r="F12">
-        <v>175</v>
-      </c>
-      <c r="G12">
-        <v>70</v>
-      </c>
-      <c r="H12">
-        <v>350</v>
-      </c>
-      <c r="I12" t="str">
-        <v>พักผ่อนรอรถบัสไปแชงกรี-ลา</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>Day 5</v>
-      </c>
-      <c r="B13" t="str">
-        <v>มื้อค่ำ</v>
-      </c>
-      <c r="C13" t="str">
-        <v>ร้านอาหารทิเบต จิ้งจิ้งเตอะมานีฉือ (静静的嘛呢石藏餐吧)</v>
-      </c>
-      <c r="D13" t="str">
-        <v>ซี่โครงแกะย่างทิเบต, ชาเนยจามรีร้อน, ขนมปังบาบานมจามรี, ผัดเนื้อจามรี</v>
-      </c>
-      <c r="E13">
-        <v>65</v>
-      </c>
-      <c r="F13">
-        <v>325</v>
-      </c>
-      <c r="G13">
-        <v>130</v>
-      </c>
-      <c r="H13">
-        <v>650</v>
-      </c>
-      <c r="I13" t="str">
-        <v>ร้านอาหารทิเบตชื่อดังประตูเหนือตู๋เค่อจง</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>Day 6</v>
-      </c>
-      <c r="B14" t="str">
-        <v>มื้อเช้า</v>
-      </c>
-      <c r="C14" t="str">
-        <v>ร้านอาหารเช้าใกล้ที่พัก เมืองโบราณตู๋เค่อจง</v>
-      </c>
-      <c r="D14" t="str">
-        <v>ซาลาเปานึ่งสด, ชาร้อน, โจ๊กเนื้อจามรี, ไข่ต้ม</v>
-      </c>
-      <c r="E14">
-        <v>15</v>
-      </c>
-      <c r="F14">
-        <v>75</v>
-      </c>
-      <c r="G14">
-        <v>30</v>
-      </c>
-      <c r="H14">
-        <v>150</v>
-      </c>
-      <c r="I14" t="str">
-        <v>อาหารเช้าก่อนขึ้นที่สูงผู่ต๋าชั่ว</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>Day 6</v>
-      </c>
-      <c r="B15" t="str">
-        <v>มื้อเที่ยง</v>
-      </c>
-      <c r="C15" t="str">
-        <v>ศูนย์บริการนักท่องเที่ยวอุทยานแห่งชาติผู่ต๋าชั่ว</v>
-      </c>
-      <c r="D15" t="str">
-        <v>ข้าวกล่องร้อน, บะหมี่ซุปเนื้อ, ชาขิงคลายหนาว</v>
-      </c>
-      <c r="E15">
-        <v>35</v>
-      </c>
-      <c r="F15">
-        <v>175</v>
-      </c>
-      <c r="G15">
-        <v>70</v>
-      </c>
-      <c r="H15">
-        <v>350</v>
-      </c>
-      <c r="I15" t="str">
-        <v>ทานในอาคารศูนย์บริการคลายหนาว</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>Day 6</v>
-      </c>
-      <c r="B16" t="str">
-        <v>มื้อเย็น</v>
-      </c>
-      <c r="C16" t="str">
-        <v>ร้านปิ้งย่างบนแผ่นหิน หงหง (宏宏无烟石板烧烤)</v>
-      </c>
-      <c r="D16" t="str">
-        <v>ปิ้งย่างแผ่นหินเนื้อจามรี, เห็ดป่าย่างเนย, มันฝรั่งทิเบต</v>
-      </c>
-      <c r="E16">
-        <v>60</v>
-      </c>
-      <c r="F16">
-        <v>300</v>
-      </c>
-      <c r="G16">
-        <v>120</v>
-      </c>
-      <c r="H16">
-        <v>600</v>
-      </c>
-      <c r="I16" t="str">
-        <v>ปิ้งย่างบนแผ่นหินร้อนไร้ควันยอดนิยม</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>Day 7</v>
-      </c>
-      <c r="B17" t="str">
-        <v>มื้อเช้า</v>
-      </c>
-      <c r="C17" t="str">
-        <v>ตลาดเช้าจินเฉียวเซี่ยงหยาง (金桥向阳菜市场)</v>
-      </c>
-      <c r="D17" t="str">
-        <v>นมจามรีต้มสด, ปาท่องโก๋ยักษ์, เสี่ยวหลงเปาทิเบต</v>
-      </c>
-      <c r="E17">
-        <v>15</v>
-      </c>
-      <c r="F17">
-        <v>75</v>
-      </c>
-      <c r="G17">
-        <v>30</v>
-      </c>
-      <c r="H17">
-        <v>150</v>
-      </c>
-      <c r="I17" t="str">
-        <v>สัมผัสวิถีชีวิตชาวบ้านยามเช้า</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>Day 7</v>
-      </c>
-      <c r="B18" t="str">
-        <v>มื้อเที่ยง</v>
-      </c>
-      <c r="C18" t="str">
-        <v>ศูนย์บริการนักท่องเที่ยววัดซงจ้านหลิน</v>
-      </c>
-      <c r="D18" t="str">
-        <v>ข้าวราดแกงยูนนาน, บะหมี่ซุปเนื้อน้ำใส</v>
-      </c>
-      <c r="E18">
-        <v>30</v>
-      </c>
-      <c r="F18">
-        <v>150</v>
-      </c>
-      <c r="G18">
-        <v>60</v>
-      </c>
-      <c r="H18">
-        <v>300</v>
-      </c>
-      <c r="I18" t="str">
-        <v>ทานก่อนขึ้นรถไฟความเร็วสูงกลับลี่เจียง</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>Day 7</v>
-      </c>
-      <c r="B19" t="str">
-        <v>มื้อค่ำ</v>
-      </c>
-      <c r="C19" t="str">
-        <v>ตลาดโต้รุ่งจงอี้ ลี่เจียง / ซอยอาหารน่าซี</v>
-      </c>
-      <c r="D19" t="str">
-        <v>หม้อไฟปลาหิมะยูนนาน, ปิ้งย่างน่าซี, วุ้นถั่วไก่ (鸡豆凉粉)</v>
-      </c>
-      <c r="E19">
-        <v>50</v>
-      </c>
-      <c r="F19">
-        <v>250</v>
-      </c>
-      <c r="G19">
-        <v>100</v>
-      </c>
-      <c r="H19">
-        <v>500</v>
-      </c>
-      <c r="I19" t="str">
-        <v>ฉลองค่ำคืนสุดท้ายในลี่เจียง</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v>Day 8</v>
-      </c>
-      <c r="B20" t="str">
-        <v>มื้อเช้า</v>
-      </c>
-      <c r="C20" t="str">
-        <v>ร้านอาหารเช้าหน้าสนามบินลี่เจียง (LJG)</v>
-      </c>
-      <c r="D20" t="str">
-        <v>กาแฟร้อน, ซาลาเปา, แซนด์วิชเบาๆ</v>
-      </c>
-      <c r="E20">
-        <v>15</v>
-      </c>
-      <c r="F20">
-        <v>75</v>
-      </c>
-      <c r="G20">
-        <v>30</v>
-      </c>
-      <c r="H20">
-        <v>150</v>
-      </c>
-      <c r="I20" t="str">
-        <v>ก่อนขึ้นไฟลท์ MU-5922</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v>Day 8</v>
-      </c>
-      <c r="B21" t="str">
-        <v>มื้อเที่ยง</v>
-      </c>
-      <c r="C21" t="str">
-        <v>ร้านกว่างอี้ฟั่นเตี้ยน (广益饭店 北门街店 คุนหมิง)</v>
-      </c>
-      <c r="D21" t="str">
-        <v>หมูสามชั้นตุ๋นน้ำแดงยูนนาน, ไก่ผัดพริกแห้ง, ซุปเห็ดรวม</v>
-      </c>
-      <c r="E21">
-        <v>50</v>
-      </c>
-      <c r="F21">
-        <v>250</v>
-      </c>
-      <c r="G21">
-        <v>100</v>
-      </c>
-      <c r="H21">
-        <v>500</v>
-      </c>
-      <c r="I21" t="str">
-        <v>ร้านอาหารยูนนานเก่าแก่ใกล้สวนชุ่ยหู</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v>Day 8</v>
-      </c>
-      <c r="B22" t="str">
-        <v>มื้อค่ำ</v>
-      </c>
-      <c r="C22" t="str">
-        <v>สนามบินคุนหมิงฉางสุ่ย (KMG) ก่อนบินกลับ</v>
-      </c>
-      <c r="D22" t="str">
-        <v>ก๋วยเตี๋ยวร้อน, ชายูนนาน, ขนมเปี๊ยะสด</v>
-      </c>
-      <c r="E22">
-        <v>40</v>
-      </c>
-      <c r="F22">
-        <v>200</v>
-      </c>
-      <c r="G22">
-        <v>80</v>
-      </c>
-      <c r="H22">
-        <v>400</v>
-      </c>
-      <c r="I22" t="str">
-        <v>ทานก่อนผ่านเกตขึ้นเครื่องกลับไทย</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str">
-        <v>รวมทั้งหมด</v>
-      </c>
-      <c r="B23" t="str">
-        <v>21 มื้อ ตลอดทริป</v>
-      </c>
-      <c r="C23" t="str">
-        <v>รวมทุกร้านอาหาร/สตรีทฟู้ด/ตลาดสด/คาเฟ่</v>
-      </c>
-      <c r="D23" t="str">
-        <v>ครอบคลุมครบทุกมื้อเช้า เที่ยง ค่ำ ตลอด 8 วัน</v>
-      </c>
-      <c r="E23">
-        <v>770</v>
-      </c>
-      <c r="F23">
-        <v>3850</v>
-      </c>
-      <c r="G23">
-        <v>1540</v>
-      </c>
-      <c r="H23">
-        <v>7700</v>
-      </c>
-      <c r="I23" t="str">
-        <v>ประมาณการเฉลี่ย ¥770 (฿3,850)/คน (รวม 2 คน ฿7,700)</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I23"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G27"/>

</xml_diff>